<commit_message>
Shorten parking yard, vehicle type, and used-for codes to 2 letters
e.g. MT1-KC-D3-BW-001 (was MT1-KHC-DM25-BWC-001). Tehsil code unchanged.
</commit_message>
<xml_diff>
--- a/vehicle_codes/Multan1_Vehicle_Codes.xlsx
+++ b/vehicle_codes/Multan1_Vehicle_Codes.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-DM25-BWC-001</t>
+          <t>MT1-KC-D3-BW-001</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-WEX-LSF-001</t>
+          <t>MT1-KC-WE-LF-001</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-TTR-COM-001</t>
+          <t>MT1-KC-TT-CO-001</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-MSW-SWP-001</t>
+          <t>MT1-KC-MS-SW-001</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-TTR-BWC-002</t>
+          <t>MT1-KC-TT-BW-002</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-TTR-BWC-003</t>
+          <t>MT1-KC-TT-BW-003</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-TTR-BWC-004</t>
+          <t>MT1-KC-TT-BW-004</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-TRL-BWC-001</t>
+          <t>MT1-KC-TL-BW-001</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-001</t>
+          <t>MT1-KC-LR-CO-001</t>
         </is>
       </c>
     </row>
@@ -843,7 +843,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-002</t>
+          <t>MT1-KC-LR-CO-002</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-003</t>
+          <t>MT1-KC-LR-CO-003</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-004</t>
+          <t>MT1-KC-LR-CO-004</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-005</t>
+          <t>MT1-KC-LR-CO-005</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-006</t>
+          <t>MT1-KC-LR-DT-006</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-007</t>
+          <t>MT1-KC-LR-CO-007</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-DM20-LSF-001</t>
+          <t>MT1-KC-D2-LF-001</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-008</t>
+          <t>MT1-KC-LR-DT-008</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-009</t>
+          <t>MT1-KC-LR-DT-009</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-010</t>
+          <t>MT1-KC-LR-DT-010</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-011</t>
+          <t>MT1-KC-LR-CO-011</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-012</t>
+          <t>MT1-KC-LR-CO-012</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-013</t>
+          <t>MT1-KC-LR-DT-013</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-014</t>
+          <t>MT1-KC-LR-DT-014</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-015</t>
+          <t>MT1-KC-LR-DT-015</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-016</t>
+          <t>MT1-KC-LR-DT-016</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-017</t>
+          <t>MT1-KC-LR-DT-017</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-018</t>
+          <t>MT1-KC-LR-DT-018</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-019</t>
+          <t>MT1-KC-LR-DT-019</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-020</t>
+          <t>MT1-KC-LR-DT-020</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-021</t>
+          <t>MT1-KC-LR-DT-021</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-022</t>
+          <t>MT1-KC-LR-CO-022</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-023</t>
+          <t>MT1-KC-LR-DT-023</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-024</t>
+          <t>MT1-KC-LR-DT-024</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-025</t>
+          <t>MT1-KC-LR-DT-025</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-026</t>
+          <t>MT1-KC-LR-DT-026</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-027</t>
+          <t>MT1-KC-LR-DT-027</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-028</t>
+          <t>MT1-KC-LR-DT-028</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-029</t>
+          <t>MT1-KC-LR-DT-029</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-030</t>
+          <t>MT1-KC-LR-DT-030</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-031</t>
+          <t>MT1-KC-LR-DT-031</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-032</t>
+          <t>MT1-KC-LR-DT-032</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-033</t>
+          <t>MT1-KC-LR-DT-033</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-034</t>
+          <t>MT1-KC-LR-DT-034</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-035</t>
+          <t>MT1-KC-LR-DT-035</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-036</t>
+          <t>MT1-KC-LR-DT-036</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-037</t>
+          <t>MT1-KC-LR-DT-037</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-038</t>
+          <t>MT1-KC-LR-DT-038</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2173,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-039</t>
+          <t>MT1-KC-LR-CO-039</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-040</t>
+          <t>MT1-KC-LR-DT-040</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-041</t>
+          <t>MT1-KC-LR-DT-041</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-042</t>
+          <t>MT1-KC-LR-DT-042</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-043</t>
+          <t>MT1-KC-LR-DT-043</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-044</t>
+          <t>MT1-KC-LR-DT-044</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-045</t>
+          <t>MT1-KC-LR-DT-045</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-046</t>
+          <t>MT1-KC-LR-DT-046</t>
         </is>
       </c>
     </row>
@@ -2453,7 +2453,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-047</t>
+          <t>MT1-KC-LR-DT-047</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-048</t>
+          <t>MT1-KC-LR-DT-048</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-049</t>
+          <t>MT1-KC-LR-DT-049</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-050</t>
+          <t>MT1-KC-LR-DT-050</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-051</t>
+          <t>MT1-KC-LR-CO-051</t>
         </is>
       </c>
     </row>
@@ -2628,7 +2628,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-052</t>
+          <t>MT1-KC-LR-DT-052</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-053</t>
+          <t>MT1-KC-LR-DT-053</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-054</t>
+          <t>MT1-KC-LR-DT-054</t>
         </is>
       </c>
     </row>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-055</t>
+          <t>MT1-KC-LR-DT-055</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-CP7-CBC-001</t>
+          <t>MT1-KC-CM-CB-001</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-TTR-BWC-005</t>
+          <t>MT1-KC-TT-BW-005</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-TFB-BWC-001</t>
+          <t>MT1-KC-TB-BW-001</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-056</t>
+          <t>MT1-KC-LR-DT-056</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-057</t>
+          <t>MT1-KC-LR-DT-057</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-058</t>
+          <t>MT1-KC-LR-DT-058</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2978,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-059</t>
+          <t>MT1-KC-LR-DT-059</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-060</t>
+          <t>MT1-KC-LR-DT-060</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-COM-061</t>
+          <t>MT1-KC-LR-CO-061</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-062</t>
+          <t>MT1-KC-LR-DT-062</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-063</t>
+          <t>MT1-KC-LR-DT-063</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3153,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-064</t>
+          <t>MT1-KC-LR-DT-064</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-065</t>
+          <t>MT1-KC-LR-DT-065</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-066</t>
+          <t>MT1-KC-LR-DT-066</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-067</t>
+          <t>MT1-KC-LR-DT-067</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>MT1-KHC-LDR-DTD-068</t>
+          <t>MT1-KC-LR-DT-068</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-069</t>
+          <t>MT1-MR-LR-DT-069</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-070</t>
+          <t>MT1-MR-LR-DT-070</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-071</t>
+          <t>MT1-MR-LR-CO-071</t>
         </is>
       </c>
     </row>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-072</t>
+          <t>MT1-MR-LR-CO-072</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-073</t>
+          <t>MT1-MR-LR-CO-073</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-074</t>
+          <t>MT1-MR-LR-CO-074</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-075</t>
+          <t>MT1-MR-LR-CO-075</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-076</t>
+          <t>MT1-MR-LR-CO-076</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-077</t>
+          <t>MT1-MR-LR-DT-077</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-078</t>
+          <t>MT1-MR-LR-DT-078</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-079</t>
+          <t>MT1-MR-LR-CO-079</t>
         </is>
       </c>
     </row>
@@ -3713,7 +3713,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-080</t>
+          <t>MT1-MR-LR-CO-080</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-081</t>
+          <t>MT1-MR-LR-CO-081</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-082</t>
+          <t>MT1-MR-LR-CO-082</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-083</t>
+          <t>MT1-MR-LR-CO-083</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-084</t>
+          <t>MT1-MR-LR-CO-084</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-085</t>
+          <t>MT1-MR-LR-DT-085</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-086</t>
+          <t>MT1-MR-LR-CO-086</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-087</t>
+          <t>MT1-MR-LR-DT-087</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-088</t>
+          <t>MT1-MR-LR-DT-088</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-089</t>
+          <t>MT1-MR-LR-CO-089</t>
         </is>
       </c>
     </row>
@@ -4063,7 +4063,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-090</t>
+          <t>MT1-MR-LR-CO-090</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4098,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-091</t>
+          <t>MT1-MR-LR-CO-091</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-092</t>
+          <t>MT1-MR-LR-CO-092</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-093</t>
+          <t>MT1-MR-LR-DT-093</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM20-TCP-002</t>
+          <t>MT1-MR-D2-TC-002</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM20-TCP-003</t>
+          <t>MT1-MR-D2-TC-003</t>
         </is>
       </c>
     </row>
@@ -4273,7 +4273,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-002</t>
+          <t>MT1-MR-TL-BW-002</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-094</t>
+          <t>MT1-MR-LR-DT-094</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-095</t>
+          <t>MT1-MR-LR-DT-095</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-096</t>
+          <t>MT1-MR-LR-DT-096</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-097</t>
+          <t>MT1-MR-LR-DT-097</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-098</t>
+          <t>MT1-MR-LR-DT-098</t>
         </is>
       </c>
     </row>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-099</t>
+          <t>MT1-MR-LR-DT-099</t>
         </is>
       </c>
     </row>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-100</t>
+          <t>MT1-MR-LR-DT-100</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-101</t>
+          <t>MT1-MR-LR-DT-101</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-102</t>
+          <t>MT1-MR-LR-CO-102</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-103</t>
+          <t>MT1-MR-LR-DT-103</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-104</t>
+          <t>MT1-MR-LR-DT-104</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4693,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-105</t>
+          <t>MT1-MR-LR-DT-105</t>
         </is>
       </c>
     </row>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-106</t>
+          <t>MT1-MR-LR-DT-106</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4763,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-107</t>
+          <t>MT1-MR-LR-DT-107</t>
         </is>
       </c>
     </row>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-108</t>
+          <t>MT1-MR-LR-DT-108</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-109</t>
+          <t>MT1-MR-LR-DT-109</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-110</t>
+          <t>MT1-MR-LR-DT-110</t>
         </is>
       </c>
     </row>
@@ -4903,7 +4903,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-111</t>
+          <t>MT1-MR-LR-DT-111</t>
         </is>
       </c>
     </row>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-112</t>
+          <t>MT1-MR-LR-DT-112</t>
         </is>
       </c>
     </row>
@@ -4973,7 +4973,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-113</t>
+          <t>MT1-MR-LR-DT-113</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-114</t>
+          <t>MT1-MR-LR-DT-114</t>
         </is>
       </c>
     </row>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-115</t>
+          <t>MT1-MR-LR-DT-115</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5078,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-116</t>
+          <t>MT1-MR-LR-DT-116</t>
         </is>
       </c>
     </row>
@@ -5113,7 +5113,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-117</t>
+          <t>MT1-MR-LR-DT-117</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-118</t>
+          <t>MT1-MR-LR-DT-118</t>
         </is>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-119</t>
+          <t>MT1-MR-LR-DT-119</t>
         </is>
       </c>
     </row>
@@ -5218,7 +5218,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-120</t>
+          <t>MT1-MR-LR-DT-120</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5253,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-121</t>
+          <t>MT1-MR-LR-CO-121</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-122</t>
+          <t>MT1-MR-LR-CO-122</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5323,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-123</t>
+          <t>MT1-MR-LR-CO-123</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5358,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-124</t>
+          <t>MT1-MR-LR-CO-124</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-125</t>
+          <t>MT1-MR-LR-DT-125</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-006</t>
+          <t>MT1-MR-TT-BW-006</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-007</t>
+          <t>MT1-MR-TT-BW-007</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-008</t>
+          <t>MT1-MR-TT-BW-008</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-009</t>
+          <t>MT1-MR-TT-BW-009</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-003</t>
+          <t>MT1-MR-TL-BW-003</t>
         </is>
       </c>
     </row>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-126</t>
+          <t>MT1-MR-LR-DT-126</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5638,7 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-127</t>
+          <t>MT1-MR-LR-DT-127</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-128</t>
+          <t>MT1-MR-LR-DT-128</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-VSW-SWP-001</t>
+          <t>MT1-MR-VS-SW-001</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5743,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-129</t>
+          <t>MT1-MR-LR-DT-129</t>
         </is>
       </c>
     </row>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-130</t>
+          <t>MT1-MR-LR-DT-130</t>
         </is>
       </c>
     </row>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-131</t>
+          <t>MT1-MR-LR-DT-131</t>
         </is>
       </c>
     </row>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-132</t>
+          <t>MT1-MR-LR-DT-132</t>
         </is>
       </c>
     </row>
@@ -5883,7 +5883,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-133</t>
+          <t>MT1-MR-LR-CO-133</t>
         </is>
       </c>
     </row>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-134</t>
+          <t>MT1-MR-LR-DT-134</t>
         </is>
       </c>
     </row>
@@ -5953,7 +5953,7 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-135</t>
+          <t>MT1-MR-LR-DT-135</t>
         </is>
       </c>
     </row>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-136</t>
+          <t>MT1-MR-LR-CO-136</t>
         </is>
       </c>
     </row>
@@ -6023,7 +6023,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-001</t>
+          <t>MT1-MR-D1-TC-001</t>
         </is>
       </c>
     </row>
@@ -6058,7 +6058,7 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-137</t>
+          <t>MT1-MR-LR-DT-137</t>
         </is>
       </c>
     </row>
@@ -6093,7 +6093,7 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-004</t>
+          <t>MT1-MR-TL-BW-004</t>
         </is>
       </c>
     </row>
@@ -6128,7 +6128,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-010</t>
+          <t>MT1-MR-TT-BW-010</t>
         </is>
       </c>
     </row>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-WBZ-WSH-001</t>
+          <t>MT1-MR-WB-WA-001</t>
         </is>
       </c>
     </row>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-MSW-SWP-002</t>
+          <t>MT1-MR-MS-SW-002</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-MSW-SWP-003</t>
+          <t>MT1-MR-MS-SW-003</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-CAR-CBC-001</t>
+          <t>MT1-MR-CA-CB-001</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-CAR-CBC-002</t>
+          <t>MT1-MR-CA-CB-002</t>
         </is>
       </c>
     </row>
@@ -6338,7 +6338,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-011</t>
+          <t>MT1-MR-TT-BW-011</t>
         </is>
       </c>
     </row>
@@ -6373,7 +6373,7 @@
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-138</t>
+          <t>MT1-MR-LR-CO-138</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-139</t>
+          <t>MT1-MR-LR-CO-139</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-140</t>
+          <t>MT1-MR-LR-CO-140</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6478,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-012</t>
+          <t>MT1-MR-TT-BW-012</t>
         </is>
       </c>
     </row>
@@ -6513,7 +6513,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-013</t>
+          <t>MT1-MR-TT-BW-013</t>
         </is>
       </c>
     </row>
@@ -6548,7 +6548,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-141</t>
+          <t>MT1-MR-LR-CO-141</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-014</t>
+          <t>MT1-MR-TT-BW-014</t>
         </is>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-015</t>
+          <t>MT1-MR-TT-BW-015</t>
         </is>
       </c>
     </row>
@@ -6653,7 +6653,7 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-142</t>
+          <t>MT1-MR-LR-DT-142</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-016</t>
+          <t>MT1-MR-TT-BW-016</t>
         </is>
       </c>
     </row>
@@ -6723,7 +6723,7 @@
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-143</t>
+          <t>MT1-MR-LR-CO-143</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-017</t>
+          <t>MT1-MR-TT-BW-017</t>
         </is>
       </c>
     </row>
@@ -6793,7 +6793,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-MSW-SWP-004</t>
+          <t>MT1-MR-MS-SW-004</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-MSW-SWP-005</t>
+          <t>MT1-MR-MS-SW-005</t>
         </is>
       </c>
     </row>
@@ -6863,7 +6863,7 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-018</t>
+          <t>MT1-MR-TT-BW-018</t>
         </is>
       </c>
     </row>
@@ -6898,7 +6898,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-002</t>
+          <t>MT1-MR-D1-TC-002</t>
         </is>
       </c>
     </row>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-003</t>
+          <t>MT1-MR-D1-TC-003</t>
         </is>
       </c>
     </row>
@@ -6968,7 +6968,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-019</t>
+          <t>MT1-MR-TT-BW-019</t>
         </is>
       </c>
     </row>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-WBZ-WSH-002</t>
+          <t>MT1-MR-WB-WA-002</t>
         </is>
       </c>
     </row>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-020</t>
+          <t>MT1-MR-TT-BW-020</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-021</t>
+          <t>MT1-MR-TT-BW-021</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-022</t>
+          <t>MT1-MR-TT-BW-022</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-023</t>
+          <t>MT1-MR-TT-BW-023</t>
         </is>
       </c>
     </row>
@@ -7178,7 +7178,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-004</t>
+          <t>MT1-MR-D1-TC-004</t>
         </is>
       </c>
     </row>
@@ -7213,7 +7213,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-005</t>
+          <t>MT1-MR-D1-TC-005</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7248,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-006</t>
+          <t>MT1-MR-D1-TC-006</t>
         </is>
       </c>
     </row>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-MSW-SWP-006</t>
+          <t>MT1-MR-MS-SW-006</t>
         </is>
       </c>
     </row>
@@ -7318,7 +7318,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-WBZ-WSH-003</t>
+          <t>MT1-MR-WB-WA-003</t>
         </is>
       </c>
     </row>
@@ -7353,7 +7353,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-024</t>
+          <t>MT1-MR-TT-BW-024</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-025</t>
+          <t>MT1-MR-TT-BW-025</t>
         </is>
       </c>
     </row>
@@ -7423,7 +7423,7 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-WBZ-WSH-004</t>
+          <t>MT1-MR-WB-WA-004</t>
         </is>
       </c>
     </row>
@@ -7458,7 +7458,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-007</t>
+          <t>MT1-MR-D1-TC-007</t>
         </is>
       </c>
     </row>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TTR-BWC-026</t>
+          <t>MT1-MR-TT-BW-026</t>
         </is>
       </c>
     </row>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM20-TCP-004</t>
+          <t>MT1-MR-D2-TC-004</t>
         </is>
       </c>
     </row>
@@ -7563,7 +7563,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-DM10-TCP-008</t>
+          <t>MT1-MR-D1-TC-008</t>
         </is>
       </c>
     </row>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-CNC-CBC-001</t>
+          <t>MT1-MR-CC-CB-001</t>
         </is>
       </c>
     </row>
@@ -7633,7 +7633,7 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-005</t>
+          <t>MT1-MR-TL-BW-005</t>
         </is>
       </c>
     </row>
@@ -7668,7 +7668,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-144</t>
+          <t>MT1-MR-LR-DT-144</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-145</t>
+          <t>MT1-MR-LR-CO-145</t>
         </is>
       </c>
     </row>
@@ -7738,7 +7738,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-146</t>
+          <t>MT1-MR-LR-DT-146</t>
         </is>
       </c>
     </row>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-147</t>
+          <t>MT1-MR-LR-CO-147</t>
         </is>
       </c>
     </row>
@@ -7808,7 +7808,7 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-148</t>
+          <t>MT1-MR-LR-DT-148</t>
         </is>
       </c>
     </row>
@@ -7843,7 +7843,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-149</t>
+          <t>MT1-MR-LR-DT-149</t>
         </is>
       </c>
     </row>
@@ -7878,7 +7878,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-150</t>
+          <t>MT1-MR-LR-DT-150</t>
         </is>
       </c>
     </row>
@@ -7913,7 +7913,7 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-151</t>
+          <t>MT1-MR-LR-DT-151</t>
         </is>
       </c>
     </row>
@@ -7948,7 +7948,7 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-152</t>
+          <t>MT1-MR-LR-DT-152</t>
         </is>
       </c>
     </row>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-153</t>
+          <t>MT1-MR-LR-CO-153</t>
         </is>
       </c>
     </row>
@@ -8018,7 +8018,7 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-154</t>
+          <t>MT1-MR-LR-DT-154</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8053,7 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-155</t>
+          <t>MT1-MR-LR-CO-155</t>
         </is>
       </c>
     </row>
@@ -8088,7 +8088,7 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-156</t>
+          <t>MT1-MR-LR-CO-156</t>
         </is>
       </c>
     </row>
@@ -8123,7 +8123,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-157</t>
+          <t>MT1-MR-LR-CO-157</t>
         </is>
       </c>
     </row>
@@ -8158,7 +8158,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-158</t>
+          <t>MT1-MR-LR-DT-158</t>
         </is>
       </c>
     </row>
@@ -8193,7 +8193,7 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-159</t>
+          <t>MT1-MR-LR-DT-159</t>
         </is>
       </c>
     </row>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-160</t>
+          <t>MT1-MR-LR-DT-160</t>
         </is>
       </c>
     </row>
@@ -8263,7 +8263,7 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-161</t>
+          <t>MT1-MR-LR-DT-161</t>
         </is>
       </c>
     </row>
@@ -8298,7 +8298,7 @@
       </c>
       <c r="G224" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-162</t>
+          <t>MT1-MR-LR-DT-162</t>
         </is>
       </c>
     </row>
@@ -8333,7 +8333,7 @@
       </c>
       <c r="G225" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-163</t>
+          <t>MT1-MR-LR-DT-163</t>
         </is>
       </c>
     </row>
@@ -8368,7 +8368,7 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-164</t>
+          <t>MT1-MR-LR-DT-164</t>
         </is>
       </c>
     </row>
@@ -8403,7 +8403,7 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-165</t>
+          <t>MT1-MR-LR-DT-165</t>
         </is>
       </c>
     </row>
@@ -8438,7 +8438,7 @@
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-166</t>
+          <t>MT1-MR-LR-DT-166</t>
         </is>
       </c>
     </row>
@@ -8473,7 +8473,7 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-167</t>
+          <t>MT1-MR-LR-DT-167</t>
         </is>
       </c>
     </row>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-168</t>
+          <t>MT1-MR-LR-DT-168</t>
         </is>
       </c>
     </row>
@@ -8543,7 +8543,7 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-169</t>
+          <t>MT1-MR-LR-CO-169</t>
         </is>
       </c>
     </row>
@@ -8578,7 +8578,7 @@
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-170</t>
+          <t>MT1-MR-LR-DT-170</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8613,7 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-006</t>
+          <t>MT1-MR-TL-BW-006</t>
         </is>
       </c>
     </row>
@@ -8648,7 +8648,7 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-007</t>
+          <t>MT1-MR-TL-BW-007</t>
         </is>
       </c>
     </row>
@@ -8683,7 +8683,7 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-008</t>
+          <t>MT1-MR-TL-BW-008</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-TRL-BWC-009</t>
+          <t>MT1-MR-TL-BW-009</t>
         </is>
       </c>
     </row>
@@ -8753,7 +8753,7 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-DTD-171</t>
+          <t>MT1-MR-LR-DT-171</t>
         </is>
       </c>
     </row>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="G238" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-172</t>
+          <t>MT1-MR-LR-CO-172</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>MT1-MKR-LDR-COM-173</t>
+          <t>MT1-MR-LR-CO-173</t>
         </is>
       </c>
     </row>
@@ -8858,7 +8858,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-DTD-174</t>
+          <t>MT1-QR-LR-DT-174</t>
         </is>
       </c>
     </row>
@@ -8893,7 +8893,7 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-DTD-175</t>
+          <t>MT1-QR-LR-DT-175</t>
         </is>
       </c>
     </row>
@@ -8928,7 +8928,7 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-COM-176</t>
+          <t>MT1-QR-LR-CO-176</t>
         </is>
       </c>
     </row>
@@ -8963,7 +8963,7 @@
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-DTD-177</t>
+          <t>MT1-QR-LR-DT-177</t>
         </is>
       </c>
     </row>
@@ -8998,7 +8998,7 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-COM-178</t>
+          <t>MT1-QR-LR-CO-178</t>
         </is>
       </c>
     </row>
@@ -9033,7 +9033,7 @@
       </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-DTD-179</t>
+          <t>MT1-QR-LR-DT-179</t>
         </is>
       </c>
     </row>
@@ -9068,7 +9068,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-COM-180</t>
+          <t>MT1-QR-LR-CO-180</t>
         </is>
       </c>
     </row>
@@ -9103,7 +9103,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-COM-181</t>
+          <t>MT1-QR-LR-CO-181</t>
         </is>
       </c>
     </row>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>MT1-QPR-LDR-COM-182</t>
+          <t>MT1-QR-LR-CO-182</t>
         </is>
       </c>
     </row>
@@ -9173,7 +9173,7 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-LDR-DTD-183</t>
+          <t>MT1-GM-LR-DT-183</t>
         </is>
       </c>
     </row>
@@ -9208,7 +9208,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CDZ-LSF-001</t>
+          <t>MT1-GM-CD-LF-001</t>
         </is>
       </c>
     </row>
@@ -9243,7 +9243,7 @@
       </c>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-TFB-BWC-002</t>
+          <t>MT1-GM-TB-BW-002</t>
         </is>
       </c>
     </row>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-WBZ-WSH-005</t>
+          <t>MT1-GM-WB-WA-005</t>
         </is>
       </c>
     </row>
@@ -9313,7 +9313,7 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-WBZ-WSH-006</t>
+          <t>MT1-GM-WB-WA-006</t>
         </is>
       </c>
     </row>
@@ -9348,7 +9348,7 @@
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-FEL-BWC-001</t>
+          <t>MT1-GM-FL-BW-001</t>
         </is>
       </c>
     </row>
@@ -9383,7 +9383,7 @@
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-FEL-BWC-002</t>
+          <t>MT1-GM-FL-BW-002</t>
         </is>
       </c>
     </row>
@@ -9418,7 +9418,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CP7-CBC-002</t>
+          <t>MT1-GM-CM-CB-002</t>
         </is>
       </c>
     </row>
@@ -9453,7 +9453,7 @@
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CP7-CBC-003</t>
+          <t>MT1-GM-CM-CB-003</t>
         </is>
       </c>
     </row>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CP7-CBC-004</t>
+          <t>MT1-GM-CM-CB-004</t>
         </is>
       </c>
     </row>
@@ -9523,7 +9523,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CP7-CBC-005</t>
+          <t>MT1-GM-CM-CB-005</t>
         </is>
       </c>
     </row>
@@ -9558,7 +9558,7 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CP7-CBC-006</t>
+          <t>MT1-GM-CM-CB-006</t>
         </is>
       </c>
     </row>
@@ -9593,7 +9593,7 @@
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CP7-CBC-007</t>
+          <t>MT1-GM-CM-CB-007</t>
         </is>
       </c>
     </row>
@@ -9628,7 +9628,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CP7-CBC-008</t>
+          <t>MT1-GM-CM-CB-008</t>
         </is>
       </c>
     </row>
@@ -9663,7 +9663,7 @@
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-HVL-COM-001</t>
+          <t>MT1-GM-HL-CO-001</t>
         </is>
       </c>
     </row>
@@ -9698,7 +9698,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CNC-CBC-002</t>
+          <t>MT1-GM-CC-CB-002</t>
         </is>
       </c>
     </row>
@@ -9733,7 +9733,7 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CNC-CBC-003</t>
+          <t>MT1-GM-CC-CB-003</t>
         </is>
       </c>
     </row>
@@ -9768,7 +9768,7 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-TFB-BWC-003</t>
+          <t>MT1-GM-TB-BW-003</t>
         </is>
       </c>
     </row>
@@ -9803,7 +9803,7 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-DM10-TCP-009</t>
+          <t>MT1-GM-D1-TC-009</t>
         </is>
       </c>
     </row>
@@ -9838,7 +9838,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CAR-CBC-003</t>
+          <t>MT1-GM-CA-CB-003</t>
         </is>
       </c>
     </row>
@@ -9873,7 +9873,7 @@
       </c>
       <c r="G269" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CAR-CBC-004</t>
+          <t>MT1-GM-CA-CB-004</t>
         </is>
       </c>
     </row>
@@ -9908,7 +9908,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CAR-CBC-005</t>
+          <t>MT1-GM-CA-CB-005</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CAR-CBC-006</t>
+          <t>MT1-GM-CA-CB-006</t>
         </is>
       </c>
     </row>
@@ -9978,7 +9978,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CAR-CBC-007</t>
+          <t>MT1-GM-CA-CB-007</t>
         </is>
       </c>
     </row>
@@ -10013,7 +10013,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CAR-CBC-008</t>
+          <t>MT1-GM-CA-CB-008</t>
         </is>
       </c>
     </row>
@@ -10048,7 +10048,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>MT1-GLM-CAR-CBC-009</t>
+          <t>MT1-GM-CA-CB-009</t>
         </is>
       </c>
     </row>
@@ -10080,7 +10080,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TEHSIL-PARKINGYARD-VEHICLETYPE-USEDFOR-NUMBER   (e.g. MT1-KHC-DM25-BWC-001)</t>
+          <t>TEHSIL-PARKINGYARD-VEHICLETYPE-USEDFOR-NUMBER   (e.g. MT1-KC-D3-BW-001)</t>
         </is>
       </c>
     </row>
@@ -10149,7 +10149,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>GLM</t>
+          <t>GM</t>
         </is>
       </c>
     </row>
@@ -10161,7 +10161,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>KHC</t>
+          <t>KC</t>
         </is>
       </c>
     </row>
@@ -10173,7 +10173,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>MKR</t>
+          <t>MR</t>
         </is>
       </c>
     </row>
@@ -10185,7 +10185,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>QPR</t>
+          <t>QR</t>
         </is>
       </c>
     </row>
@@ -10216,7 +10216,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
@@ -10228,7 +10228,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>CDZ</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
@@ -10240,7 +10240,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>CP7</t>
+          <t>CM</t>
         </is>
       </c>
     </row>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>CNC</t>
+          <t>CC</t>
         </is>
       </c>
     </row>
@@ -10264,7 +10264,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>DM10</t>
+          <t>D1</t>
         </is>
       </c>
     </row>
@@ -10276,7 +10276,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>DM20</t>
+          <t>D2</t>
         </is>
       </c>
     </row>
@@ -10288,7 +10288,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>DM25</t>
+          <t>D3</t>
         </is>
       </c>
     </row>
@@ -10300,7 +10300,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>FL</t>
         </is>
       </c>
     </row>
@@ -10312,7 +10312,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>HVL</t>
+          <t>HL</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>LDR</t>
+          <t>LR</t>
         </is>
       </c>
     </row>
@@ -10336,7 +10336,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>MSW</t>
+          <t>MS</t>
         </is>
       </c>
     </row>
@@ -10348,7 +10348,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>TFB</t>
+          <t>TB</t>
         </is>
       </c>
     </row>
@@ -10360,7 +10360,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>TRL</t>
+          <t>TL</t>
         </is>
       </c>
     </row>
@@ -10372,7 +10372,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>TTR</t>
+          <t>TT</t>
         </is>
       </c>
     </row>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>VSW</t>
+          <t>VS</t>
         </is>
       </c>
     </row>
@@ -10396,7 +10396,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>WBZ</t>
+          <t>WB</t>
         </is>
       </c>
     </row>
@@ -10408,7 +10408,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>WEX</t>
+          <t>WE</t>
         </is>
       </c>
     </row>
@@ -10439,7 +10439,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>BWC</t>
+          <t>BW</t>
         </is>
       </c>
     </row>
@@ -10451,7 +10451,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>COM</t>
+          <t>CO</t>
         </is>
       </c>
     </row>
@@ -10463,7 +10463,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>CB</t>
         </is>
       </c>
     </row>
@@ -10475,7 +10475,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>DTD</t>
+          <t>DT</t>
         </is>
       </c>
     </row>
@@ -10487,7 +10487,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>LSF</t>
+          <t>LF</t>
         </is>
       </c>
     </row>
@@ -10499,7 +10499,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>SWP</t>
+          <t>SW</t>
         </is>
       </c>
     </row>
@@ -10511,7 +10511,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>TCP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -10523,7 +10523,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>WA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Multan-2 vehicle code workbook; widen Code Key lookup ranges
Multan2_Vehicle_Codes.xlsx mirrors the Multan-1 template: formula-driven
New Vehicle Code column, dropdown-validated input columns, and a Code Key
sheet extended with Multan-2's tehsil code plus the vehicle types (Gully
Sucker, Drain Cleaner, Rickshaw Shower) and used-for category (De-Silting)
found in its source data that weren't in the original list. Parking Yard
data isn't in the Multan-2 source file, so that column and the codes that
depend on it are left blank pending yard names.

Also widened the Code Key INDEX/MATCH ranges in both workbooks with buffer
rows, so adding a new tehsil/yard/type/use to Code Key later actually
takes effect (previously the ranges were sized to the exact row count,
so a new row silently fell outside the formula's lookup range).
</commit_message>
<xml_diff>
--- a/vehicle_codes/Multan1_Vehicle_Codes.xlsx
+++ b/vehicle_codes/Multan1_Vehicle_Codes.xlsx
@@ -1485,7 +1485,7 @@
         <v>11</v>
       </c>
       <c r="G2" s="2" t="str">
-        <f aca="false">IF(OR(B2="",C2="",E2="",F2=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B2,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F2,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C2,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E2,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C2,C2),"000"))</f>
+        <f aca="false">IF(OR(B2="",C2="",E2="",F2=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B2,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F2,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C2,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E2,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C2,C2),"000"))</f>
         <v>MT1-KC-D3-BW-001</v>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
         <v>11</v>
       </c>
       <c r="G3" s="2" t="str">
-        <f aca="false">IF(OR(B3="",C3="",E3="",F3=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B3,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F3,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C3,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E3,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C3,C3),"000"))</f>
+        <f aca="false">IF(OR(B3="",C3="",E3="",F3=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B3,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F3,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C3,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E3,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C3,C3),"000"))</f>
         <v>MT1-KC-WE-LF-001</v>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
         <v>11</v>
       </c>
       <c r="G4" s="2" t="str">
-        <f aca="false">IF(OR(B4="",C4="",E4="",F4=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B4,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F4,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C4,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E4,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C4,C4),"000"))</f>
+        <f aca="false">IF(OR(B4="",C4="",E4="",F4=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B4,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F4,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C4,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E4,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C4,C4),"000"))</f>
         <v>MT1-KC-TT-CO-001</v>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
         <v>11</v>
       </c>
       <c r="G5" s="2" t="str">
-        <f aca="false">IF(OR(B5="",C5="",E5="",F5=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B5,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F5,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C5,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E5,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C5,C5),"000"))</f>
+        <f aca="false">IF(OR(B5="",C5="",E5="",F5=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B5,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F5,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C5,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E5,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C5,C5),"000"))</f>
         <v>MT1-KC-MS-SW-001</v>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
         <v>11</v>
       </c>
       <c r="G6" s="2" t="str">
-        <f aca="false">IF(OR(B6="",C6="",E6="",F6=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B6,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F6,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C6,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E6,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C6,C6),"000"))</f>
+        <f aca="false">IF(OR(B6="",C6="",E6="",F6=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B6,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F6,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C6,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E6,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C6,C6),"000"))</f>
         <v>MT1-KC-TT-BW-002</v>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
         <v>11</v>
       </c>
       <c r="G7" s="2" t="str">
-        <f aca="false">IF(OR(B7="",C7="",E7="",F7=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B7,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F7,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C7,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E7,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C7,C7),"000"))</f>
+        <f aca="false">IF(OR(B7="",C7="",E7="",F7=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B7,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F7,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C7,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E7,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C7,C7),"000"))</f>
         <v>MT1-KC-TT-BW-003</v>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
         <v>11</v>
       </c>
       <c r="G8" s="2" t="str">
-        <f aca="false">IF(OR(B8="",C8="",E8="",F8=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B8,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F8,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C8,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E8,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C8,C8),"000"))</f>
+        <f aca="false">IF(OR(B8="",C8="",E8="",F8=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B8,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F8,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C8,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E8,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C8,C8),"000"))</f>
         <v>MT1-KC-TT-BW-004</v>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
         <v>11</v>
       </c>
       <c r="G9" s="2" t="str">
-        <f aca="false">IF(OR(B9="",C9="",E9="",F9=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B9,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F9,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C9,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E9,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C9,C9),"000"))</f>
+        <f aca="false">IF(OR(B9="",C9="",E9="",F9=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B9,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F9,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C9,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E9,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C9,C9),"000"))</f>
         <v>MT1-KC-TL-BW-001</v>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
         <v>11</v>
       </c>
       <c r="G10" s="2" t="str">
-        <f aca="false">IF(OR(B10="",C10="",E10="",F10=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B10,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F10,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C10,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E10,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C10,C10),"000"))</f>
+        <f aca="false">IF(OR(B10="",C10="",E10="",F10=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B10,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F10,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C10,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E10,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C10,C10),"000"))</f>
         <v>MT1-KC-LR-CO-001</v>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
         <v>11</v>
       </c>
       <c r="G11" s="2" t="str">
-        <f aca="false">IF(OR(B11="",C11="",E11="",F11=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B11,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F11,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C11,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E11,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C11,C11),"000"))</f>
+        <f aca="false">IF(OR(B11="",C11="",E11="",F11=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B11,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F11,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C11,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E11,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C11,C11),"000"))</f>
         <v>MT1-KC-LR-CO-002</v>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
         <v>11</v>
       </c>
       <c r="G12" s="2" t="str">
-        <f aca="false">IF(OR(B12="",C12="",E12="",F12=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B12,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F12,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C12,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E12,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C12,C12),"000"))</f>
+        <f aca="false">IF(OR(B12="",C12="",E12="",F12=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B12,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F12,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C12,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E12,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C12,C12),"000"))</f>
         <v>MT1-KC-LR-CO-003</v>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
         <v>11</v>
       </c>
       <c r="G13" s="2" t="str">
-        <f aca="false">IF(OR(B13="",C13="",E13="",F13=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B13,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F13,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C13,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E13,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C13,C13),"000"))</f>
+        <f aca="false">IF(OR(B13="",C13="",E13="",F13=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B13,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F13,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C13,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E13,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C13,C13),"000"))</f>
         <v>MT1-KC-LR-CO-004</v>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
         <v>11</v>
       </c>
       <c r="G14" s="2" t="str">
-        <f aca="false">IF(OR(B14="",C14="",E14="",F14=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B14,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F14,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C14,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E14,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C14,C14),"000"))</f>
+        <f aca="false">IF(OR(B14="",C14="",E14="",F14=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B14,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F14,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C14,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E14,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C14,C14),"000"))</f>
         <v>MT1-KC-LR-CO-005</v>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
         <v>11</v>
       </c>
       <c r="G15" s="2" t="str">
-        <f aca="false">IF(OR(B15="",C15="",E15="",F15=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B15,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F15,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C15,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E15,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C15,C15),"000"))</f>
+        <f aca="false">IF(OR(B15="",C15="",E15="",F15=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B15,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F15,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C15,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E15,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C15,C15),"000"))</f>
         <v>MT1-KC-LR-DT-006</v>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
         <v>11</v>
       </c>
       <c r="G16" s="2" t="str">
-        <f aca="false">IF(OR(B16="",C16="",E16="",F16=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B16,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F16,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C16,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E16,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C16,C16),"000"))</f>
+        <f aca="false">IF(OR(B16="",C16="",E16="",F16=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B16,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F16,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C16,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E16,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C16,C16),"000"))</f>
         <v>MT1-KC-LR-CO-007</v>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
         <v>11</v>
       </c>
       <c r="G17" s="2" t="str">
-        <f aca="false">IF(OR(B17="",C17="",E17="",F17=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B17,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F17,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C17,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E17,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C17,C17),"000"))</f>
+        <f aca="false">IF(OR(B17="",C17="",E17="",F17=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B17,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F17,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C17,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E17,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C17,C17),"000"))</f>
         <v>MT1-KC-D2-LF-001</v>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
         <v>11</v>
       </c>
       <c r="G18" s="2" t="str">
-        <f aca="false">IF(OR(B18="",C18="",E18="",F18=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B18,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F18,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C18,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E18,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C18,C18),"000"))</f>
+        <f aca="false">IF(OR(B18="",C18="",E18="",F18=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B18,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F18,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C18,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E18,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C18,C18),"000"))</f>
         <v>MT1-KC-LR-DT-008</v>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
         <v>11</v>
       </c>
       <c r="G19" s="2" t="str">
-        <f aca="false">IF(OR(B19="",C19="",E19="",F19=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B19,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F19,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C19,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E19,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C19,C19),"000"))</f>
+        <f aca="false">IF(OR(B19="",C19="",E19="",F19=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B19,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F19,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C19,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E19,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C19,C19),"000"))</f>
         <v>MT1-KC-LR-DT-009</v>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
         <v>11</v>
       </c>
       <c r="G20" s="2" t="str">
-        <f aca="false">IF(OR(B20="",C20="",E20="",F20=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B20,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F20,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C20,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E20,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C20,C20),"000"))</f>
+        <f aca="false">IF(OR(B20="",C20="",E20="",F20=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B20,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F20,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C20,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E20,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C20,C20),"000"))</f>
         <v>MT1-KC-LR-DT-010</v>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
         <v>11</v>
       </c>
       <c r="G21" s="2" t="str">
-        <f aca="false">IF(OR(B21="",C21="",E21="",F21=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B21,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F21,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C21,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E21,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C21,C21),"000"))</f>
+        <f aca="false">IF(OR(B21="",C21="",E21="",F21=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B21,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F21,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C21,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E21,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C21,C21),"000"))</f>
         <v>MT1-KC-LR-CO-011</v>
       </c>
     </row>
@@ -1965,7 +1965,7 @@
         <v>11</v>
       </c>
       <c r="G22" s="2" t="str">
-        <f aca="false">IF(OR(B22="",C22="",E22="",F22=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B22,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F22,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C22,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E22,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C22,C22),"000"))</f>
+        <f aca="false">IF(OR(B22="",C22="",E22="",F22=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B22,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F22,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C22,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E22,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C22,C22),"000"))</f>
         <v>MT1-KC-LR-CO-012</v>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
         <v>11</v>
       </c>
       <c r="G23" s="2" t="str">
-        <f aca="false">IF(OR(B23="",C23="",E23="",F23=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B23,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F23,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C23,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E23,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C23,C23),"000"))</f>
+        <f aca="false">IF(OR(B23="",C23="",E23="",F23=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B23,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F23,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C23,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E23,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C23,C23),"000"))</f>
         <v>MT1-KC-LR-DT-013</v>
       </c>
     </row>
@@ -2013,7 +2013,7 @@
         <v>11</v>
       </c>
       <c r="G24" s="2" t="str">
-        <f aca="false">IF(OR(B24="",C24="",E24="",F24=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B24,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F24,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C24,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E24,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C24,C24),"000"))</f>
+        <f aca="false">IF(OR(B24="",C24="",E24="",F24=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B24,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F24,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C24,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E24,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C24,C24),"000"))</f>
         <v>MT1-KC-LR-DT-014</v>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
         <v>11</v>
       </c>
       <c r="G25" s="2" t="str">
-        <f aca="false">IF(OR(B25="",C25="",E25="",F25=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B25,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F25,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C25,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E25,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C25,C25),"000"))</f>
+        <f aca="false">IF(OR(B25="",C25="",E25="",F25=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B25,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F25,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C25,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E25,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C25,C25),"000"))</f>
         <v>MT1-KC-LR-DT-015</v>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
         <v>11</v>
       </c>
       <c r="G26" s="2" t="str">
-        <f aca="false">IF(OR(B26="",C26="",E26="",F26=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B26,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F26,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C26,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E26,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C26,C26),"000"))</f>
+        <f aca="false">IF(OR(B26="",C26="",E26="",F26=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B26,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F26,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C26,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E26,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C26,C26),"000"))</f>
         <v>MT1-KC-LR-DT-016</v>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
         <v>11</v>
       </c>
       <c r="G27" s="2" t="str">
-        <f aca="false">IF(OR(B27="",C27="",E27="",F27=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B27,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F27,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C27,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E27,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C27,C27),"000"))</f>
+        <f aca="false">IF(OR(B27="",C27="",E27="",F27=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B27,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F27,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C27,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E27,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C27,C27),"000"))</f>
         <v>MT1-KC-LR-DT-017</v>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
         <v>11</v>
       </c>
       <c r="G28" s="2" t="str">
-        <f aca="false">IF(OR(B28="",C28="",E28="",F28=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B28,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F28,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C28,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E28,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C28,C28),"000"))</f>
+        <f aca="false">IF(OR(B28="",C28="",E28="",F28=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B28,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F28,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C28,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E28,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C28,C28),"000"))</f>
         <v>MT1-KC-LR-DT-018</v>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
         <v>11</v>
       </c>
       <c r="G29" s="2" t="str">
-        <f aca="false">IF(OR(B29="",C29="",E29="",F29=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B29,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F29,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C29,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E29,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C29,C29),"000"))</f>
+        <f aca="false">IF(OR(B29="",C29="",E29="",F29=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B29,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F29,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C29,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E29,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C29,C29),"000"))</f>
         <v>MT1-KC-LR-DT-019</v>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
         <v>11</v>
       </c>
       <c r="G30" s="2" t="str">
-        <f aca="false">IF(OR(B30="",C30="",E30="",F30=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B30,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F30,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C30,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E30,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C30,C30),"000"))</f>
+        <f aca="false">IF(OR(B30="",C30="",E30="",F30=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B30,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F30,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C30,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E30,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C30,C30),"000"))</f>
         <v>MT1-KC-LR-DT-020</v>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
         <v>11</v>
       </c>
       <c r="G31" s="2" t="str">
-        <f aca="false">IF(OR(B31="",C31="",E31="",F31=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B31,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F31,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C31,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E31,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C31,C31),"000"))</f>
+        <f aca="false">IF(OR(B31="",C31="",E31="",F31=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B31,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F31,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C31,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E31,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C31,C31),"000"))</f>
         <v>MT1-KC-LR-DT-021</v>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
         <v>11</v>
       </c>
       <c r="G32" s="2" t="str">
-        <f aca="false">IF(OR(B32="",C32="",E32="",F32=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B32,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F32,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C32,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E32,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C32,C32),"000"))</f>
+        <f aca="false">IF(OR(B32="",C32="",E32="",F32=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B32,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F32,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C32,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E32,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C32,C32),"000"))</f>
         <v>MT1-KC-LR-CO-022</v>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
         <v>11</v>
       </c>
       <c r="G33" s="2" t="str">
-        <f aca="false">IF(OR(B33="",C33="",E33="",F33=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B33,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F33,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C33,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E33,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C33,C33),"000"))</f>
+        <f aca="false">IF(OR(B33="",C33="",E33="",F33=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B33,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F33,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C33,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E33,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C33,C33),"000"))</f>
         <v>MT1-KC-LR-DT-023</v>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
         <v>11</v>
       </c>
       <c r="G34" s="2" t="str">
-        <f aca="false">IF(OR(B34="",C34="",E34="",F34=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B34,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F34,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C34,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E34,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C34,C34),"000"))</f>
+        <f aca="false">IF(OR(B34="",C34="",E34="",F34=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B34,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F34,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C34,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E34,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C34,C34),"000"))</f>
         <v>MT1-KC-LR-DT-024</v>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
         <v>11</v>
       </c>
       <c r="G35" s="2" t="str">
-        <f aca="false">IF(OR(B35="",C35="",E35="",F35=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B35,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F35,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C35,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E35,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C35,C35),"000"))</f>
+        <f aca="false">IF(OR(B35="",C35="",E35="",F35=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B35,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F35,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C35,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E35,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C35,C35),"000"))</f>
         <v>MT1-KC-LR-DT-025</v>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
         <v>11</v>
       </c>
       <c r="G36" s="2" t="str">
-        <f aca="false">IF(OR(B36="",C36="",E36="",F36=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B36,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F36,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C36,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E36,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C36,C36),"000"))</f>
+        <f aca="false">IF(OR(B36="",C36="",E36="",F36=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B36,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F36,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C36,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E36,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C36,C36),"000"))</f>
         <v>MT1-KC-LR-DT-026</v>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
         <v>11</v>
       </c>
       <c r="G37" s="2" t="str">
-        <f aca="false">IF(OR(B37="",C37="",E37="",F37=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B37,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F37,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C37,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E37,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C37,C37),"000"))</f>
+        <f aca="false">IF(OR(B37="",C37="",E37="",F37=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B37,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F37,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C37,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E37,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C37,C37),"000"))</f>
         <v>MT1-KC-LR-DT-027</v>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
         <v>11</v>
       </c>
       <c r="G38" s="2" t="str">
-        <f aca="false">IF(OR(B38="",C38="",E38="",F38=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B38,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F38,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C38,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E38,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C38,C38),"000"))</f>
+        <f aca="false">IF(OR(B38="",C38="",E38="",F38=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B38,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F38,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C38,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E38,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C38,C38),"000"))</f>
         <v>MT1-KC-LR-DT-028</v>
       </c>
     </row>
@@ -2373,7 +2373,7 @@
         <v>11</v>
       </c>
       <c r="G39" s="2" t="str">
-        <f aca="false">IF(OR(B39="",C39="",E39="",F39=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B39,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F39,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C39,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E39,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C39,C39),"000"))</f>
+        <f aca="false">IF(OR(B39="",C39="",E39="",F39=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B39,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F39,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C39,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E39,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C39,C39),"000"))</f>
         <v>MT1-KC-LR-DT-029</v>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
         <v>11</v>
       </c>
       <c r="G40" s="2" t="str">
-        <f aca="false">IF(OR(B40="",C40="",E40="",F40=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B40,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F40,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C40,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E40,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C40,C40),"000"))</f>
+        <f aca="false">IF(OR(B40="",C40="",E40="",F40=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B40,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F40,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C40,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E40,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C40,C40),"000"))</f>
         <v>MT1-KC-LR-DT-030</v>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
         <v>11</v>
       </c>
       <c r="G41" s="2" t="str">
-        <f aca="false">IF(OR(B41="",C41="",E41="",F41=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B41,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F41,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C41,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E41,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C41,C41),"000"))</f>
+        <f aca="false">IF(OR(B41="",C41="",E41="",F41=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B41,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F41,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C41,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E41,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C41,C41),"000"))</f>
         <v>MT1-KC-LR-DT-031</v>
       </c>
     </row>
@@ -2445,7 +2445,7 @@
         <v>11</v>
       </c>
       <c r="G42" s="2" t="str">
-        <f aca="false">IF(OR(B42="",C42="",E42="",F42=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B42,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F42,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C42,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E42,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C42,C42),"000"))</f>
+        <f aca="false">IF(OR(B42="",C42="",E42="",F42=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B42,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F42,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C42,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E42,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C42,C42),"000"))</f>
         <v>MT1-KC-LR-DT-032</v>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
         <v>11</v>
       </c>
       <c r="G43" s="2" t="str">
-        <f aca="false">IF(OR(B43="",C43="",E43="",F43=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B43,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F43,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C43,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E43,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C43,C43),"000"))</f>
+        <f aca="false">IF(OR(B43="",C43="",E43="",F43=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B43,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F43,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C43,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E43,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C43,C43),"000"))</f>
         <v>MT1-KC-LR-DT-033</v>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
         <v>11</v>
       </c>
       <c r="G44" s="2" t="str">
-        <f aca="false">IF(OR(B44="",C44="",E44="",F44=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B44,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F44,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C44,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E44,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C44,C44),"000"))</f>
+        <f aca="false">IF(OR(B44="",C44="",E44="",F44=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B44,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F44,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C44,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E44,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C44,C44),"000"))</f>
         <v>MT1-KC-LR-DT-034</v>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
         <v>11</v>
       </c>
       <c r="G45" s="2" t="str">
-        <f aca="false">IF(OR(B45="",C45="",E45="",F45=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B45,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F45,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C45,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E45,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C45,C45),"000"))</f>
+        <f aca="false">IF(OR(B45="",C45="",E45="",F45=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B45,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F45,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C45,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E45,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C45,C45),"000"))</f>
         <v>MT1-KC-LR-DT-035</v>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
         <v>11</v>
       </c>
       <c r="G46" s="2" t="str">
-        <f aca="false">IF(OR(B46="",C46="",E46="",F46=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B46,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F46,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C46,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E46,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C46,C46),"000"))</f>
+        <f aca="false">IF(OR(B46="",C46="",E46="",F46=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B46,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F46,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C46,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E46,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C46,C46),"000"))</f>
         <v>MT1-KC-LR-DT-036</v>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
         <v>11</v>
       </c>
       <c r="G47" s="2" t="str">
-        <f aca="false">IF(OR(B47="",C47="",E47="",F47=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B47,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F47,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C47,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E47,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C47,C47),"000"))</f>
+        <f aca="false">IF(OR(B47="",C47="",E47="",F47=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B47,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F47,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C47,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E47,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C47,C47),"000"))</f>
         <v>MT1-KC-LR-DT-037</v>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
         <v>11</v>
       </c>
       <c r="G48" s="2" t="str">
-        <f aca="false">IF(OR(B48="",C48="",E48="",F48=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B48,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F48,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C48,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E48,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C48,C48),"000"))</f>
+        <f aca="false">IF(OR(B48="",C48="",E48="",F48=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B48,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F48,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C48,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E48,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C48,C48),"000"))</f>
         <v>MT1-KC-LR-DT-038</v>
       </c>
     </row>
@@ -2613,7 +2613,7 @@
         <v>11</v>
       </c>
       <c r="G49" s="2" t="str">
-        <f aca="false">IF(OR(B49="",C49="",E49="",F49=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B49,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F49,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C49,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E49,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C49,C49),"000"))</f>
+        <f aca="false">IF(OR(B49="",C49="",E49="",F49=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B49,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F49,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C49,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E49,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C49,C49),"000"))</f>
         <v>MT1-KC-LR-CO-039</v>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
         <v>11</v>
       </c>
       <c r="G50" s="2" t="str">
-        <f aca="false">IF(OR(B50="",C50="",E50="",F50=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B50,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F50,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C50,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E50,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C50,C50),"000"))</f>
+        <f aca="false">IF(OR(B50="",C50="",E50="",F50=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B50,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F50,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C50,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E50,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C50,C50),"000"))</f>
         <v>MT1-KC-LR-DT-040</v>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
         <v>11</v>
       </c>
       <c r="G51" s="2" t="str">
-        <f aca="false">IF(OR(B51="",C51="",E51="",F51=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B51,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F51,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C51,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E51,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C51,C51),"000"))</f>
+        <f aca="false">IF(OR(B51="",C51="",E51="",F51=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B51,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F51,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C51,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E51,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C51,C51),"000"))</f>
         <v>MT1-KC-LR-DT-041</v>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
         <v>11</v>
       </c>
       <c r="G52" s="2" t="str">
-        <f aca="false">IF(OR(B52="",C52="",E52="",F52=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B52,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F52,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C52,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E52,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C52,C52),"000"))</f>
+        <f aca="false">IF(OR(B52="",C52="",E52="",F52=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B52,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F52,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C52,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E52,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C52,C52),"000"))</f>
         <v>MT1-KC-LR-DT-042</v>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
         <v>11</v>
       </c>
       <c r="G53" s="2" t="str">
-        <f aca="false">IF(OR(B53="",C53="",E53="",F53=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B53,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F53,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C53,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E53,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C53,C53),"000"))</f>
+        <f aca="false">IF(OR(B53="",C53="",E53="",F53=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B53,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F53,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C53,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E53,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C53,C53),"000"))</f>
         <v>MT1-KC-LR-DT-043</v>
       </c>
     </row>
@@ -2733,7 +2733,7 @@
         <v>11</v>
       </c>
       <c r="G54" s="2" t="str">
-        <f aca="false">IF(OR(B54="",C54="",E54="",F54=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B54,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F54,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C54,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E54,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C54,C54),"000"))</f>
+        <f aca="false">IF(OR(B54="",C54="",E54="",F54=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B54,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F54,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C54,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E54,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C54,C54),"000"))</f>
         <v>MT1-KC-LR-DT-044</v>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
         <v>11</v>
       </c>
       <c r="G55" s="2" t="str">
-        <f aca="false">IF(OR(B55="",C55="",E55="",F55=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B55,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F55,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C55,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E55,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C55,C55),"000"))</f>
+        <f aca="false">IF(OR(B55="",C55="",E55="",F55=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B55,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F55,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C55,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E55,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C55,C55),"000"))</f>
         <v>MT1-KC-LR-DT-045</v>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
         <v>11</v>
       </c>
       <c r="G56" s="2" t="str">
-        <f aca="false">IF(OR(B56="",C56="",E56="",F56=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B56,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F56,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C56,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E56,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C56,C56),"000"))</f>
+        <f aca="false">IF(OR(B56="",C56="",E56="",F56=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B56,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F56,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C56,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E56,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C56,C56),"000"))</f>
         <v>MT1-KC-LR-DT-046</v>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
         <v>11</v>
       </c>
       <c r="G57" s="2" t="str">
-        <f aca="false">IF(OR(B57="",C57="",E57="",F57=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B57,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F57,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C57,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E57,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C57,C57),"000"))</f>
+        <f aca="false">IF(OR(B57="",C57="",E57="",F57=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B57,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F57,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C57,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E57,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C57,C57),"000"))</f>
         <v>MT1-KC-LR-DT-047</v>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
         <v>11</v>
       </c>
       <c r="G58" s="2" t="str">
-        <f aca="false">IF(OR(B58="",C58="",E58="",F58=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B58,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F58,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C58,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E58,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C58,C58),"000"))</f>
+        <f aca="false">IF(OR(B58="",C58="",E58="",F58=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B58,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F58,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C58,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E58,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C58,C58),"000"))</f>
         <v>MT1-KC-LR-DT-048</v>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
         <v>11</v>
       </c>
       <c r="G59" s="2" t="str">
-        <f aca="false">IF(OR(B59="",C59="",E59="",F59=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B59,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F59,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C59,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E59,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C59,C59),"000"))</f>
+        <f aca="false">IF(OR(B59="",C59="",E59="",F59=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B59,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F59,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C59,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E59,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C59,C59),"000"))</f>
         <v>MT1-KC-LR-DT-049</v>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
         <v>11</v>
       </c>
       <c r="G60" s="2" t="str">
-        <f aca="false">IF(OR(B60="",C60="",E60="",F60=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B60,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F60,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C60,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E60,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C60,C60),"000"))</f>
+        <f aca="false">IF(OR(B60="",C60="",E60="",F60=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B60,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F60,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C60,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E60,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C60,C60),"000"))</f>
         <v>MT1-KC-LR-DT-050</v>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
         <v>11</v>
       </c>
       <c r="G61" s="2" t="str">
-        <f aca="false">IF(OR(B61="",C61="",E61="",F61=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B61,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F61,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C61,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E61,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C61,C61),"000"))</f>
+        <f aca="false">IF(OR(B61="",C61="",E61="",F61=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B61,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F61,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C61,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E61,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C61,C61),"000"))</f>
         <v>MT1-KC-LR-CO-051</v>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
         <v>11</v>
       </c>
       <c r="G62" s="2" t="str">
-        <f aca="false">IF(OR(B62="",C62="",E62="",F62=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B62,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F62,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C62,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E62,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C62,C62),"000"))</f>
+        <f aca="false">IF(OR(B62="",C62="",E62="",F62=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B62,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F62,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C62,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E62,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C62,C62),"000"))</f>
         <v>MT1-KC-LR-DT-052</v>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
         <v>11</v>
       </c>
       <c r="G63" s="2" t="str">
-        <f aca="false">IF(OR(B63="",C63="",E63="",F63=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B63,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F63,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C63,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E63,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C63,C63),"000"))</f>
+        <f aca="false">IF(OR(B63="",C63="",E63="",F63=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B63,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F63,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C63,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E63,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C63,C63),"000"))</f>
         <v>MT1-KC-LR-DT-053</v>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
         <v>11</v>
       </c>
       <c r="G64" s="2" t="str">
-        <f aca="false">IF(OR(B64="",C64="",E64="",F64=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B64,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F64,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C64,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E64,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C64,C64),"000"))</f>
+        <f aca="false">IF(OR(B64="",C64="",E64="",F64=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B64,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F64,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C64,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E64,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C64,C64),"000"))</f>
         <v>MT1-KC-LR-DT-054</v>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
         <v>11</v>
       </c>
       <c r="G65" s="2" t="str">
-        <f aca="false">IF(OR(B65="",C65="",E65="",F65=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B65,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F65,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C65,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E65,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C65,C65),"000"))</f>
+        <f aca="false">IF(OR(B65="",C65="",E65="",F65=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B65,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F65,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C65,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E65,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C65,C65),"000"))</f>
         <v>MT1-KC-LR-DT-055</v>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
         <v>11</v>
       </c>
       <c r="G66" s="2" t="str">
-        <f aca="false">IF(OR(B66="",C66="",E66="",F66=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B66,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F66,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C66,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E66,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C66,C66),"000"))</f>
+        <f aca="false">IF(OR(B66="",C66="",E66="",F66=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B66,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F66,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C66,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E66,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C66,C66),"000"))</f>
         <v>MT1-KC-CM-CB-001</v>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
         <v>11</v>
       </c>
       <c r="G67" s="2" t="str">
-        <f aca="false">IF(OR(B67="",C67="",E67="",F67=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B67,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F67,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C67,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E67,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C67,C67),"000"))</f>
+        <f aca="false">IF(OR(B67="",C67="",E67="",F67=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B67,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F67,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C67,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E67,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C67,C67),"000"))</f>
         <v>MT1-KC-TT-BW-005</v>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
         <v>11</v>
       </c>
       <c r="G68" s="2" t="str">
-        <f aca="false">IF(OR(B68="",C68="",E68="",F68=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B68,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F68,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C68,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E68,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C68,C68),"000"))</f>
+        <f aca="false">IF(OR(B68="",C68="",E68="",F68=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B68,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F68,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C68,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E68,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C68,C68),"000"))</f>
         <v>MT1-KC-TB-BW-001</v>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
         <v>11</v>
       </c>
       <c r="G69" s="2" t="str">
-        <f aca="false">IF(OR(B69="",C69="",E69="",F69=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B69,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F69,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C69,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E69,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C69,C69),"000"))</f>
+        <f aca="false">IF(OR(B69="",C69="",E69="",F69=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B69,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F69,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C69,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E69,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C69,C69),"000"))</f>
         <v>MT1-KC-LR-DT-056</v>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
         <v>11</v>
       </c>
       <c r="G70" s="2" t="str">
-        <f aca="false">IF(OR(B70="",C70="",E70="",F70=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B70,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F70,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C70,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E70,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C70,C70),"000"))</f>
+        <f aca="false">IF(OR(B70="",C70="",E70="",F70=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B70,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F70,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C70,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E70,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C70,C70),"000"))</f>
         <v>MT1-KC-LR-DT-057</v>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
         <v>11</v>
       </c>
       <c r="G71" s="2" t="str">
-        <f aca="false">IF(OR(B71="",C71="",E71="",F71=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B71,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F71,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C71,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E71,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C71,C71),"000"))</f>
+        <f aca="false">IF(OR(B71="",C71="",E71="",F71=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B71,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F71,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C71,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E71,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C71,C71),"000"))</f>
         <v>MT1-KC-LR-DT-058</v>
       </c>
     </row>
@@ -3165,7 +3165,7 @@
         <v>11</v>
       </c>
       <c r="G72" s="2" t="str">
-        <f aca="false">IF(OR(B72="",C72="",E72="",F72=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B72,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F72,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C72,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E72,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C72,C72),"000"))</f>
+        <f aca="false">IF(OR(B72="",C72="",E72="",F72=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B72,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F72,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C72,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E72,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C72,C72),"000"))</f>
         <v>MT1-KC-LR-DT-059</v>
       </c>
     </row>
@@ -3189,7 +3189,7 @@
         <v>11</v>
       </c>
       <c r="G73" s="2" t="str">
-        <f aca="false">IF(OR(B73="",C73="",E73="",F73=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B73,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F73,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C73,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E73,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C73,C73),"000"))</f>
+        <f aca="false">IF(OR(B73="",C73="",E73="",F73=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B73,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F73,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C73,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E73,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C73,C73),"000"))</f>
         <v>MT1-KC-LR-DT-060</v>
       </c>
     </row>
@@ -3213,7 +3213,7 @@
         <v>11</v>
       </c>
       <c r="G74" s="2" t="str">
-        <f aca="false">IF(OR(B74="",C74="",E74="",F74=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B74,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F74,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C74,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E74,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C74,C74),"000"))</f>
+        <f aca="false">IF(OR(B74="",C74="",E74="",F74=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B74,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F74,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C74,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E74,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C74,C74),"000"))</f>
         <v>MT1-KC-LR-CO-061</v>
       </c>
     </row>
@@ -3237,7 +3237,7 @@
         <v>11</v>
       </c>
       <c r="G75" s="2" t="str">
-        <f aca="false">IF(OR(B75="",C75="",E75="",F75=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B75,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F75,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C75,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E75,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C75,C75),"000"))</f>
+        <f aca="false">IF(OR(B75="",C75="",E75="",F75=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B75,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F75,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C75,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E75,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C75,C75),"000"))</f>
         <v>MT1-KC-LR-DT-062</v>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
         <v>11</v>
       </c>
       <c r="G76" s="2" t="str">
-        <f aca="false">IF(OR(B76="",C76="",E76="",F76=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B76,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F76,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C76,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E76,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C76,C76),"000"))</f>
+        <f aca="false">IF(OR(B76="",C76="",E76="",F76=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B76,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F76,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C76,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E76,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C76,C76),"000"))</f>
         <v>MT1-KC-LR-DT-063</v>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
         <v>11</v>
       </c>
       <c r="G77" s="2" t="str">
-        <f aca="false">IF(OR(B77="",C77="",E77="",F77=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B77,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F77,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C77,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E77,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C77,C77),"000"))</f>
+        <f aca="false">IF(OR(B77="",C77="",E77="",F77=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B77,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F77,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C77,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E77,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C77,C77),"000"))</f>
         <v>MT1-KC-LR-DT-064</v>
       </c>
     </row>
@@ -3309,7 +3309,7 @@
         <v>11</v>
       </c>
       <c r="G78" s="2" t="str">
-        <f aca="false">IF(OR(B78="",C78="",E78="",F78=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B78,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F78,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C78,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E78,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C78,C78),"000"))</f>
+        <f aca="false">IF(OR(B78="",C78="",E78="",F78=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B78,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F78,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C78,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E78,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C78,C78),"000"))</f>
         <v>MT1-KC-LR-DT-065</v>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
         <v>11</v>
       </c>
       <c r="G79" s="2" t="str">
-        <f aca="false">IF(OR(B79="",C79="",E79="",F79=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B79,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F79,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C79,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E79,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C79,C79),"000"))</f>
+        <f aca="false">IF(OR(B79="",C79="",E79="",F79=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B79,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F79,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C79,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E79,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C79,C79),"000"))</f>
         <v>MT1-KC-LR-DT-066</v>
       </c>
     </row>
@@ -3357,7 +3357,7 @@
         <v>11</v>
       </c>
       <c r="G80" s="2" t="str">
-        <f aca="false">IF(OR(B80="",C80="",E80="",F80=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B80,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F80,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C80,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E80,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C80,C80),"000"))</f>
+        <f aca="false">IF(OR(B80="",C80="",E80="",F80=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B80,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F80,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C80,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E80,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C80,C80),"000"))</f>
         <v>MT1-KC-LR-DT-067</v>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
         <v>11</v>
       </c>
       <c r="G81" s="2" t="str">
-        <f aca="false">IF(OR(B81="",C81="",E81="",F81=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B81,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F81,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C81,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E81,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C81,C81),"000"))</f>
+        <f aca="false">IF(OR(B81="",C81="",E81="",F81=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B81,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F81,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C81,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E81,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C81,C81),"000"))</f>
         <v>MT1-KC-LR-DT-068</v>
       </c>
     </row>
@@ -3405,7 +3405,7 @@
         <v>105</v>
       </c>
       <c r="G82" s="2" t="str">
-        <f aca="false">IF(OR(B82="",C82="",E82="",F82=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B82,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F82,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C82,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E82,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C82,C82),"000"))</f>
+        <f aca="false">IF(OR(B82="",C82="",E82="",F82=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B82,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F82,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C82,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E82,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C82,C82),"000"))</f>
         <v>MT1-MR-LR-DT-069</v>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
         <v>105</v>
       </c>
       <c r="G83" s="2" t="str">
-        <f aca="false">IF(OR(B83="",C83="",E83="",F83=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B83,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F83,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C83,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E83,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C83,C83),"000"))</f>
+        <f aca="false">IF(OR(B83="",C83="",E83="",F83=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B83,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F83,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C83,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E83,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C83,C83),"000"))</f>
         <v>MT1-MR-LR-DT-070</v>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
         <v>105</v>
       </c>
       <c r="G84" s="2" t="str">
-        <f aca="false">IF(OR(B84="",C84="",E84="",F84=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B84,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F84,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C84,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E84,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C84,C84),"000"))</f>
+        <f aca="false">IF(OR(B84="",C84="",E84="",F84=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B84,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F84,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C84,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E84,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C84,C84),"000"))</f>
         <v>MT1-MR-LR-CO-071</v>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
         <v>105</v>
       </c>
       <c r="G85" s="2" t="str">
-        <f aca="false">IF(OR(B85="",C85="",E85="",F85=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B85,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F85,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C85,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E85,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C85,C85),"000"))</f>
+        <f aca="false">IF(OR(B85="",C85="",E85="",F85=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B85,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F85,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C85,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E85,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C85,C85),"000"))</f>
         <v>MT1-MR-LR-CO-072</v>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
         <v>105</v>
       </c>
       <c r="G86" s="2" t="str">
-        <f aca="false">IF(OR(B86="",C86="",E86="",F86=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B86,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F86,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C86,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E86,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C86,C86),"000"))</f>
+        <f aca="false">IF(OR(B86="",C86="",E86="",F86=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B86,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F86,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C86,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E86,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C86,C86),"000"))</f>
         <v>MT1-MR-LR-CO-073</v>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
         <v>105</v>
       </c>
       <c r="G87" s="2" t="str">
-        <f aca="false">IF(OR(B87="",C87="",E87="",F87=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B87,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F87,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C87,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E87,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C87,C87),"000"))</f>
+        <f aca="false">IF(OR(B87="",C87="",E87="",F87=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B87,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F87,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C87,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E87,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C87,C87),"000"))</f>
         <v>MT1-MR-LR-CO-074</v>
       </c>
     </row>
@@ -3549,7 +3549,7 @@
         <v>105</v>
       </c>
       <c r="G88" s="2" t="str">
-        <f aca="false">IF(OR(B88="",C88="",E88="",F88=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B88,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F88,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C88,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E88,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C88,C88),"000"))</f>
+        <f aca="false">IF(OR(B88="",C88="",E88="",F88=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B88,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F88,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C88,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E88,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C88,C88),"000"))</f>
         <v>MT1-MR-LR-CO-075</v>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
         <v>105</v>
       </c>
       <c r="G89" s="2" t="str">
-        <f aca="false">IF(OR(B89="",C89="",E89="",F89=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B89,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F89,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C89,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E89,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C89,C89),"000"))</f>
+        <f aca="false">IF(OR(B89="",C89="",E89="",F89=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B89,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F89,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C89,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E89,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C89,C89),"000"))</f>
         <v>MT1-MR-LR-CO-076</v>
       </c>
     </row>
@@ -3597,7 +3597,7 @@
         <v>105</v>
       </c>
       <c r="G90" s="2" t="str">
-        <f aca="false">IF(OR(B90="",C90="",E90="",F90=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B90,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F90,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C90,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E90,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C90,C90),"000"))</f>
+        <f aca="false">IF(OR(B90="",C90="",E90="",F90=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B90,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F90,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C90,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E90,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C90,C90),"000"))</f>
         <v>MT1-MR-LR-DT-077</v>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
         <v>105</v>
       </c>
       <c r="G91" s="2" t="str">
-        <f aca="false">IF(OR(B91="",C91="",E91="",F91=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B91,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F91,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C91,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E91,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C91,C91),"000"))</f>
+        <f aca="false">IF(OR(B91="",C91="",E91="",F91=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B91,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F91,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C91,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E91,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C91,C91),"000"))</f>
         <v>MT1-MR-LR-DT-078</v>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
         <v>105</v>
       </c>
       <c r="G92" s="2" t="str">
-        <f aca="false">IF(OR(B92="",C92="",E92="",F92=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B92,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F92,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C92,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E92,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C92,C92),"000"))</f>
+        <f aca="false">IF(OR(B92="",C92="",E92="",F92=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B92,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F92,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C92,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E92,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C92,C92),"000"))</f>
         <v>MT1-MR-LR-CO-079</v>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
         <v>105</v>
       </c>
       <c r="G93" s="2" t="str">
-        <f aca="false">IF(OR(B93="",C93="",E93="",F93=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B93,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F93,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C93,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E93,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C93,C93),"000"))</f>
+        <f aca="false">IF(OR(B93="",C93="",E93="",F93=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B93,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F93,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C93,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E93,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C93,C93),"000"))</f>
         <v>MT1-MR-LR-CO-080</v>
       </c>
     </row>
@@ -3693,7 +3693,7 @@
         <v>105</v>
       </c>
       <c r="G94" s="2" t="str">
-        <f aca="false">IF(OR(B94="",C94="",E94="",F94=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B94,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F94,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C94,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E94,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C94,C94),"000"))</f>
+        <f aca="false">IF(OR(B94="",C94="",E94="",F94=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B94,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F94,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C94,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E94,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C94,C94),"000"))</f>
         <v>MT1-MR-LR-CO-081</v>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
         <v>105</v>
       </c>
       <c r="G95" s="2" t="str">
-        <f aca="false">IF(OR(B95="",C95="",E95="",F95=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B95,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F95,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C95,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E95,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C95,C95),"000"))</f>
+        <f aca="false">IF(OR(B95="",C95="",E95="",F95=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B95,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F95,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C95,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E95,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C95,C95),"000"))</f>
         <v>MT1-MR-LR-CO-082</v>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
         <v>105</v>
       </c>
       <c r="G96" s="2" t="str">
-        <f aca="false">IF(OR(B96="",C96="",E96="",F96=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B96,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F96,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C96,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E96,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C96,C96),"000"))</f>
+        <f aca="false">IF(OR(B96="",C96="",E96="",F96=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B96,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F96,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C96,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E96,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C96,C96),"000"))</f>
         <v>MT1-MR-LR-CO-083</v>
       </c>
     </row>
@@ -3765,7 +3765,7 @@
         <v>105</v>
       </c>
       <c r="G97" s="2" t="str">
-        <f aca="false">IF(OR(B97="",C97="",E97="",F97=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B97,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F97,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C97,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E97,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C97,C97),"000"))</f>
+        <f aca="false">IF(OR(B97="",C97="",E97="",F97=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B97,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F97,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C97,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E97,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C97,C97),"000"))</f>
         <v>MT1-MR-LR-CO-084</v>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
         <v>105</v>
       </c>
       <c r="G98" s="2" t="str">
-        <f aca="false">IF(OR(B98="",C98="",E98="",F98=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B98,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F98,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C98,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E98,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C98,C98),"000"))</f>
+        <f aca="false">IF(OR(B98="",C98="",E98="",F98=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B98,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F98,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C98,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E98,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C98,C98),"000"))</f>
         <v>MT1-MR-LR-DT-085</v>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
         <v>105</v>
       </c>
       <c r="G99" s="2" t="str">
-        <f aca="false">IF(OR(B99="",C99="",E99="",F99=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B99,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F99,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C99,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E99,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C99,C99),"000"))</f>
+        <f aca="false">IF(OR(B99="",C99="",E99="",F99=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B99,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F99,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C99,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E99,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C99,C99),"000"))</f>
         <v>MT1-MR-LR-CO-086</v>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
         <v>105</v>
       </c>
       <c r="G100" s="2" t="str">
-        <f aca="false">IF(OR(B100="",C100="",E100="",F100=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B100,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F100,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C100,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E100,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C100,C100),"000"))</f>
+        <f aca="false">IF(OR(B100="",C100="",E100="",F100=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B100,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F100,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C100,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E100,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C100,C100),"000"))</f>
         <v>MT1-MR-LR-DT-087</v>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
         <v>105</v>
       </c>
       <c r="G101" s="2" t="str">
-        <f aca="false">IF(OR(B101="",C101="",E101="",F101=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B101,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F101,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C101,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E101,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C101,C101),"000"))</f>
+        <f aca="false">IF(OR(B101="",C101="",E101="",F101=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B101,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F101,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C101,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E101,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C101,C101),"000"))</f>
         <v>MT1-MR-LR-DT-088</v>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
         <v>105</v>
       </c>
       <c r="G102" s="2" t="str">
-        <f aca="false">IF(OR(B102="",C102="",E102="",F102=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B102,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F102,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C102,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E102,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C102,C102),"000"))</f>
+        <f aca="false">IF(OR(B102="",C102="",E102="",F102=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B102,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F102,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C102,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E102,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C102,C102),"000"))</f>
         <v>MT1-MR-LR-CO-089</v>
       </c>
     </row>
@@ -3909,7 +3909,7 @@
         <v>105</v>
       </c>
       <c r="G103" s="2" t="str">
-        <f aca="false">IF(OR(B103="",C103="",E103="",F103=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B103,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F103,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C103,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E103,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C103,C103),"000"))</f>
+        <f aca="false">IF(OR(B103="",C103="",E103="",F103=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B103,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F103,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C103,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E103,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C103,C103),"000"))</f>
         <v>MT1-MR-LR-CO-090</v>
       </c>
     </row>
@@ -3933,7 +3933,7 @@
         <v>105</v>
       </c>
       <c r="G104" s="2" t="str">
-        <f aca="false">IF(OR(B104="",C104="",E104="",F104=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B104,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F104,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C104,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E104,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C104,C104),"000"))</f>
+        <f aca="false">IF(OR(B104="",C104="",E104="",F104=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B104,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F104,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C104,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E104,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C104,C104),"000"))</f>
         <v>MT1-MR-LR-CO-091</v>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
         <v>105</v>
       </c>
       <c r="G105" s="2" t="str">
-        <f aca="false">IF(OR(B105="",C105="",E105="",F105=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B105,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F105,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C105,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E105,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C105,C105),"000"))</f>
+        <f aca="false">IF(OR(B105="",C105="",E105="",F105=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B105,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F105,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C105,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E105,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C105,C105),"000"))</f>
         <v>MT1-MR-LR-CO-092</v>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
         <v>105</v>
       </c>
       <c r="G106" s="2" t="str">
-        <f aca="false">IF(OR(B106="",C106="",E106="",F106=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B106,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F106,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C106,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E106,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C106,C106),"000"))</f>
+        <f aca="false">IF(OR(B106="",C106="",E106="",F106=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B106,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F106,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C106,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E106,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C106,C106),"000"))</f>
         <v>MT1-MR-LR-DT-093</v>
       </c>
     </row>
@@ -4005,7 +4005,7 @@
         <v>105</v>
       </c>
       <c r="G107" s="2" t="str">
-        <f aca="false">IF(OR(B107="",C107="",E107="",F107=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B107,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F107,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C107,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E107,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C107,C107),"000"))</f>
+        <f aca="false">IF(OR(B107="",C107="",E107="",F107=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B107,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F107,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C107,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E107,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C107,C107),"000"))</f>
         <v>MT1-MR-D2-TC-002</v>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
         <v>105</v>
       </c>
       <c r="G108" s="2" t="str">
-        <f aca="false">IF(OR(B108="",C108="",E108="",F108=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B108,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F108,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C108,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E108,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C108,C108),"000"))</f>
+        <f aca="false">IF(OR(B108="",C108="",E108="",F108=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B108,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F108,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C108,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E108,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C108,C108),"000"))</f>
         <v>MT1-MR-D2-TC-003</v>
       </c>
     </row>
@@ -4053,7 +4053,7 @@
         <v>105</v>
       </c>
       <c r="G109" s="2" t="str">
-        <f aca="false">IF(OR(B109="",C109="",E109="",F109=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B109,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F109,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C109,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E109,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C109,C109),"000"))</f>
+        <f aca="false">IF(OR(B109="",C109="",E109="",F109=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B109,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F109,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C109,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E109,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C109,C109),"000"))</f>
         <v>MT1-MR-TL-BW-002</v>
       </c>
     </row>
@@ -4077,7 +4077,7 @@
         <v>105</v>
       </c>
       <c r="G110" s="2" t="str">
-        <f aca="false">IF(OR(B110="",C110="",E110="",F110=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B110,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F110,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C110,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E110,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C110,C110),"000"))</f>
+        <f aca="false">IF(OR(B110="",C110="",E110="",F110=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B110,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F110,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C110,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E110,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C110,C110),"000"))</f>
         <v>MT1-MR-LR-DT-094</v>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
         <v>105</v>
       </c>
       <c r="G111" s="2" t="str">
-        <f aca="false">IF(OR(B111="",C111="",E111="",F111=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B111,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F111,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C111,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E111,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C111,C111),"000"))</f>
+        <f aca="false">IF(OR(B111="",C111="",E111="",F111=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B111,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F111,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C111,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E111,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C111,C111),"000"))</f>
         <v>MT1-MR-LR-DT-095</v>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
         <v>105</v>
       </c>
       <c r="G112" s="2" t="str">
-        <f aca="false">IF(OR(B112="",C112="",E112="",F112=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B112,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F112,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C112,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E112,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C112,C112),"000"))</f>
+        <f aca="false">IF(OR(B112="",C112="",E112="",F112=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B112,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F112,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C112,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E112,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C112,C112),"000"))</f>
         <v>MT1-MR-LR-DT-096</v>
       </c>
     </row>
@@ -4149,7 +4149,7 @@
         <v>105</v>
       </c>
       <c r="G113" s="2" t="str">
-        <f aca="false">IF(OR(B113="",C113="",E113="",F113=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B113,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F113,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C113,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E113,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C113,C113),"000"))</f>
+        <f aca="false">IF(OR(B113="",C113="",E113="",F113=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B113,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F113,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C113,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E113,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C113,C113),"000"))</f>
         <v>MT1-MR-LR-DT-097</v>
       </c>
     </row>
@@ -4173,7 +4173,7 @@
         <v>105</v>
       </c>
       <c r="G114" s="2" t="str">
-        <f aca="false">IF(OR(B114="",C114="",E114="",F114=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B114,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F114,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C114,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E114,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C114,C114),"000"))</f>
+        <f aca="false">IF(OR(B114="",C114="",E114="",F114=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B114,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F114,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C114,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E114,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C114,C114),"000"))</f>
         <v>MT1-MR-LR-DT-098</v>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
         <v>105</v>
       </c>
       <c r="G115" s="2" t="str">
-        <f aca="false">IF(OR(B115="",C115="",E115="",F115=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B115,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F115,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C115,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E115,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C115,C115),"000"))</f>
+        <f aca="false">IF(OR(B115="",C115="",E115="",F115=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B115,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F115,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C115,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E115,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C115,C115),"000"))</f>
         <v>MT1-MR-LR-DT-099</v>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
         <v>105</v>
       </c>
       <c r="G116" s="2" t="str">
-        <f aca="false">IF(OR(B116="",C116="",E116="",F116=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B116,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F116,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C116,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E116,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C116,C116),"000"))</f>
+        <f aca="false">IF(OR(B116="",C116="",E116="",F116=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B116,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F116,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C116,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E116,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C116,C116),"000"))</f>
         <v>MT1-MR-LR-DT-100</v>
       </c>
     </row>
@@ -4245,7 +4245,7 @@
         <v>105</v>
       </c>
       <c r="G117" s="2" t="str">
-        <f aca="false">IF(OR(B117="",C117="",E117="",F117=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B117,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F117,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C117,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E117,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C117,C117),"000"))</f>
+        <f aca="false">IF(OR(B117="",C117="",E117="",F117=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B117,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F117,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C117,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E117,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C117,C117),"000"))</f>
         <v>MT1-MR-LR-DT-101</v>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
         <v>105</v>
       </c>
       <c r="G118" s="2" t="str">
-        <f aca="false">IF(OR(B118="",C118="",E118="",F118=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B118,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F118,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C118,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E118,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C118,C118),"000"))</f>
+        <f aca="false">IF(OR(B118="",C118="",E118="",F118=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B118,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F118,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C118,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E118,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C118,C118),"000"))</f>
         <v>MT1-MR-LR-CO-102</v>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
         <v>105</v>
       </c>
       <c r="G119" s="2" t="str">
-        <f aca="false">IF(OR(B119="",C119="",E119="",F119=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B119,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F119,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C119,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E119,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C119,C119),"000"))</f>
+        <f aca="false">IF(OR(B119="",C119="",E119="",F119=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B119,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F119,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C119,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E119,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C119,C119),"000"))</f>
         <v>MT1-MR-LR-DT-103</v>
       </c>
     </row>
@@ -4317,7 +4317,7 @@
         <v>105</v>
       </c>
       <c r="G120" s="2" t="str">
-        <f aca="false">IF(OR(B120="",C120="",E120="",F120=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B120,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F120,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C120,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E120,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C120,C120),"000"))</f>
+        <f aca="false">IF(OR(B120="",C120="",E120="",F120=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B120,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F120,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C120,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E120,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C120,C120),"000"))</f>
         <v>MT1-MR-LR-DT-104</v>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
         <v>105</v>
       </c>
       <c r="G121" s="2" t="str">
-        <f aca="false">IF(OR(B121="",C121="",E121="",F121=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B121,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F121,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C121,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E121,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C121,C121),"000"))</f>
+        <f aca="false">IF(OR(B121="",C121="",E121="",F121=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B121,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F121,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C121,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E121,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C121,C121),"000"))</f>
         <v>MT1-MR-LR-DT-105</v>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
         <v>105</v>
       </c>
       <c r="G122" s="2" t="str">
-        <f aca="false">IF(OR(B122="",C122="",E122="",F122=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B122,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F122,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C122,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E122,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C122,C122),"000"))</f>
+        <f aca="false">IF(OR(B122="",C122="",E122="",F122=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B122,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F122,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C122,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E122,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C122,C122),"000"))</f>
         <v>MT1-MR-LR-DT-106</v>
       </c>
     </row>
@@ -4389,7 +4389,7 @@
         <v>105</v>
       </c>
       <c r="G123" s="2" t="str">
-        <f aca="false">IF(OR(B123="",C123="",E123="",F123=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B123,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F123,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C123,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E123,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C123,C123),"000"))</f>
+        <f aca="false">IF(OR(B123="",C123="",E123="",F123=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B123,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F123,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C123,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E123,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C123,C123),"000"))</f>
         <v>MT1-MR-LR-DT-107</v>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
         <v>105</v>
       </c>
       <c r="G124" s="2" t="str">
-        <f aca="false">IF(OR(B124="",C124="",E124="",F124=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B124,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F124,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C124,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E124,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C124,C124),"000"))</f>
+        <f aca="false">IF(OR(B124="",C124="",E124="",F124=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B124,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F124,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C124,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E124,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C124,C124),"000"))</f>
         <v>MT1-MR-LR-DT-108</v>
       </c>
     </row>
@@ -4437,7 +4437,7 @@
         <v>105</v>
       </c>
       <c r="G125" s="2" t="str">
-        <f aca="false">IF(OR(B125="",C125="",E125="",F125=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B125,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F125,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C125,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E125,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C125,C125),"000"))</f>
+        <f aca="false">IF(OR(B125="",C125="",E125="",F125=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B125,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F125,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C125,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E125,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C125,C125),"000"))</f>
         <v>MT1-MR-LR-DT-109</v>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
         <v>105</v>
       </c>
       <c r="G126" s="2" t="str">
-        <f aca="false">IF(OR(B126="",C126="",E126="",F126=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B126,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F126,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C126,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E126,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C126,C126),"000"))</f>
+        <f aca="false">IF(OR(B126="",C126="",E126="",F126=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B126,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F126,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C126,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E126,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C126,C126),"000"))</f>
         <v>MT1-MR-LR-DT-110</v>
       </c>
     </row>
@@ -4485,7 +4485,7 @@
         <v>105</v>
       </c>
       <c r="G127" s="2" t="str">
-        <f aca="false">IF(OR(B127="",C127="",E127="",F127=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B127,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F127,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C127,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E127,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C127,C127),"000"))</f>
+        <f aca="false">IF(OR(B127="",C127="",E127="",F127=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B127,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F127,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C127,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E127,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C127,C127),"000"))</f>
         <v>MT1-MR-LR-DT-111</v>
       </c>
     </row>
@@ -4509,7 +4509,7 @@
         <v>105</v>
       </c>
       <c r="G128" s="2" t="str">
-        <f aca="false">IF(OR(B128="",C128="",E128="",F128=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B128,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F128,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C128,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E128,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C128,C128),"000"))</f>
+        <f aca="false">IF(OR(B128="",C128="",E128="",F128=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B128,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F128,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C128,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E128,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C128,C128),"000"))</f>
         <v>MT1-MR-LR-DT-112</v>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
         <v>105</v>
       </c>
       <c r="G129" s="2" t="str">
-        <f aca="false">IF(OR(B129="",C129="",E129="",F129=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B129,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F129,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C129,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E129,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C129,C129),"000"))</f>
+        <f aca="false">IF(OR(B129="",C129="",E129="",F129=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B129,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F129,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C129,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E129,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C129,C129),"000"))</f>
         <v>MT1-MR-LR-DT-113</v>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
         <v>105</v>
       </c>
       <c r="G130" s="2" t="str">
-        <f aca="false">IF(OR(B130="",C130="",E130="",F130=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B130,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F130,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C130,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E130,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C130,C130),"000"))</f>
+        <f aca="false">IF(OR(B130="",C130="",E130="",F130=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B130,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F130,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C130,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E130,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C130,C130),"000"))</f>
         <v>MT1-MR-LR-DT-114</v>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
         <v>105</v>
       </c>
       <c r="G131" s="2" t="str">
-        <f aca="false">IF(OR(B131="",C131="",E131="",F131=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B131,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F131,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C131,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E131,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C131,C131),"000"))</f>
+        <f aca="false">IF(OR(B131="",C131="",E131="",F131=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B131,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F131,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C131,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E131,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C131,C131),"000"))</f>
         <v>MT1-MR-LR-DT-115</v>
       </c>
     </row>
@@ -4605,7 +4605,7 @@
         <v>105</v>
       </c>
       <c r="G132" s="2" t="str">
-        <f aca="false">IF(OR(B132="",C132="",E132="",F132=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B132,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F132,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C132,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E132,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C132,C132),"000"))</f>
+        <f aca="false">IF(OR(B132="",C132="",E132="",F132=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B132,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F132,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C132,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E132,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C132,C132),"000"))</f>
         <v>MT1-MR-LR-DT-116</v>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
         <v>105</v>
       </c>
       <c r="G133" s="2" t="str">
-        <f aca="false">IF(OR(B133="",C133="",E133="",F133=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B133,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F133,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C133,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E133,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C133,C133),"000"))</f>
+        <f aca="false">IF(OR(B133="",C133="",E133="",F133=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B133,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F133,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C133,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E133,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C133,C133),"000"))</f>
         <v>MT1-MR-LR-DT-117</v>
       </c>
     </row>
@@ -4653,7 +4653,7 @@
         <v>105</v>
       </c>
       <c r="G134" s="2" t="str">
-        <f aca="false">IF(OR(B134="",C134="",E134="",F134=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B134,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F134,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C134,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E134,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C134,C134),"000"))</f>
+        <f aca="false">IF(OR(B134="",C134="",E134="",F134=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B134,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F134,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C134,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E134,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C134,C134),"000"))</f>
         <v>MT1-MR-LR-DT-118</v>
       </c>
     </row>
@@ -4677,7 +4677,7 @@
         <v>105</v>
       </c>
       <c r="G135" s="2" t="str">
-        <f aca="false">IF(OR(B135="",C135="",E135="",F135=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B135,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F135,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C135,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E135,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C135,C135),"000"))</f>
+        <f aca="false">IF(OR(B135="",C135="",E135="",F135=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B135,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F135,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C135,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E135,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C135,C135),"000"))</f>
         <v>MT1-MR-LR-DT-119</v>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
         <v>105</v>
       </c>
       <c r="G136" s="2" t="str">
-        <f aca="false">IF(OR(B136="",C136="",E136="",F136=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B136,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F136,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C136,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E136,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C136,C136),"000"))</f>
+        <f aca="false">IF(OR(B136="",C136="",E136="",F136=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B136,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F136,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C136,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E136,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C136,C136),"000"))</f>
         <v>MT1-MR-LR-DT-120</v>
       </c>
     </row>
@@ -4725,7 +4725,7 @@
         <v>105</v>
       </c>
       <c r="G137" s="2" t="str">
-        <f aca="false">IF(OR(B137="",C137="",E137="",F137=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B137,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F137,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C137,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E137,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C137,C137),"000"))</f>
+        <f aca="false">IF(OR(B137="",C137="",E137="",F137=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B137,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F137,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C137,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E137,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C137,C137),"000"))</f>
         <v>MT1-MR-LR-CO-121</v>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
         <v>105</v>
       </c>
       <c r="G138" s="2" t="str">
-        <f aca="false">IF(OR(B138="",C138="",E138="",F138=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B138,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F138,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C138,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E138,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C138,C138),"000"))</f>
+        <f aca="false">IF(OR(B138="",C138="",E138="",F138=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B138,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F138,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C138,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E138,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C138,C138),"000"))</f>
         <v>MT1-MR-LR-CO-122</v>
       </c>
     </row>
@@ -4773,7 +4773,7 @@
         <v>105</v>
       </c>
       <c r="G139" s="2" t="str">
-        <f aca="false">IF(OR(B139="",C139="",E139="",F139=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B139,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F139,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C139,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E139,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C139,C139),"000"))</f>
+        <f aca="false">IF(OR(B139="",C139="",E139="",F139=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B139,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F139,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C139,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E139,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C139,C139),"000"))</f>
         <v>MT1-MR-LR-CO-123</v>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
         <v>105</v>
       </c>
       <c r="G140" s="2" t="str">
-        <f aca="false">IF(OR(B140="",C140="",E140="",F140=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B140,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F140,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C140,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E140,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C140,C140),"000"))</f>
+        <f aca="false">IF(OR(B140="",C140="",E140="",F140=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B140,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F140,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C140,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E140,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C140,C140),"000"))</f>
         <v>MT1-MR-LR-CO-124</v>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
         <v>105</v>
       </c>
       <c r="G141" s="2" t="str">
-        <f aca="false">IF(OR(B141="",C141="",E141="",F141=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B141,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F141,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C141,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E141,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C141,C141),"000"))</f>
+        <f aca="false">IF(OR(B141="",C141="",E141="",F141=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B141,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F141,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C141,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E141,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C141,C141),"000"))</f>
         <v>MT1-MR-LR-DT-125</v>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
         <v>105</v>
       </c>
       <c r="G142" s="2" t="str">
-        <f aca="false">IF(OR(B142="",C142="",E142="",F142=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B142,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F142,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C142,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E142,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C142,C142),"000"))</f>
+        <f aca="false">IF(OR(B142="",C142="",E142="",F142=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B142,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F142,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C142,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E142,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C142,C142),"000"))</f>
         <v>MT1-MR-TT-BW-006</v>
       </c>
     </row>
@@ -4869,7 +4869,7 @@
         <v>105</v>
       </c>
       <c r="G143" s="2" t="str">
-        <f aca="false">IF(OR(B143="",C143="",E143="",F143=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B143,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F143,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C143,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E143,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C143,C143),"000"))</f>
+        <f aca="false">IF(OR(B143="",C143="",E143="",F143=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B143,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F143,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C143,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E143,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C143,C143),"000"))</f>
         <v>MT1-MR-TT-BW-007</v>
       </c>
     </row>
@@ -4893,7 +4893,7 @@
         <v>105</v>
       </c>
       <c r="G144" s="2" t="str">
-        <f aca="false">IF(OR(B144="",C144="",E144="",F144=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B144,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F144,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C144,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E144,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C144,C144),"000"))</f>
+        <f aca="false">IF(OR(B144="",C144="",E144="",F144=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B144,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F144,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C144,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E144,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C144,C144),"000"))</f>
         <v>MT1-MR-TT-BW-008</v>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
         <v>105</v>
       </c>
       <c r="G145" s="2" t="str">
-        <f aca="false">IF(OR(B145="",C145="",E145="",F145=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B145,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F145,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C145,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E145,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C145,C145),"000"))</f>
+        <f aca="false">IF(OR(B145="",C145="",E145="",F145=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B145,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F145,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C145,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E145,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C145,C145),"000"))</f>
         <v>MT1-MR-TT-BW-009</v>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
         <v>105</v>
       </c>
       <c r="G146" s="2" t="str">
-        <f aca="false">IF(OR(B146="",C146="",E146="",F146=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B146,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F146,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C146,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E146,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C146,C146),"000"))</f>
+        <f aca="false">IF(OR(B146="",C146="",E146="",F146=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B146,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F146,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C146,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E146,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C146,C146),"000"))</f>
         <v>MT1-MR-TL-BW-003</v>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
         <v>105</v>
       </c>
       <c r="G147" s="2" t="str">
-        <f aca="false">IF(OR(B147="",C147="",E147="",F147=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B147,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F147,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C147,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E147,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C147,C147),"000"))</f>
+        <f aca="false">IF(OR(B147="",C147="",E147="",F147=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B147,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F147,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C147,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E147,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C147,C147),"000"))</f>
         <v>MT1-MR-LR-DT-126</v>
       </c>
     </row>
@@ -4989,7 +4989,7 @@
         <v>105</v>
       </c>
       <c r="G148" s="2" t="str">
-        <f aca="false">IF(OR(B148="",C148="",E148="",F148=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B148,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F148,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C148,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E148,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C148,C148),"000"))</f>
+        <f aca="false">IF(OR(B148="",C148="",E148="",F148=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B148,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F148,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C148,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E148,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C148,C148),"000"))</f>
         <v>MT1-MR-LR-DT-127</v>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
         <v>105</v>
       </c>
       <c r="G149" s="2" t="str">
-        <f aca="false">IF(OR(B149="",C149="",E149="",F149=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B149,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F149,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C149,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E149,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C149,C149),"000"))</f>
+        <f aca="false">IF(OR(B149="",C149="",E149="",F149=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B149,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F149,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C149,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E149,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C149,C149),"000"))</f>
         <v>MT1-MR-LR-DT-128</v>
       </c>
     </row>
@@ -5037,7 +5037,7 @@
         <v>105</v>
       </c>
       <c r="G150" s="2" t="str">
-        <f aca="false">IF(OR(B150="",C150="",E150="",F150=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B150,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F150,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C150,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E150,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C150,C150),"000"))</f>
+        <f aca="false">IF(OR(B150="",C150="",E150="",F150=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B150,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F150,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C150,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E150,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C150,C150),"000"))</f>
         <v>MT1-MR-VS-SW-001</v>
       </c>
     </row>
@@ -5061,7 +5061,7 @@
         <v>105</v>
       </c>
       <c r="G151" s="2" t="str">
-        <f aca="false">IF(OR(B151="",C151="",E151="",F151=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B151,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F151,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C151,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E151,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C151,C151),"000"))</f>
+        <f aca="false">IF(OR(B151="",C151="",E151="",F151=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B151,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F151,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C151,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E151,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C151,C151),"000"))</f>
         <v>MT1-MR-LR-DT-129</v>
       </c>
     </row>
@@ -5085,7 +5085,7 @@
         <v>105</v>
       </c>
       <c r="G152" s="2" t="str">
-        <f aca="false">IF(OR(B152="",C152="",E152="",F152=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B152,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F152,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C152,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E152,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C152,C152),"000"))</f>
+        <f aca="false">IF(OR(B152="",C152="",E152="",F152=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B152,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F152,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C152,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E152,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C152,C152),"000"))</f>
         <v>MT1-MR-LR-DT-130</v>
       </c>
     </row>
@@ -5109,7 +5109,7 @@
         <v>105</v>
       </c>
       <c r="G153" s="2" t="str">
-        <f aca="false">IF(OR(B153="",C153="",E153="",F153=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B153,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F153,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C153,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E153,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C153,C153),"000"))</f>
+        <f aca="false">IF(OR(B153="",C153="",E153="",F153=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B153,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F153,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C153,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E153,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C153,C153),"000"))</f>
         <v>MT1-MR-LR-DT-131</v>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
         <v>105</v>
       </c>
       <c r="G154" s="2" t="str">
-        <f aca="false">IF(OR(B154="",C154="",E154="",F154=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B154,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F154,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C154,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E154,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C154,C154),"000"))</f>
+        <f aca="false">IF(OR(B154="",C154="",E154="",F154=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B154,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F154,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C154,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E154,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C154,C154),"000"))</f>
         <v>MT1-MR-LR-DT-132</v>
       </c>
     </row>
@@ -5157,7 +5157,7 @@
         <v>105</v>
       </c>
       <c r="G155" s="2" t="str">
-        <f aca="false">IF(OR(B155="",C155="",E155="",F155=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B155,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F155,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C155,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E155,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C155,C155),"000"))</f>
+        <f aca="false">IF(OR(B155="",C155="",E155="",F155=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B155,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F155,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C155,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E155,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C155,C155),"000"))</f>
         <v>MT1-MR-LR-CO-133</v>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
         <v>105</v>
       </c>
       <c r="G156" s="2" t="str">
-        <f aca="false">IF(OR(B156="",C156="",E156="",F156=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B156,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F156,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C156,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E156,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C156,C156),"000"))</f>
+        <f aca="false">IF(OR(B156="",C156="",E156="",F156=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B156,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F156,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C156,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E156,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C156,C156),"000"))</f>
         <v>MT1-MR-LR-DT-134</v>
       </c>
     </row>
@@ -5205,7 +5205,7 @@
         <v>105</v>
       </c>
       <c r="G157" s="2" t="str">
-        <f aca="false">IF(OR(B157="",C157="",E157="",F157=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B157,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F157,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C157,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E157,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C157,C157),"000"))</f>
+        <f aca="false">IF(OR(B157="",C157="",E157="",F157=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B157,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F157,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C157,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E157,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C157,C157),"000"))</f>
         <v>MT1-MR-LR-DT-135</v>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
         <v>105</v>
       </c>
       <c r="G158" s="2" t="str">
-        <f aca="false">IF(OR(B158="",C158="",E158="",F158=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B158,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F158,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C158,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E158,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C158,C158),"000"))</f>
+        <f aca="false">IF(OR(B158="",C158="",E158="",F158=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B158,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F158,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C158,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E158,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C158,C158),"000"))</f>
         <v>MT1-MR-LR-CO-136</v>
       </c>
     </row>
@@ -5253,7 +5253,7 @@
         <v>105</v>
       </c>
       <c r="G159" s="2" t="str">
-        <f aca="false">IF(OR(B159="",C159="",E159="",F159=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B159,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F159,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C159,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E159,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C159,C159),"000"))</f>
+        <f aca="false">IF(OR(B159="",C159="",E159="",F159=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B159,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F159,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C159,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E159,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C159,C159),"000"))</f>
         <v>MT1-MR-D1-TC-001</v>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
         <v>105</v>
       </c>
       <c r="G160" s="2" t="str">
-        <f aca="false">IF(OR(B160="",C160="",E160="",F160=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B160,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F160,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C160,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E160,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C160,C160),"000"))</f>
+        <f aca="false">IF(OR(B160="",C160="",E160="",F160=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B160,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F160,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C160,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E160,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C160,C160),"000"))</f>
         <v>MT1-MR-LR-DT-137</v>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
         <v>105</v>
       </c>
       <c r="G161" s="2" t="str">
-        <f aca="false">IF(OR(B161="",C161="",E161="",F161=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B161,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F161,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C161,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E161,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C161,C161),"000"))</f>
+        <f aca="false">IF(OR(B161="",C161="",E161="",F161=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B161,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F161,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C161,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E161,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C161,C161),"000"))</f>
         <v>MT1-MR-TL-BW-004</v>
       </c>
     </row>
@@ -5325,7 +5325,7 @@
         <v>105</v>
       </c>
       <c r="G162" s="2" t="str">
-        <f aca="false">IF(OR(B162="",C162="",E162="",F162=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B162,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F162,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C162,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E162,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C162,C162),"000"))</f>
+        <f aca="false">IF(OR(B162="",C162="",E162="",F162=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B162,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F162,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C162,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E162,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C162,C162),"000"))</f>
         <v>MT1-MR-TT-BW-010</v>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
         <v>105</v>
       </c>
       <c r="G163" s="2" t="str">
-        <f aca="false">IF(OR(B163="",C163="",E163="",F163=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B163,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F163,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C163,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E163,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C163,C163),"000"))</f>
+        <f aca="false">IF(OR(B163="",C163="",E163="",F163=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B163,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F163,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C163,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E163,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C163,C163),"000"))</f>
         <v>MT1-MR-WB-WA-001</v>
       </c>
     </row>
@@ -5373,7 +5373,7 @@
         <v>105</v>
       </c>
       <c r="G164" s="2" t="str">
-        <f aca="false">IF(OR(B164="",C164="",E164="",F164=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B164,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F164,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C164,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E164,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C164,C164),"000"))</f>
+        <f aca="false">IF(OR(B164="",C164="",E164="",F164=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B164,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F164,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C164,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E164,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C164,C164),"000"))</f>
         <v>MT1-MR-MS-SW-002</v>
       </c>
     </row>
@@ -5397,7 +5397,7 @@
         <v>105</v>
       </c>
       <c r="G165" s="2" t="str">
-        <f aca="false">IF(OR(B165="",C165="",E165="",F165=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B165,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F165,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C165,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E165,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C165,C165),"000"))</f>
+        <f aca="false">IF(OR(B165="",C165="",E165="",F165=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B165,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F165,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C165,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E165,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C165,C165),"000"))</f>
         <v>MT1-MR-MS-SW-003</v>
       </c>
     </row>
@@ -5421,7 +5421,7 @@
         <v>105</v>
       </c>
       <c r="G166" s="2" t="str">
-        <f aca="false">IF(OR(B166="",C166="",E166="",F166=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B166,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F166,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C166,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E166,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C166,C166),"000"))</f>
+        <f aca="false">IF(OR(B166="",C166="",E166="",F166=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B166,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F166,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C166,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E166,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C166,C166),"000"))</f>
         <v>MT1-MR-CA-CB-001</v>
       </c>
     </row>
@@ -5445,7 +5445,7 @@
         <v>105</v>
       </c>
       <c r="G167" s="2" t="str">
-        <f aca="false">IF(OR(B167="",C167="",E167="",F167=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B167,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F167,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C167,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E167,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C167,C167),"000"))</f>
+        <f aca="false">IF(OR(B167="",C167="",E167="",F167=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B167,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F167,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C167,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E167,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C167,C167),"000"))</f>
         <v>MT1-MR-CA-CB-002</v>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
         <v>105</v>
       </c>
       <c r="G168" s="2" t="str">
-        <f aca="false">IF(OR(B168="",C168="",E168="",F168=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B168,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F168,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C168,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E168,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C168,C168),"000"))</f>
+        <f aca="false">IF(OR(B168="",C168="",E168="",F168=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B168,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F168,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C168,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E168,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C168,C168),"000"))</f>
         <v>MT1-MR-TT-BW-011</v>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
         <v>105</v>
       </c>
       <c r="G169" s="2" t="str">
-        <f aca="false">IF(OR(B169="",C169="",E169="",F169=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B169,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F169,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C169,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E169,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C169,C169),"000"))</f>
+        <f aca="false">IF(OR(B169="",C169="",E169="",F169=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B169,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F169,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C169,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E169,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C169,C169),"000"))</f>
         <v>MT1-MR-LR-CO-138</v>
       </c>
     </row>
@@ -5517,7 +5517,7 @@
         <v>105</v>
       </c>
       <c r="G170" s="2" t="str">
-        <f aca="false">IF(OR(B170="",C170="",E170="",F170=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B170,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F170,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C170,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E170,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C170,C170),"000"))</f>
+        <f aca="false">IF(OR(B170="",C170="",E170="",F170=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B170,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F170,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C170,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E170,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C170,C170),"000"))</f>
         <v>MT1-MR-LR-CO-139</v>
       </c>
     </row>
@@ -5541,7 +5541,7 @@
         <v>105</v>
       </c>
       <c r="G171" s="2" t="str">
-        <f aca="false">IF(OR(B171="",C171="",E171="",F171=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B171,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F171,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C171,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E171,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C171,C171),"000"))</f>
+        <f aca="false">IF(OR(B171="",C171="",E171="",F171=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B171,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F171,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C171,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E171,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C171,C171),"000"))</f>
         <v>MT1-MR-LR-CO-140</v>
       </c>
     </row>
@@ -5565,7 +5565,7 @@
         <v>105</v>
       </c>
       <c r="G172" s="2" t="str">
-        <f aca="false">IF(OR(B172="",C172="",E172="",F172=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B172,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F172,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C172,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E172,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C172,C172),"000"))</f>
+        <f aca="false">IF(OR(B172="",C172="",E172="",F172=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B172,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F172,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C172,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E172,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C172,C172),"000"))</f>
         <v>MT1-MR-TT-BW-012</v>
       </c>
     </row>
@@ -5589,7 +5589,7 @@
         <v>105</v>
       </c>
       <c r="G173" s="2" t="str">
-        <f aca="false">IF(OR(B173="",C173="",E173="",F173=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B173,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F173,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C173,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E173,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C173,C173),"000"))</f>
+        <f aca="false">IF(OR(B173="",C173="",E173="",F173=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B173,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F173,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C173,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E173,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C173,C173),"000"))</f>
         <v>MT1-MR-TT-BW-013</v>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
         <v>105</v>
       </c>
       <c r="G174" s="2" t="str">
-        <f aca="false">IF(OR(B174="",C174="",E174="",F174=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B174,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F174,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C174,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E174,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C174,C174),"000"))</f>
+        <f aca="false">IF(OR(B174="",C174="",E174="",F174=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B174,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F174,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C174,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E174,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C174,C174),"000"))</f>
         <v>MT1-MR-LR-CO-141</v>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
         <v>105</v>
       </c>
       <c r="G175" s="2" t="str">
-        <f aca="false">IF(OR(B175="",C175="",E175="",F175=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B175,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F175,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C175,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E175,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C175,C175),"000"))</f>
+        <f aca="false">IF(OR(B175="",C175="",E175="",F175=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B175,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F175,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C175,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E175,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C175,C175),"000"))</f>
         <v>MT1-MR-TT-BW-014</v>
       </c>
     </row>
@@ -5661,7 +5661,7 @@
         <v>105</v>
       </c>
       <c r="G176" s="2" t="str">
-        <f aca="false">IF(OR(B176="",C176="",E176="",F176=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B176,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F176,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C176,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E176,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C176,C176),"000"))</f>
+        <f aca="false">IF(OR(B176="",C176="",E176="",F176=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B176,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F176,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C176,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E176,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C176,C176),"000"))</f>
         <v>MT1-MR-TT-BW-015</v>
       </c>
     </row>
@@ -5685,7 +5685,7 @@
         <v>105</v>
       </c>
       <c r="G177" s="2" t="str">
-        <f aca="false">IF(OR(B177="",C177="",E177="",F177=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B177,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F177,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C177,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E177,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C177,C177),"000"))</f>
+        <f aca="false">IF(OR(B177="",C177="",E177="",F177=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B177,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F177,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C177,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E177,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C177,C177),"000"))</f>
         <v>MT1-MR-LR-DT-142</v>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
         <v>105</v>
       </c>
       <c r="G178" s="2" t="str">
-        <f aca="false">IF(OR(B178="",C178="",E178="",F178=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B178,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F178,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C178,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E178,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C178,C178),"000"))</f>
+        <f aca="false">IF(OR(B178="",C178="",E178="",F178=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B178,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F178,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C178,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E178,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C178,C178),"000"))</f>
         <v>MT1-MR-TT-BW-016</v>
       </c>
     </row>
@@ -5733,7 +5733,7 @@
         <v>105</v>
       </c>
       <c r="G179" s="2" t="str">
-        <f aca="false">IF(OR(B179="",C179="",E179="",F179=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B179,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F179,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C179,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E179,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C179,C179),"000"))</f>
+        <f aca="false">IF(OR(B179="",C179="",E179="",F179=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B179,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F179,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C179,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E179,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C179,C179),"000"))</f>
         <v>MT1-MR-LR-CO-143</v>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
         <v>105</v>
       </c>
       <c r="G180" s="2" t="str">
-        <f aca="false">IF(OR(B180="",C180="",E180="",F180=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B180,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F180,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C180,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E180,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C180,C180),"000"))</f>
+        <f aca="false">IF(OR(B180="",C180="",E180="",F180=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B180,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F180,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C180,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E180,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C180,C180),"000"))</f>
         <v>MT1-MR-TT-BW-017</v>
       </c>
     </row>
@@ -5781,7 +5781,7 @@
         <v>105</v>
       </c>
       <c r="G181" s="2" t="str">
-        <f aca="false">IF(OR(B181="",C181="",E181="",F181=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B181,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F181,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C181,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E181,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C181,C181),"000"))</f>
+        <f aca="false">IF(OR(B181="",C181="",E181="",F181=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B181,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F181,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C181,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E181,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C181,C181),"000"))</f>
         <v>MT1-MR-MS-SW-004</v>
       </c>
     </row>
@@ -5805,7 +5805,7 @@
         <v>105</v>
       </c>
       <c r="G182" s="2" t="str">
-        <f aca="false">IF(OR(B182="",C182="",E182="",F182=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B182,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F182,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C182,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E182,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C182,C182),"000"))</f>
+        <f aca="false">IF(OR(B182="",C182="",E182="",F182=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B182,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F182,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C182,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E182,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C182,C182),"000"))</f>
         <v>MT1-MR-MS-SW-005</v>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
         <v>105</v>
       </c>
       <c r="G183" s="2" t="str">
-        <f aca="false">IF(OR(B183="",C183="",E183="",F183=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B183,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F183,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C183,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E183,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C183,C183),"000"))</f>
+        <f aca="false">IF(OR(B183="",C183="",E183="",F183=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B183,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F183,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C183,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E183,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C183,C183),"000"))</f>
         <v>MT1-MR-TT-BW-018</v>
       </c>
     </row>
@@ -5853,7 +5853,7 @@
         <v>105</v>
       </c>
       <c r="G184" s="2" t="str">
-        <f aca="false">IF(OR(B184="",C184="",E184="",F184=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B184,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F184,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C184,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E184,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C184,C184),"000"))</f>
+        <f aca="false">IF(OR(B184="",C184="",E184="",F184=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B184,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F184,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C184,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E184,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C184,C184),"000"))</f>
         <v>MT1-MR-D1-TC-002</v>
       </c>
     </row>
@@ -5877,7 +5877,7 @@
         <v>105</v>
       </c>
       <c r="G185" s="2" t="str">
-        <f aca="false">IF(OR(B185="",C185="",E185="",F185=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B185,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F185,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C185,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E185,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C185,C185),"000"))</f>
+        <f aca="false">IF(OR(B185="",C185="",E185="",F185=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B185,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F185,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C185,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E185,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C185,C185),"000"))</f>
         <v>MT1-MR-D1-TC-003</v>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
         <v>105</v>
       </c>
       <c r="G186" s="2" t="str">
-        <f aca="false">IF(OR(B186="",C186="",E186="",F186=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B186,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F186,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C186,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E186,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C186,C186),"000"))</f>
+        <f aca="false">IF(OR(B186="",C186="",E186="",F186=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B186,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F186,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C186,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E186,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C186,C186),"000"))</f>
         <v>MT1-MR-TT-BW-019</v>
       </c>
     </row>
@@ -5925,7 +5925,7 @@
         <v>105</v>
       </c>
       <c r="G187" s="2" t="str">
-        <f aca="false">IF(OR(B187="",C187="",E187="",F187=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B187,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F187,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C187,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E187,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C187,C187),"000"))</f>
+        <f aca="false">IF(OR(B187="",C187="",E187="",F187=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B187,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F187,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C187,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E187,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C187,C187),"000"))</f>
         <v>MT1-MR-WB-WA-002</v>
       </c>
     </row>
@@ -5949,7 +5949,7 @@
         <v>105</v>
       </c>
       <c r="G188" s="2" t="str">
-        <f aca="false">IF(OR(B188="",C188="",E188="",F188=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B188,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F188,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C188,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E188,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C188,C188),"000"))</f>
+        <f aca="false">IF(OR(B188="",C188="",E188="",F188=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B188,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F188,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C188,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E188,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C188,C188),"000"))</f>
         <v>MT1-MR-TT-BW-020</v>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
         <v>105</v>
       </c>
       <c r="G189" s="2" t="str">
-        <f aca="false">IF(OR(B189="",C189="",E189="",F189=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B189,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F189,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C189,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E189,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C189,C189),"000"))</f>
+        <f aca="false">IF(OR(B189="",C189="",E189="",F189=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B189,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F189,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C189,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E189,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C189,C189),"000"))</f>
         <v>MT1-MR-TT-BW-021</v>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
         <v>105</v>
       </c>
       <c r="G190" s="2" t="str">
-        <f aca="false">IF(OR(B190="",C190="",E190="",F190=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B190,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F190,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C190,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E190,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C190,C190),"000"))</f>
+        <f aca="false">IF(OR(B190="",C190="",E190="",F190=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B190,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F190,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C190,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E190,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C190,C190),"000"))</f>
         <v>MT1-MR-TT-BW-022</v>
       </c>
     </row>
@@ -6021,7 +6021,7 @@
         <v>105</v>
       </c>
       <c r="G191" s="2" t="str">
-        <f aca="false">IF(OR(B191="",C191="",E191="",F191=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B191,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F191,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C191,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E191,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C191,C191),"000"))</f>
+        <f aca="false">IF(OR(B191="",C191="",E191="",F191=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B191,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F191,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C191,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E191,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C191,C191),"000"))</f>
         <v>MT1-MR-TT-BW-023</v>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
         <v>105</v>
       </c>
       <c r="G192" s="2" t="str">
-        <f aca="false">IF(OR(B192="",C192="",E192="",F192=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B192,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F192,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C192,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E192,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C192,C192),"000"))</f>
+        <f aca="false">IF(OR(B192="",C192="",E192="",F192=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B192,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F192,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C192,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E192,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C192,C192),"000"))</f>
         <v>MT1-MR-D1-TC-004</v>
       </c>
     </row>
@@ -6069,7 +6069,7 @@
         <v>105</v>
       </c>
       <c r="G193" s="2" t="str">
-        <f aca="false">IF(OR(B193="",C193="",E193="",F193=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B193,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F193,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C193,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E193,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C193,C193),"000"))</f>
+        <f aca="false">IF(OR(B193="",C193="",E193="",F193=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B193,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F193,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C193,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E193,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C193,C193),"000"))</f>
         <v>MT1-MR-D1-TC-005</v>
       </c>
     </row>
@@ -6093,7 +6093,7 @@
         <v>105</v>
       </c>
       <c r="G194" s="2" t="str">
-        <f aca="false">IF(OR(B194="",C194="",E194="",F194=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B194,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F194,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C194,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E194,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C194,C194),"000"))</f>
+        <f aca="false">IF(OR(B194="",C194="",E194="",F194=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B194,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F194,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C194,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E194,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C194,C194),"000"))</f>
         <v>MT1-MR-D1-TC-006</v>
       </c>
     </row>
@@ -6117,7 +6117,7 @@
         <v>105</v>
       </c>
       <c r="G195" s="2" t="str">
-        <f aca="false">IF(OR(B195="",C195="",E195="",F195=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B195,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F195,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C195,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E195,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C195,C195),"000"))</f>
+        <f aca="false">IF(OR(B195="",C195="",E195="",F195=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B195,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F195,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C195,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E195,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C195,C195),"000"))</f>
         <v>MT1-MR-MS-SW-006</v>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
         <v>105</v>
       </c>
       <c r="G196" s="2" t="str">
-        <f aca="false">IF(OR(B196="",C196="",E196="",F196=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B196,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F196,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C196,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E196,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C196,C196),"000"))</f>
+        <f aca="false">IF(OR(B196="",C196="",E196="",F196=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B196,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F196,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C196,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E196,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C196,C196),"000"))</f>
         <v>MT1-MR-WB-WA-003</v>
       </c>
     </row>
@@ -6165,7 +6165,7 @@
         <v>105</v>
       </c>
       <c r="G197" s="2" t="str">
-        <f aca="false">IF(OR(B197="",C197="",E197="",F197=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B197,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F197,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C197,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E197,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C197,C197),"000"))</f>
+        <f aca="false">IF(OR(B197="",C197="",E197="",F197=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B197,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F197,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C197,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E197,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C197,C197),"000"))</f>
         <v>MT1-MR-TT-BW-024</v>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
         <v>105</v>
       </c>
       <c r="G198" s="2" t="str">
-        <f aca="false">IF(OR(B198="",C198="",E198="",F198=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B198,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F198,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C198,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E198,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C198,C198),"000"))</f>
+        <f aca="false">IF(OR(B198="",C198="",E198="",F198=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B198,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F198,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C198,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E198,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C198,C198),"000"))</f>
         <v>MT1-MR-TT-BW-025</v>
       </c>
     </row>
@@ -6213,7 +6213,7 @@
         <v>105</v>
       </c>
       <c r="G199" s="2" t="str">
-        <f aca="false">IF(OR(B199="",C199="",E199="",F199=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B199,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F199,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C199,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E199,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C199,C199),"000"))</f>
+        <f aca="false">IF(OR(B199="",C199="",E199="",F199=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B199,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F199,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C199,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E199,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C199,C199),"000"))</f>
         <v>MT1-MR-WB-WA-004</v>
       </c>
     </row>
@@ -6237,7 +6237,7 @@
         <v>105</v>
       </c>
       <c r="G200" s="2" t="str">
-        <f aca="false">IF(OR(B200="",C200="",E200="",F200=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B200,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F200,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C200,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E200,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C200,C200),"000"))</f>
+        <f aca="false">IF(OR(B200="",C200="",E200="",F200=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B200,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F200,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C200,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E200,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C200,C200),"000"))</f>
         <v>MT1-MR-D1-TC-007</v>
       </c>
     </row>
@@ -6261,7 +6261,7 @@
         <v>105</v>
       </c>
       <c r="G201" s="2" t="str">
-        <f aca="false">IF(OR(B201="",C201="",E201="",F201=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B201,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F201,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C201,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E201,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C201,C201),"000"))</f>
+        <f aca="false">IF(OR(B201="",C201="",E201="",F201=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B201,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F201,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C201,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E201,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C201,C201),"000"))</f>
         <v>MT1-MR-TT-BW-026</v>
       </c>
     </row>
@@ -6285,7 +6285,7 @@
         <v>105</v>
       </c>
       <c r="G202" s="2" t="str">
-        <f aca="false">IF(OR(B202="",C202="",E202="",F202=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B202,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F202,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C202,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E202,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C202,C202),"000"))</f>
+        <f aca="false">IF(OR(B202="",C202="",E202="",F202=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B202,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F202,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C202,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E202,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C202,C202),"000"))</f>
         <v>MT1-MR-D2-TC-004</v>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
         <v>105</v>
       </c>
       <c r="G203" s="2" t="str">
-        <f aca="false">IF(OR(B203="",C203="",E203="",F203=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B203,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F203,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C203,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E203,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C203,C203),"000"))</f>
+        <f aca="false">IF(OR(B203="",C203="",E203="",F203=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B203,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F203,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C203,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E203,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C203,C203),"000"))</f>
         <v>MT1-MR-D1-TC-008</v>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
         <v>105</v>
       </c>
       <c r="G204" s="2" t="str">
-        <f aca="false">IF(OR(B204="",C204="",E204="",F204=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B204,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F204,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C204,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E204,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C204,C204),"000"))</f>
+        <f aca="false">IF(OR(B204="",C204="",E204="",F204=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B204,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F204,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C204,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E204,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C204,C204),"000"))</f>
         <v>MT1-MR-CC-CB-001</v>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
         <v>105</v>
       </c>
       <c r="G205" s="2" t="str">
-        <f aca="false">IF(OR(B205="",C205="",E205="",F205=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B205,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F205,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C205,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E205,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C205,C205),"000"))</f>
+        <f aca="false">IF(OR(B205="",C205="",E205="",F205=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B205,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F205,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C205,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E205,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C205,C205),"000"))</f>
         <v>MT1-MR-TL-BW-005</v>
       </c>
     </row>
@@ -6381,7 +6381,7 @@
         <v>105</v>
       </c>
       <c r="G206" s="2" t="str">
-        <f aca="false">IF(OR(B206="",C206="",E206="",F206=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B206,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F206,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C206,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E206,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C206,C206),"000"))</f>
+        <f aca="false">IF(OR(B206="",C206="",E206="",F206=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B206,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F206,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C206,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E206,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C206,C206),"000"))</f>
         <v>MT1-MR-LR-DT-144</v>
       </c>
     </row>
@@ -6405,7 +6405,7 @@
         <v>105</v>
       </c>
       <c r="G207" s="2" t="str">
-        <f aca="false">IF(OR(B207="",C207="",E207="",F207=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B207,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F207,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C207,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E207,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C207,C207),"000"))</f>
+        <f aca="false">IF(OR(B207="",C207="",E207="",F207=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B207,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F207,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C207,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E207,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C207,C207),"000"))</f>
         <v>MT1-MR-LR-CO-145</v>
       </c>
     </row>
@@ -6429,7 +6429,7 @@
         <v>105</v>
       </c>
       <c r="G208" s="2" t="str">
-        <f aca="false">IF(OR(B208="",C208="",E208="",F208=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B208,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F208,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C208,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E208,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C208,C208),"000"))</f>
+        <f aca="false">IF(OR(B208="",C208="",E208="",F208=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B208,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F208,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C208,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E208,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C208,C208),"000"))</f>
         <v>MT1-MR-LR-DT-146</v>
       </c>
     </row>
@@ -6453,7 +6453,7 @@
         <v>105</v>
       </c>
       <c r="G209" s="2" t="str">
-        <f aca="false">IF(OR(B209="",C209="",E209="",F209=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B209,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F209,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C209,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E209,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C209,C209),"000"))</f>
+        <f aca="false">IF(OR(B209="",C209="",E209="",F209=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B209,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F209,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C209,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E209,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C209,C209),"000"))</f>
         <v>MT1-MR-LR-CO-147</v>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
         <v>105</v>
       </c>
       <c r="G210" s="2" t="str">
-        <f aca="false">IF(OR(B210="",C210="",E210="",F210=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B210,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F210,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C210,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E210,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C210,C210),"000"))</f>
+        <f aca="false">IF(OR(B210="",C210="",E210="",F210=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B210,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F210,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C210,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E210,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C210,C210),"000"))</f>
         <v>MT1-MR-LR-DT-148</v>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
         <v>105</v>
       </c>
       <c r="G211" s="2" t="str">
-        <f aca="false">IF(OR(B211="",C211="",E211="",F211=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B211,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F211,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C211,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E211,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C211,C211),"000"))</f>
+        <f aca="false">IF(OR(B211="",C211="",E211="",F211=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B211,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F211,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C211,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E211,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C211,C211),"000"))</f>
         <v>MT1-MR-LR-DT-149</v>
       </c>
     </row>
@@ -6525,7 +6525,7 @@
         <v>105</v>
       </c>
       <c r="G212" s="2" t="str">
-        <f aca="false">IF(OR(B212="",C212="",E212="",F212=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B212,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F212,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C212,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E212,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C212,C212),"000"))</f>
+        <f aca="false">IF(OR(B212="",C212="",E212="",F212=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B212,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F212,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C212,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E212,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C212,C212),"000"))</f>
         <v>MT1-MR-LR-DT-150</v>
       </c>
     </row>
@@ -6549,7 +6549,7 @@
         <v>105</v>
       </c>
       <c r="G213" s="2" t="str">
-        <f aca="false">IF(OR(B213="",C213="",E213="",F213=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B213,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F213,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C213,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E213,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C213,C213),"000"))</f>
+        <f aca="false">IF(OR(B213="",C213="",E213="",F213=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B213,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F213,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C213,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E213,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C213,C213),"000"))</f>
         <v>MT1-MR-LR-DT-151</v>
       </c>
     </row>
@@ -6573,7 +6573,7 @@
         <v>105</v>
       </c>
       <c r="G214" s="2" t="str">
-        <f aca="false">IF(OR(B214="",C214="",E214="",F214=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B214,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F214,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C214,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E214,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C214,C214),"000"))</f>
+        <f aca="false">IF(OR(B214="",C214="",E214="",F214=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B214,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F214,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C214,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E214,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C214,C214),"000"))</f>
         <v>MT1-MR-LR-DT-152</v>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
         <v>105</v>
       </c>
       <c r="G215" s="2" t="str">
-        <f aca="false">IF(OR(B215="",C215="",E215="",F215=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B215,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F215,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C215,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E215,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C215,C215),"000"))</f>
+        <f aca="false">IF(OR(B215="",C215="",E215="",F215=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B215,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F215,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C215,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E215,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C215,C215),"000"))</f>
         <v>MT1-MR-LR-CO-153</v>
       </c>
     </row>
@@ -6621,7 +6621,7 @@
         <v>105</v>
       </c>
       <c r="G216" s="2" t="str">
-        <f aca="false">IF(OR(B216="",C216="",E216="",F216=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B216,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F216,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C216,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E216,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C216,C216),"000"))</f>
+        <f aca="false">IF(OR(B216="",C216="",E216="",F216=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B216,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F216,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C216,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E216,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C216,C216),"000"))</f>
         <v>MT1-MR-LR-DT-154</v>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
         <v>105</v>
       </c>
       <c r="G217" s="2" t="str">
-        <f aca="false">IF(OR(B217="",C217="",E217="",F217=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B217,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F217,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C217,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E217,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C217,C217),"000"))</f>
+        <f aca="false">IF(OR(B217="",C217="",E217="",F217=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B217,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F217,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C217,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E217,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C217,C217),"000"))</f>
         <v>MT1-MR-LR-CO-155</v>
       </c>
     </row>
@@ -6669,7 +6669,7 @@
         <v>105</v>
       </c>
       <c r="G218" s="2" t="str">
-        <f aca="false">IF(OR(B218="",C218="",E218="",F218=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B218,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F218,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C218,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E218,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C218,C218),"000"))</f>
+        <f aca="false">IF(OR(B218="",C218="",E218="",F218=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B218,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F218,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C218,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E218,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C218,C218),"000"))</f>
         <v>MT1-MR-LR-CO-156</v>
       </c>
     </row>
@@ -6693,7 +6693,7 @@
         <v>105</v>
       </c>
       <c r="G219" s="2" t="str">
-        <f aca="false">IF(OR(B219="",C219="",E219="",F219=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B219,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F219,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C219,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E219,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C219,C219),"000"))</f>
+        <f aca="false">IF(OR(B219="",C219="",E219="",F219=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B219,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F219,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C219,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E219,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C219,C219),"000"))</f>
         <v>MT1-MR-LR-CO-157</v>
       </c>
     </row>
@@ -6717,7 +6717,7 @@
         <v>105</v>
       </c>
       <c r="G220" s="2" t="str">
-        <f aca="false">IF(OR(B220="",C220="",E220="",F220=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B220,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F220,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C220,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E220,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C220,C220),"000"))</f>
+        <f aca="false">IF(OR(B220="",C220="",E220="",F220=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B220,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F220,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C220,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E220,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C220,C220),"000"))</f>
         <v>MT1-MR-LR-DT-158</v>
       </c>
     </row>
@@ -6741,7 +6741,7 @@
         <v>105</v>
       </c>
       <c r="G221" s="2" t="str">
-        <f aca="false">IF(OR(B221="",C221="",E221="",F221=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B221,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F221,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C221,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E221,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C221,C221),"000"))</f>
+        <f aca="false">IF(OR(B221="",C221="",E221="",F221=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B221,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F221,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C221,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E221,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C221,C221),"000"))</f>
         <v>MT1-MR-LR-DT-159</v>
       </c>
     </row>
@@ -6765,7 +6765,7 @@
         <v>105</v>
       </c>
       <c r="G222" s="2" t="str">
-        <f aca="false">IF(OR(B222="",C222="",E222="",F222=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B222,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F222,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C222,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E222,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C222,C222),"000"))</f>
+        <f aca="false">IF(OR(B222="",C222="",E222="",F222=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B222,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F222,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C222,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E222,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C222,C222),"000"))</f>
         <v>MT1-MR-LR-DT-160</v>
       </c>
     </row>
@@ -6789,7 +6789,7 @@
         <v>105</v>
       </c>
       <c r="G223" s="2" t="str">
-        <f aca="false">IF(OR(B223="",C223="",E223="",F223=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B223,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F223,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C223,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E223,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C223,C223),"000"))</f>
+        <f aca="false">IF(OR(B223="",C223="",E223="",F223=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B223,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F223,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C223,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E223,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C223,C223),"000"))</f>
         <v>MT1-MR-LR-DT-161</v>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
         <v>105</v>
       </c>
       <c r="G224" s="2" t="str">
-        <f aca="false">IF(OR(B224="",C224="",E224="",F224=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B224,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F224,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C224,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E224,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C224,C224),"000"))</f>
+        <f aca="false">IF(OR(B224="",C224="",E224="",F224=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B224,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F224,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C224,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E224,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C224,C224),"000"))</f>
         <v>MT1-MR-LR-DT-162</v>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
         <v>105</v>
       </c>
       <c r="G225" s="2" t="str">
-        <f aca="false">IF(OR(B225="",C225="",E225="",F225=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B225,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F225,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C225,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E225,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C225,C225),"000"))</f>
+        <f aca="false">IF(OR(B225="",C225="",E225="",F225=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B225,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F225,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C225,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E225,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C225,C225),"000"))</f>
         <v>MT1-MR-LR-DT-163</v>
       </c>
     </row>
@@ -6861,7 +6861,7 @@
         <v>105</v>
       </c>
       <c r="G226" s="2" t="str">
-        <f aca="false">IF(OR(B226="",C226="",E226="",F226=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B226,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F226,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C226,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E226,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C226,C226),"000"))</f>
+        <f aca="false">IF(OR(B226="",C226="",E226="",F226=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B226,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F226,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C226,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E226,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C226,C226),"000"))</f>
         <v>MT1-MR-LR-DT-164</v>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
         <v>105</v>
       </c>
       <c r="G227" s="2" t="str">
-        <f aca="false">IF(OR(B227="",C227="",E227="",F227=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B227,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F227,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C227,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E227,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C227,C227),"000"))</f>
+        <f aca="false">IF(OR(B227="",C227="",E227="",F227=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B227,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F227,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C227,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E227,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C227,C227),"000"))</f>
         <v>MT1-MR-LR-DT-165</v>
       </c>
     </row>
@@ -6909,7 +6909,7 @@
         <v>105</v>
       </c>
       <c r="G228" s="2" t="str">
-        <f aca="false">IF(OR(B228="",C228="",E228="",F228=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B228,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F228,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C228,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E228,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C228,C228),"000"))</f>
+        <f aca="false">IF(OR(B228="",C228="",E228="",F228=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B228,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F228,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C228,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E228,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C228,C228),"000"))</f>
         <v>MT1-MR-LR-DT-166</v>
       </c>
     </row>
@@ -6933,7 +6933,7 @@
         <v>105</v>
       </c>
       <c r="G229" s="2" t="str">
-        <f aca="false">IF(OR(B229="",C229="",E229="",F229=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B229,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F229,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C229,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E229,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C229,C229),"000"))</f>
+        <f aca="false">IF(OR(B229="",C229="",E229="",F229=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B229,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F229,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C229,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E229,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C229,C229),"000"))</f>
         <v>MT1-MR-LR-DT-167</v>
       </c>
     </row>
@@ -6957,7 +6957,7 @@
         <v>105</v>
       </c>
       <c r="G230" s="2" t="str">
-        <f aca="false">IF(OR(B230="",C230="",E230="",F230=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B230,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F230,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C230,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E230,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C230,C230),"000"))</f>
+        <f aca="false">IF(OR(B230="",C230="",E230="",F230=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B230,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F230,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C230,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E230,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C230,C230),"000"))</f>
         <v>MT1-MR-LR-DT-168</v>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
         <v>105</v>
       </c>
       <c r="G231" s="2" t="str">
-        <f aca="false">IF(OR(B231="",C231="",E231="",F231=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B231,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F231,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C231,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E231,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C231,C231),"000"))</f>
+        <f aca="false">IF(OR(B231="",C231="",E231="",F231=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B231,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F231,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C231,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E231,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C231,C231),"000"))</f>
         <v>MT1-MR-LR-CO-169</v>
       </c>
     </row>
@@ -7005,7 +7005,7 @@
         <v>105</v>
       </c>
       <c r="G232" s="2" t="str">
-        <f aca="false">IF(OR(B232="",C232="",E232="",F232=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B232,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F232,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C232,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E232,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C232,C232),"000"))</f>
+        <f aca="false">IF(OR(B232="",C232="",E232="",F232=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B232,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F232,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C232,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E232,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C232,C232),"000"))</f>
         <v>MT1-MR-LR-DT-170</v>
       </c>
     </row>
@@ -7029,7 +7029,7 @@
         <v>105</v>
       </c>
       <c r="G233" s="2" t="str">
-        <f aca="false">IF(OR(B233="",C233="",E233="",F233=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B233,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F233,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C233,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E233,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C233,C233),"000"))</f>
+        <f aca="false">IF(OR(B233="",C233="",E233="",F233=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B233,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F233,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C233,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E233,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C233,C233),"000"))</f>
         <v>MT1-MR-TL-BW-006</v>
       </c>
     </row>
@@ -7053,7 +7053,7 @@
         <v>105</v>
       </c>
       <c r="G234" s="2" t="str">
-        <f aca="false">IF(OR(B234="",C234="",E234="",F234=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B234,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F234,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C234,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E234,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C234,C234),"000"))</f>
+        <f aca="false">IF(OR(B234="",C234="",E234="",F234=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B234,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F234,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C234,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E234,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C234,C234),"000"))</f>
         <v>MT1-MR-TL-BW-007</v>
       </c>
     </row>
@@ -7077,7 +7077,7 @@
         <v>105</v>
       </c>
       <c r="G235" s="2" t="str">
-        <f aca="false">IF(OR(B235="",C235="",E235="",F235=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B235,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F235,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C235,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E235,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C235,C235),"000"))</f>
+        <f aca="false">IF(OR(B235="",C235="",E235="",F235=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B235,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F235,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C235,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E235,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C235,C235),"000"))</f>
         <v>MT1-MR-TL-BW-008</v>
       </c>
     </row>
@@ -7101,7 +7101,7 @@
         <v>105</v>
       </c>
       <c r="G236" s="2" t="str">
-        <f aca="false">IF(OR(B236="",C236="",E236="",F236=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B236,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F236,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C236,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E236,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C236,C236),"000"))</f>
+        <f aca="false">IF(OR(B236="",C236="",E236="",F236=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B236,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F236,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C236,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E236,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C236,C236),"000"))</f>
         <v>MT1-MR-TL-BW-009</v>
       </c>
     </row>
@@ -7125,7 +7125,7 @@
         <v>105</v>
       </c>
       <c r="G237" s="2" t="str">
-        <f aca="false">IF(OR(B237="",C237="",E237="",F237=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B237,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F237,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C237,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E237,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C237,C237),"000"))</f>
+        <f aca="false">IF(OR(B237="",C237="",E237="",F237=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B237,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F237,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C237,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E237,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C237,C237),"000"))</f>
         <v>MT1-MR-LR-DT-171</v>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
         <v>105</v>
       </c>
       <c r="G238" s="2" t="str">
-        <f aca="false">IF(OR(B238="",C238="",E238="",F238=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B238,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F238,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C238,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E238,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C238,C238),"000"))</f>
+        <f aca="false">IF(OR(B238="",C238="",E238="",F238=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B238,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F238,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C238,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E238,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C238,C238),"000"))</f>
         <v>MT1-MR-LR-CO-172</v>
       </c>
     </row>
@@ -7173,7 +7173,7 @@
         <v>105</v>
       </c>
       <c r="G239" s="2" t="str">
-        <f aca="false">IF(OR(B239="",C239="",E239="",F239=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B239,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F239,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C239,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E239,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C239,C239),"000"))</f>
+        <f aca="false">IF(OR(B239="",C239="",E239="",F239=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B239,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F239,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C239,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E239,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C239,C239),"000"))</f>
         <v>MT1-MR-LR-CO-173</v>
       </c>
     </row>
@@ -7197,7 +7197,7 @@
         <v>269</v>
       </c>
       <c r="G240" s="2" t="str">
-        <f aca="false">IF(OR(B240="",C240="",E240="",F240=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B240,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F240,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C240,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E240,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C240,C240),"000"))</f>
+        <f aca="false">IF(OR(B240="",C240="",E240="",F240=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B240,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F240,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C240,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E240,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C240,C240),"000"))</f>
         <v>MT1-QR-LR-DT-174</v>
       </c>
     </row>
@@ -7221,7 +7221,7 @@
         <v>269</v>
       </c>
       <c r="G241" s="2" t="str">
-        <f aca="false">IF(OR(B241="",C241="",E241="",F241=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B241,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F241,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C241,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E241,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C241,C241),"000"))</f>
+        <f aca="false">IF(OR(B241="",C241="",E241="",F241=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B241,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F241,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C241,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E241,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C241,C241),"000"))</f>
         <v>MT1-QR-LR-DT-175</v>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
         <v>269</v>
       </c>
       <c r="G242" s="2" t="str">
-        <f aca="false">IF(OR(B242="",C242="",E242="",F242=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B242,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F242,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C242,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E242,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C242,C242),"000"))</f>
+        <f aca="false">IF(OR(B242="",C242="",E242="",F242=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B242,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F242,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C242,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E242,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C242,C242),"000"))</f>
         <v>MT1-QR-LR-CO-176</v>
       </c>
     </row>
@@ -7269,7 +7269,7 @@
         <v>269</v>
       </c>
       <c r="G243" s="2" t="str">
-        <f aca="false">IF(OR(B243="",C243="",E243="",F243=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B243,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F243,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C243,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E243,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C243,C243),"000"))</f>
+        <f aca="false">IF(OR(B243="",C243="",E243="",F243=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B243,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F243,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C243,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E243,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C243,C243),"000"))</f>
         <v>MT1-QR-LR-DT-177</v>
       </c>
     </row>
@@ -7293,7 +7293,7 @@
         <v>269</v>
       </c>
       <c r="G244" s="2" t="str">
-        <f aca="false">IF(OR(B244="",C244="",E244="",F244=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B244,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F244,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C244,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E244,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C244,C244),"000"))</f>
+        <f aca="false">IF(OR(B244="",C244="",E244="",F244=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B244,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F244,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C244,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E244,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C244,C244),"000"))</f>
         <v>MT1-QR-LR-CO-178</v>
       </c>
     </row>
@@ -7317,7 +7317,7 @@
         <v>269</v>
       </c>
       <c r="G245" s="2" t="str">
-        <f aca="false">IF(OR(B245="",C245="",E245="",F245=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B245,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F245,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C245,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E245,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C245,C245),"000"))</f>
+        <f aca="false">IF(OR(B245="",C245="",E245="",F245=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B245,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F245,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C245,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E245,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C245,C245),"000"))</f>
         <v>MT1-QR-LR-DT-179</v>
       </c>
     </row>
@@ -7341,7 +7341,7 @@
         <v>269</v>
       </c>
       <c r="G246" s="2" t="str">
-        <f aca="false">IF(OR(B246="",C246="",E246="",F246=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B246,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F246,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C246,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E246,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C246,C246),"000"))</f>
+        <f aca="false">IF(OR(B246="",C246="",E246="",F246=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B246,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F246,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C246,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E246,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C246,C246),"000"))</f>
         <v>MT1-QR-LR-CO-180</v>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
         <v>269</v>
       </c>
       <c r="G247" s="2" t="str">
-        <f aca="false">IF(OR(B247="",C247="",E247="",F247=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B247,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F247,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C247,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E247,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C247,C247),"000"))</f>
+        <f aca="false">IF(OR(B247="",C247="",E247="",F247=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B247,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F247,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C247,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E247,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C247,C247),"000"))</f>
         <v>MT1-QR-LR-CO-181</v>
       </c>
     </row>
@@ -7389,7 +7389,7 @@
         <v>269</v>
       </c>
       <c r="G248" s="2" t="str">
-        <f aca="false">IF(OR(B248="",C248="",E248="",F248=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B248,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F248,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C248,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E248,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C248,C248),"000"))</f>
+        <f aca="false">IF(OR(B248="",C248="",E248="",F248=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B248,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F248,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C248,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E248,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C248,C248),"000"))</f>
         <v>MT1-QR-LR-CO-182</v>
       </c>
     </row>
@@ -7413,7 +7413,7 @@
         <v>279</v>
       </c>
       <c r="G249" s="2" t="str">
-        <f aca="false">IF(OR(B249="",C249="",E249="",F249=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B249,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F249,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C249,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E249,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C249,C249),"000"))</f>
+        <f aca="false">IF(OR(B249="",C249="",E249="",F249=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B249,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F249,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C249,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E249,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C249,C249),"000"))</f>
         <v>MT1-GM-LR-DT-183</v>
       </c>
     </row>
@@ -7437,7 +7437,7 @@
         <v>279</v>
       </c>
       <c r="G250" s="2" t="str">
-        <f aca="false">IF(OR(B250="",C250="",E250="",F250=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B250,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F250,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C250,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E250,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C250,C250),"000"))</f>
+        <f aca="false">IF(OR(B250="",C250="",E250="",F250=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B250,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F250,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C250,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E250,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C250,C250),"000"))</f>
         <v>MT1-GM-CD-LF-001</v>
       </c>
     </row>
@@ -7461,7 +7461,7 @@
         <v>279</v>
       </c>
       <c r="G251" s="2" t="str">
-        <f aca="false">IF(OR(B251="",C251="",E251="",F251=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B251,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F251,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C251,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E251,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C251,C251),"000"))</f>
+        <f aca="false">IF(OR(B251="",C251="",E251="",F251=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B251,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F251,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C251,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E251,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C251,C251),"000"))</f>
         <v>MT1-GM-TB-BW-002</v>
       </c>
     </row>
@@ -7485,7 +7485,7 @@
         <v>279</v>
       </c>
       <c r="G252" s="2" t="str">
-        <f aca="false">IF(OR(B252="",C252="",E252="",F252=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B252,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F252,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C252,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E252,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C252,C252),"000"))</f>
+        <f aca="false">IF(OR(B252="",C252="",E252="",F252=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B252,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F252,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C252,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E252,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C252,C252),"000"))</f>
         <v>MT1-GM-WB-WA-005</v>
       </c>
     </row>
@@ -7509,7 +7509,7 @@
         <v>279</v>
       </c>
       <c r="G253" s="2" t="str">
-        <f aca="false">IF(OR(B253="",C253="",E253="",F253=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B253,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F253,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C253,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E253,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C253,C253),"000"))</f>
+        <f aca="false">IF(OR(B253="",C253="",E253="",F253=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B253,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F253,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C253,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E253,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C253,C253),"000"))</f>
         <v>MT1-GM-WB-WA-006</v>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
         <v>279</v>
       </c>
       <c r="G254" s="2" t="str">
-        <f aca="false">IF(OR(B254="",C254="",E254="",F254=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B254,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F254,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C254,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E254,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C254,C254),"000"))</f>
+        <f aca="false">IF(OR(B254="",C254="",E254="",F254=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B254,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F254,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C254,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E254,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C254,C254),"000"))</f>
         <v>MT1-GM-FL-BW-001</v>
       </c>
     </row>
@@ -7557,7 +7557,7 @@
         <v>279</v>
       </c>
       <c r="G255" s="2" t="str">
-        <f aca="false">IF(OR(B255="",C255="",E255="",F255=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B255,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F255,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C255,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E255,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C255,C255),"000"))</f>
+        <f aca="false">IF(OR(B255="",C255="",E255="",F255=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B255,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F255,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C255,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E255,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C255,C255),"000"))</f>
         <v>MT1-GM-FL-BW-002</v>
       </c>
     </row>
@@ -7581,7 +7581,7 @@
         <v>279</v>
       </c>
       <c r="G256" s="2" t="str">
-        <f aca="false">IF(OR(B256="",C256="",E256="",F256=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B256,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F256,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C256,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E256,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C256,C256),"000"))</f>
+        <f aca="false">IF(OR(B256="",C256="",E256="",F256=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B256,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F256,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C256,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E256,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C256,C256),"000"))</f>
         <v>MT1-GM-CM-CB-002</v>
       </c>
     </row>
@@ -7605,7 +7605,7 @@
         <v>279</v>
       </c>
       <c r="G257" s="2" t="str">
-        <f aca="false">IF(OR(B257="",C257="",E257="",F257=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B257,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F257,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C257,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E257,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C257,C257),"000"))</f>
+        <f aca="false">IF(OR(B257="",C257="",E257="",F257=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B257,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F257,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C257,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E257,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C257,C257),"000"))</f>
         <v>MT1-GM-CM-CB-003</v>
       </c>
     </row>
@@ -7629,7 +7629,7 @@
         <v>279</v>
       </c>
       <c r="G258" s="2" t="str">
-        <f aca="false">IF(OR(B258="",C258="",E258="",F258=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B258,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F258,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C258,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E258,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C258,C258),"000"))</f>
+        <f aca="false">IF(OR(B258="",C258="",E258="",F258=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B258,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F258,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C258,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E258,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C258,C258),"000"))</f>
         <v>MT1-GM-CM-CB-004</v>
       </c>
     </row>
@@ -7653,7 +7653,7 @@
         <v>279</v>
       </c>
       <c r="G259" s="2" t="str">
-        <f aca="false">IF(OR(B259="",C259="",E259="",F259=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B259,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F259,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C259,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E259,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C259,C259),"000"))</f>
+        <f aca="false">IF(OR(B259="",C259="",E259="",F259=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B259,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F259,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C259,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E259,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C259,C259),"000"))</f>
         <v>MT1-GM-CM-CB-005</v>
       </c>
     </row>
@@ -7677,7 +7677,7 @@
         <v>279</v>
       </c>
       <c r="G260" s="2" t="str">
-        <f aca="false">IF(OR(B260="",C260="",E260="",F260=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B260,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F260,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C260,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E260,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C260,C260),"000"))</f>
+        <f aca="false">IF(OR(B260="",C260="",E260="",F260=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B260,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F260,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C260,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E260,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C260,C260),"000"))</f>
         <v>MT1-GM-CM-CB-006</v>
       </c>
     </row>
@@ -7701,7 +7701,7 @@
         <v>279</v>
       </c>
       <c r="G261" s="2" t="str">
-        <f aca="false">IF(OR(B261="",C261="",E261="",F261=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B261,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F261,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C261,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E261,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C261,C261),"000"))</f>
+        <f aca="false">IF(OR(B261="",C261="",E261="",F261=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B261,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F261,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C261,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E261,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C261,C261),"000"))</f>
         <v>MT1-GM-CM-CB-007</v>
       </c>
     </row>
@@ -7725,7 +7725,7 @@
         <v>279</v>
       </c>
       <c r="G262" s="2" t="str">
-        <f aca="false">IF(OR(B262="",C262="",E262="",F262=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B262,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F262,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C262,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E262,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C262,C262),"000"))</f>
+        <f aca="false">IF(OR(B262="",C262="",E262="",F262=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B262,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F262,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C262,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E262,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C262,C262),"000"))</f>
         <v>MT1-GM-CM-CB-008</v>
       </c>
     </row>
@@ -7749,7 +7749,7 @@
         <v>279</v>
       </c>
       <c r="G263" s="2" t="str">
-        <f aca="false">IF(OR(B263="",C263="",E263="",F263=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B263,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F263,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C263,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E263,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C263,C263),"000"))</f>
+        <f aca="false">IF(OR(B263="",C263="",E263="",F263=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B263,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F263,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C263,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E263,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C263,C263),"000"))</f>
         <v>MT1-GM-HL-CO-001</v>
       </c>
     </row>
@@ -7773,7 +7773,7 @@
         <v>279</v>
       </c>
       <c r="G264" s="2" t="str">
-        <f aca="false">IF(OR(B264="",C264="",E264="",F264=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B264,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F264,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C264,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E264,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C264,C264),"000"))</f>
+        <f aca="false">IF(OR(B264="",C264="",E264="",F264=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B264,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F264,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C264,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E264,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C264,C264),"000"))</f>
         <v>MT1-GM-CC-CB-002</v>
       </c>
     </row>
@@ -7797,7 +7797,7 @@
         <v>279</v>
       </c>
       <c r="G265" s="2" t="str">
-        <f aca="false">IF(OR(B265="",C265="",E265="",F265=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B265,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F265,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C265,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E265,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C265,C265),"000"))</f>
+        <f aca="false">IF(OR(B265="",C265="",E265="",F265=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B265,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F265,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C265,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E265,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C265,C265),"000"))</f>
         <v>MT1-GM-CC-CB-003</v>
       </c>
     </row>
@@ -7821,7 +7821,7 @@
         <v>279</v>
       </c>
       <c r="G266" s="2" t="str">
-        <f aca="false">IF(OR(B266="",C266="",E266="",F266=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B266,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F266,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C266,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E266,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C266,C266),"000"))</f>
+        <f aca="false">IF(OR(B266="",C266="",E266="",F266=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B266,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F266,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C266,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E266,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C266,C266),"000"))</f>
         <v>MT1-GM-TB-BW-003</v>
       </c>
     </row>
@@ -7845,7 +7845,7 @@
         <v>279</v>
       </c>
       <c r="G267" s="2" t="str">
-        <f aca="false">IF(OR(B267="",C267="",E267="",F267=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B267,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F267,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C267,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E267,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C267,C267),"000"))</f>
+        <f aca="false">IF(OR(B267="",C267="",E267="",F267=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B267,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F267,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C267,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E267,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C267,C267),"000"))</f>
         <v>MT1-GM-D1-TC-009</v>
       </c>
     </row>
@@ -7869,7 +7869,7 @@
         <v>279</v>
       </c>
       <c r="G268" s="2" t="str">
-        <f aca="false">IF(OR(B268="",C268="",E268="",F268=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B268,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F268,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C268,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E268,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C268,C268),"000"))</f>
+        <f aca="false">IF(OR(B268="",C268="",E268="",F268=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B268,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F268,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C268,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E268,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C268,C268),"000"))</f>
         <v>MT1-GM-CA-CB-003</v>
       </c>
     </row>
@@ -7893,7 +7893,7 @@
         <v>279</v>
       </c>
       <c r="G269" s="2" t="str">
-        <f aca="false">IF(OR(B269="",C269="",E269="",F269=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B269,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F269,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C269,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E269,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C269,C269),"000"))</f>
+        <f aca="false">IF(OR(B269="",C269="",E269="",F269=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B269,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F269,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C269,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E269,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C269,C269),"000"))</f>
         <v>MT1-GM-CA-CB-004</v>
       </c>
     </row>
@@ -7917,7 +7917,7 @@
         <v>279</v>
       </c>
       <c r="G270" s="2" t="str">
-        <f aca="false">IF(OR(B270="",C270="",E270="",F270=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B270,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F270,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C270,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E270,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C270,C270),"000"))</f>
+        <f aca="false">IF(OR(B270="",C270="",E270="",F270=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B270,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F270,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C270,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E270,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C270,C270),"000"))</f>
         <v>MT1-GM-CA-CB-005</v>
       </c>
     </row>
@@ -7941,7 +7941,7 @@
         <v>279</v>
       </c>
       <c r="G271" s="2" t="str">
-        <f aca="false">IF(OR(B271="",C271="",E271="",F271=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B271,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F271,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C271,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E271,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C271,C271),"000"))</f>
+        <f aca="false">IF(OR(B271="",C271="",E271="",F271=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B271,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F271,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C271,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E271,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C271,C271),"000"))</f>
         <v>MT1-GM-CA-CB-006</v>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
         <v>279</v>
       </c>
       <c r="G272" s="2" t="str">
-        <f aca="false">IF(OR(B272="",C272="",E272="",F272=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B272,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F272,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C272,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E272,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C272,C272),"000"))</f>
+        <f aca="false">IF(OR(B272="",C272="",E272="",F272=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B272,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F272,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C272,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E272,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C272,C272),"000"))</f>
         <v>MT1-GM-CA-CB-007</v>
       </c>
     </row>
@@ -7989,7 +7989,7 @@
         <v>279</v>
       </c>
       <c r="G273" s="2" t="str">
-        <f aca="false">IF(OR(B273="",C273="",E273="",F273=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B273,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F273,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C273,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E273,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C273,C273),"000"))</f>
+        <f aca="false">IF(OR(B273="",C273="",E273="",F273=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B273,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F273,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C273,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E273,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C273,C273),"000"))</f>
         <v>MT1-GM-CA-CB-008</v>
       </c>
     </row>
@@ -8013,1982 +8013,1982 @@
         <v>279</v>
       </c>
       <c r="G274" s="2" t="str">
-        <f aca="false">IF(OR(B274="",C274="",E274="",F274=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B274,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F274,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C274,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E274,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C274,C274),"000"))</f>
+        <f aca="false">IF(OR(B274="",C274="",E274="",F274=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B274,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F274,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C274,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E274,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C274,C274),"000"))</f>
         <v>MT1-GM-CA-CB-009</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G275" s="2" t="str">
-        <f aca="false">IF(OR(B275="",C275="",E275="",F275=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B275,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F275,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C275,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E275,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C275,C275),"000"))</f>
+        <f aca="false">IF(OR(B275="",C275="",E275="",F275=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B275,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F275,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C275,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E275,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C275,C275),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G276" s="2" t="str">
-        <f aca="false">IF(OR(B276="",C276="",E276="",F276=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B276,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F276,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C276,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E276,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C276,C276),"000"))</f>
+        <f aca="false">IF(OR(B276="",C276="",E276="",F276=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B276,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F276,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C276,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E276,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C276,C276),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G277" s="2" t="str">
-        <f aca="false">IF(OR(B277="",C277="",E277="",F277=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B277,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F277,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C277,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E277,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C277,C277),"000"))</f>
+        <f aca="false">IF(OR(B277="",C277="",E277="",F277=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B277,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F277,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C277,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E277,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C277,C277),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G278" s="2" t="str">
-        <f aca="false">IF(OR(B278="",C278="",E278="",F278=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B278,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F278,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C278,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E278,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C278,C278),"000"))</f>
+        <f aca="false">IF(OR(B278="",C278="",E278="",F278=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B278,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F278,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C278,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E278,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C278,C278),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G279" s="2" t="str">
-        <f aca="false">IF(OR(B279="",C279="",E279="",F279=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B279,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F279,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C279,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E279,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C279,C279),"000"))</f>
+        <f aca="false">IF(OR(B279="",C279="",E279="",F279=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B279,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F279,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C279,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E279,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C279,C279),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G280" s="2" t="str">
-        <f aca="false">IF(OR(B280="",C280="",E280="",F280=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B280,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F280,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C280,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E280,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C280,C280),"000"))</f>
+        <f aca="false">IF(OR(B280="",C280="",E280="",F280=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B280,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F280,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C280,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E280,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C280,C280),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G281" s="2" t="str">
-        <f aca="false">IF(OR(B281="",C281="",E281="",F281=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B281,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F281,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C281,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E281,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C281,C281),"000"))</f>
+        <f aca="false">IF(OR(B281="",C281="",E281="",F281=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B281,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F281,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C281,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E281,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C281,C281),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G282" s="2" t="str">
-        <f aca="false">IF(OR(B282="",C282="",E282="",F282=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B282,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F282,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C282,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E282,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C282,C282),"000"))</f>
+        <f aca="false">IF(OR(B282="",C282="",E282="",F282=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B282,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F282,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C282,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E282,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C282,C282),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G283" s="2" t="str">
-        <f aca="false">IF(OR(B283="",C283="",E283="",F283=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B283,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F283,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C283,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E283,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C283,C283),"000"))</f>
+        <f aca="false">IF(OR(B283="",C283="",E283="",F283=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B283,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F283,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C283,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E283,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C283,C283),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G284" s="2" t="str">
-        <f aca="false">IF(OR(B284="",C284="",E284="",F284=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B284,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F284,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C284,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E284,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C284,C284),"000"))</f>
+        <f aca="false">IF(OR(B284="",C284="",E284="",F284=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B284,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F284,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C284,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E284,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C284,C284),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G285" s="2" t="str">
-        <f aca="false">IF(OR(B285="",C285="",E285="",F285=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B285,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F285,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C285,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E285,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C285,C285),"000"))</f>
+        <f aca="false">IF(OR(B285="",C285="",E285="",F285=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B285,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F285,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C285,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E285,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C285,C285),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G286" s="2" t="str">
-        <f aca="false">IF(OR(B286="",C286="",E286="",F286=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B286,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F286,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C286,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E286,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C286,C286),"000"))</f>
+        <f aca="false">IF(OR(B286="",C286="",E286="",F286=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B286,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F286,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C286,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E286,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C286,C286),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G287" s="2" t="str">
-        <f aca="false">IF(OR(B287="",C287="",E287="",F287=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B287,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F287,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C287,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E287,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C287,C287),"000"))</f>
+        <f aca="false">IF(OR(B287="",C287="",E287="",F287=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B287,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F287,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C287,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E287,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C287,C287),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G288" s="2" t="str">
-        <f aca="false">IF(OR(B288="",C288="",E288="",F288=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B288,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F288,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C288,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E288,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C288,C288),"000"))</f>
+        <f aca="false">IF(OR(B288="",C288="",E288="",F288=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B288,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F288,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C288,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E288,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C288,C288),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G289" s="2" t="str">
-        <f aca="false">IF(OR(B289="",C289="",E289="",F289=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B289,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F289,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C289,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E289,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C289,C289),"000"))</f>
+        <f aca="false">IF(OR(B289="",C289="",E289="",F289=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B289,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F289,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C289,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E289,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C289,C289),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G290" s="2" t="str">
-        <f aca="false">IF(OR(B290="",C290="",E290="",F290=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B290,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F290,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C290,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E290,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C290,C290),"000"))</f>
+        <f aca="false">IF(OR(B290="",C290="",E290="",F290=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B290,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F290,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C290,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E290,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C290,C290),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G291" s="2" t="str">
-        <f aca="false">IF(OR(B291="",C291="",E291="",F291=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B291,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F291,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C291,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E291,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C291,C291),"000"))</f>
+        <f aca="false">IF(OR(B291="",C291="",E291="",F291=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B291,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F291,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C291,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E291,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C291,C291),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G292" s="2" t="str">
-        <f aca="false">IF(OR(B292="",C292="",E292="",F292=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B292,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F292,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C292,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E292,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C292,C292),"000"))</f>
+        <f aca="false">IF(OR(B292="",C292="",E292="",F292=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B292,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F292,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C292,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E292,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C292,C292),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G293" s="2" t="str">
-        <f aca="false">IF(OR(B293="",C293="",E293="",F293=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B293,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F293,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C293,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E293,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C293,C293),"000"))</f>
+        <f aca="false">IF(OR(B293="",C293="",E293="",F293=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B293,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F293,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C293,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E293,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C293,C293),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G294" s="2" t="str">
-        <f aca="false">IF(OR(B294="",C294="",E294="",F294=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B294,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F294,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C294,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E294,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C294,C294),"000"))</f>
+        <f aca="false">IF(OR(B294="",C294="",E294="",F294=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B294,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F294,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C294,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E294,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C294,C294),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G295" s="2" t="str">
-        <f aca="false">IF(OR(B295="",C295="",E295="",F295=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B295,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F295,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C295,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E295,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C295,C295),"000"))</f>
+        <f aca="false">IF(OR(B295="",C295="",E295="",F295=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B295,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F295,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C295,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E295,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C295,C295),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G296" s="2" t="str">
-        <f aca="false">IF(OR(B296="",C296="",E296="",F296=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B296,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F296,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C296,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E296,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C296,C296),"000"))</f>
+        <f aca="false">IF(OR(B296="",C296="",E296="",F296=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B296,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F296,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C296,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E296,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C296,C296),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G297" s="2" t="str">
-        <f aca="false">IF(OR(B297="",C297="",E297="",F297=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B297,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F297,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C297,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E297,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C297,C297),"000"))</f>
+        <f aca="false">IF(OR(B297="",C297="",E297="",F297=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B297,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F297,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C297,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E297,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C297,C297),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G298" s="2" t="str">
-        <f aca="false">IF(OR(B298="",C298="",E298="",F298=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B298,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F298,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C298,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E298,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C298,C298),"000"))</f>
+        <f aca="false">IF(OR(B298="",C298="",E298="",F298=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B298,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F298,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C298,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E298,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C298,C298),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G299" s="2" t="str">
-        <f aca="false">IF(OR(B299="",C299="",E299="",F299=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B299,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F299,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C299,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E299,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C299,C299),"000"))</f>
+        <f aca="false">IF(OR(B299="",C299="",E299="",F299=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B299,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F299,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C299,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E299,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C299,C299),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G300" s="2" t="str">
-        <f aca="false">IF(OR(B300="",C300="",E300="",F300=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B300,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F300,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C300,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E300,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C300,C300),"000"))</f>
+        <f aca="false">IF(OR(B300="",C300="",E300="",F300=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B300,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F300,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C300,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E300,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C300,C300),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G301" s="2" t="str">
-        <f aca="false">IF(OR(B301="",C301="",E301="",F301=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B301,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F301,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C301,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E301,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C301,C301),"000"))</f>
+        <f aca="false">IF(OR(B301="",C301="",E301="",F301=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B301,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F301,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C301,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E301,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C301,C301),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G302" s="2" t="str">
-        <f aca="false">IF(OR(B302="",C302="",E302="",F302=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B302,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F302,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C302,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E302,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C302,C302),"000"))</f>
+        <f aca="false">IF(OR(B302="",C302="",E302="",F302=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B302,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F302,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C302,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E302,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C302,C302),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G303" s="2" t="str">
-        <f aca="false">IF(OR(B303="",C303="",E303="",F303=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B303,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F303,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C303,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E303,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C303,C303),"000"))</f>
+        <f aca="false">IF(OR(B303="",C303="",E303="",F303=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B303,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F303,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C303,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E303,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C303,C303),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G304" s="2" t="str">
-        <f aca="false">IF(OR(B304="",C304="",E304="",F304=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B304,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F304,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C304,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E304,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C304,C304),"000"))</f>
+        <f aca="false">IF(OR(B304="",C304="",E304="",F304=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B304,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F304,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C304,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E304,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C304,C304),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G305" s="2" t="str">
-        <f aca="false">IF(OR(B305="",C305="",E305="",F305=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B305,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F305,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C305,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E305,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C305,C305),"000"))</f>
+        <f aca="false">IF(OR(B305="",C305="",E305="",F305=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B305,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F305,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C305,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E305,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C305,C305),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G306" s="2" t="str">
-        <f aca="false">IF(OR(B306="",C306="",E306="",F306=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B306,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F306,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C306,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E306,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C306,C306),"000"))</f>
+        <f aca="false">IF(OR(B306="",C306="",E306="",F306=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B306,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F306,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C306,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E306,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C306,C306),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G307" s="2" t="str">
-        <f aca="false">IF(OR(B307="",C307="",E307="",F307=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B307,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F307,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C307,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E307,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C307,C307),"000"))</f>
+        <f aca="false">IF(OR(B307="",C307="",E307="",F307=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B307,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F307,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C307,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E307,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C307,C307),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G308" s="2" t="str">
-        <f aca="false">IF(OR(B308="",C308="",E308="",F308=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B308,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F308,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C308,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E308,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C308,C308),"000"))</f>
+        <f aca="false">IF(OR(B308="",C308="",E308="",F308=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B308,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F308,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C308,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E308,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C308,C308),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G309" s="2" t="str">
-        <f aca="false">IF(OR(B309="",C309="",E309="",F309=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B309,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F309,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C309,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E309,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C309,C309),"000"))</f>
+        <f aca="false">IF(OR(B309="",C309="",E309="",F309=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B309,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F309,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C309,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E309,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C309,C309),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G310" s="2" t="str">
-        <f aca="false">IF(OR(B310="",C310="",E310="",F310=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B310,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F310,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C310,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E310,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C310,C310),"000"))</f>
+        <f aca="false">IF(OR(B310="",C310="",E310="",F310=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B310,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F310,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C310,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E310,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C310,C310),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G311" s="2" t="str">
-        <f aca="false">IF(OR(B311="",C311="",E311="",F311=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B311,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F311,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C311,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E311,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C311,C311),"000"))</f>
+        <f aca="false">IF(OR(B311="",C311="",E311="",F311=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B311,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F311,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C311,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E311,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C311,C311),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G312" s="2" t="str">
-        <f aca="false">IF(OR(B312="",C312="",E312="",F312=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B312,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F312,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C312,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E312,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C312,C312),"000"))</f>
+        <f aca="false">IF(OR(B312="",C312="",E312="",F312=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B312,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F312,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C312,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E312,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C312,C312),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G313" s="2" t="str">
-        <f aca="false">IF(OR(B313="",C313="",E313="",F313=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B313,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F313,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C313,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E313,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C313,C313),"000"))</f>
+        <f aca="false">IF(OR(B313="",C313="",E313="",F313=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B313,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F313,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C313,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E313,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C313,C313),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G314" s="2" t="str">
-        <f aca="false">IF(OR(B314="",C314="",E314="",F314=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B314,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F314,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C314,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E314,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C314,C314),"000"))</f>
+        <f aca="false">IF(OR(B314="",C314="",E314="",F314=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B314,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F314,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C314,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E314,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C314,C314),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G315" s="2" t="str">
-        <f aca="false">IF(OR(B315="",C315="",E315="",F315=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B315,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F315,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C315,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E315,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C315,C315),"000"))</f>
+        <f aca="false">IF(OR(B315="",C315="",E315="",F315=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B315,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F315,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C315,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E315,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C315,C315),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G316" s="2" t="str">
-        <f aca="false">IF(OR(B316="",C316="",E316="",F316=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B316,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F316,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C316,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E316,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C316,C316),"000"))</f>
+        <f aca="false">IF(OR(B316="",C316="",E316="",F316=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B316,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F316,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C316,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E316,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C316,C316),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G317" s="2" t="str">
-        <f aca="false">IF(OR(B317="",C317="",E317="",F317=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B317,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F317,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C317,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E317,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C317,C317),"000"))</f>
+        <f aca="false">IF(OR(B317="",C317="",E317="",F317=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B317,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F317,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C317,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E317,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C317,C317),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G318" s="2" t="str">
-        <f aca="false">IF(OR(B318="",C318="",E318="",F318=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B318,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F318,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C318,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E318,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C318,C318),"000"))</f>
+        <f aca="false">IF(OR(B318="",C318="",E318="",F318=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B318,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F318,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C318,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E318,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C318,C318),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G319" s="2" t="str">
-        <f aca="false">IF(OR(B319="",C319="",E319="",F319=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B319,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F319,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C319,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E319,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C319,C319),"000"))</f>
+        <f aca="false">IF(OR(B319="",C319="",E319="",F319=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B319,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F319,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C319,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E319,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C319,C319),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G320" s="2" t="str">
-        <f aca="false">IF(OR(B320="",C320="",E320="",F320=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B320,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F320,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C320,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E320,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C320,C320),"000"))</f>
+        <f aca="false">IF(OR(B320="",C320="",E320="",F320=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B320,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F320,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C320,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E320,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C320,C320),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G321" s="2" t="str">
-        <f aca="false">IF(OR(B321="",C321="",E321="",F321=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B321,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F321,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C321,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E321,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C321,C321),"000"))</f>
+        <f aca="false">IF(OR(B321="",C321="",E321="",F321=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B321,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F321,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C321,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E321,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C321,C321),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G322" s="2" t="str">
-        <f aca="false">IF(OR(B322="",C322="",E322="",F322=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B322,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F322,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C322,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E322,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C322,C322),"000"))</f>
+        <f aca="false">IF(OR(B322="",C322="",E322="",F322=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B322,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F322,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C322,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E322,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C322,C322),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G323" s="2" t="str">
-        <f aca="false">IF(OR(B323="",C323="",E323="",F323=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B323,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F323,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C323,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E323,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C323,C323),"000"))</f>
+        <f aca="false">IF(OR(B323="",C323="",E323="",F323=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B323,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F323,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C323,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E323,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C323,C323),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G324" s="2" t="str">
-        <f aca="false">IF(OR(B324="",C324="",E324="",F324=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B324,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F324,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C324,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E324,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C324,C324),"000"))</f>
+        <f aca="false">IF(OR(B324="",C324="",E324="",F324=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B324,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F324,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C324,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E324,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C324,C324),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G325" s="2" t="str">
-        <f aca="false">IF(OR(B325="",C325="",E325="",F325=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B325,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F325,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C325,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E325,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C325,C325),"000"))</f>
+        <f aca="false">IF(OR(B325="",C325="",E325="",F325=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B325,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F325,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C325,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E325,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C325,C325),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G326" s="2" t="str">
-        <f aca="false">IF(OR(B326="",C326="",E326="",F326=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B326,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F326,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C326,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E326,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C326,C326),"000"))</f>
+        <f aca="false">IF(OR(B326="",C326="",E326="",F326=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B326,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F326,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C326,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E326,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C326,C326),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G327" s="2" t="str">
-        <f aca="false">IF(OR(B327="",C327="",E327="",F327=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B327,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F327,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C327,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E327,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C327,C327),"000"))</f>
+        <f aca="false">IF(OR(B327="",C327="",E327="",F327=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B327,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F327,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C327,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E327,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C327,C327),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G328" s="2" t="str">
-        <f aca="false">IF(OR(B328="",C328="",E328="",F328=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B328,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F328,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C328,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E328,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C328,C328),"000"))</f>
+        <f aca="false">IF(OR(B328="",C328="",E328="",F328=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B328,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F328,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C328,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E328,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C328,C328),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G329" s="2" t="str">
-        <f aca="false">IF(OR(B329="",C329="",E329="",F329=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B329,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F329,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C329,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E329,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C329,C329),"000"))</f>
+        <f aca="false">IF(OR(B329="",C329="",E329="",F329=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B329,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F329,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C329,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E329,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C329,C329),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G330" s="2" t="str">
-        <f aca="false">IF(OR(B330="",C330="",E330="",F330=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B330,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F330,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C330,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E330,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C330,C330),"000"))</f>
+        <f aca="false">IF(OR(B330="",C330="",E330="",F330=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B330,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F330,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C330,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E330,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C330,C330),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G331" s="2" t="str">
-        <f aca="false">IF(OR(B331="",C331="",E331="",F331=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B331,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F331,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C331,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E331,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C331,C331),"000"))</f>
+        <f aca="false">IF(OR(B331="",C331="",E331="",F331=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B331,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F331,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C331,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E331,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C331,C331),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G332" s="2" t="str">
-        <f aca="false">IF(OR(B332="",C332="",E332="",F332=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B332,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F332,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C332,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E332,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C332,C332),"000"))</f>
+        <f aca="false">IF(OR(B332="",C332="",E332="",F332=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B332,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F332,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C332,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E332,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C332,C332),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G333" s="2" t="str">
-        <f aca="false">IF(OR(B333="",C333="",E333="",F333=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B333,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F333,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C333,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E333,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C333,C333),"000"))</f>
+        <f aca="false">IF(OR(B333="",C333="",E333="",F333=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B333,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F333,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C333,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E333,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C333,C333),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G334" s="2" t="str">
-        <f aca="false">IF(OR(B334="",C334="",E334="",F334=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B334,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F334,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C334,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E334,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C334,C334),"000"))</f>
+        <f aca="false">IF(OR(B334="",C334="",E334="",F334=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B334,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F334,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C334,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E334,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C334,C334),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G335" s="2" t="str">
-        <f aca="false">IF(OR(B335="",C335="",E335="",F335=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B335,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F335,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C335,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E335,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C335,C335),"000"))</f>
+        <f aca="false">IF(OR(B335="",C335="",E335="",F335=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B335,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F335,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C335,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E335,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C335,C335),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G336" s="2" t="str">
-        <f aca="false">IF(OR(B336="",C336="",E336="",F336=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B336,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F336,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C336,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E336,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C336,C336),"000"))</f>
+        <f aca="false">IF(OR(B336="",C336="",E336="",F336=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B336,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F336,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C336,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E336,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C336,C336),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G337" s="2" t="str">
-        <f aca="false">IF(OR(B337="",C337="",E337="",F337=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B337,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F337,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C337,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E337,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C337,C337),"000"))</f>
+        <f aca="false">IF(OR(B337="",C337="",E337="",F337=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B337,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F337,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C337,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E337,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C337,C337),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G338" s="2" t="str">
-        <f aca="false">IF(OR(B338="",C338="",E338="",F338=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B338,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F338,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C338,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E338,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C338,C338),"000"))</f>
+        <f aca="false">IF(OR(B338="",C338="",E338="",F338=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B338,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F338,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C338,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E338,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C338,C338),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G339" s="2" t="str">
-        <f aca="false">IF(OR(B339="",C339="",E339="",F339=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B339,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F339,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C339,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E339,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C339,C339),"000"))</f>
+        <f aca="false">IF(OR(B339="",C339="",E339="",F339=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B339,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F339,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C339,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E339,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C339,C339),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G340" s="2" t="str">
-        <f aca="false">IF(OR(B340="",C340="",E340="",F340=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B340,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F340,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C340,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E340,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C340,C340),"000"))</f>
+        <f aca="false">IF(OR(B340="",C340="",E340="",F340=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B340,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F340,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C340,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E340,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C340,C340),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G341" s="2" t="str">
-        <f aca="false">IF(OR(B341="",C341="",E341="",F341=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B341,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F341,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C341,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E341,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C341,C341),"000"))</f>
+        <f aca="false">IF(OR(B341="",C341="",E341="",F341=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B341,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F341,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C341,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E341,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C341,C341),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G342" s="2" t="str">
-        <f aca="false">IF(OR(B342="",C342="",E342="",F342=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B342,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F342,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C342,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E342,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C342,C342),"000"))</f>
+        <f aca="false">IF(OR(B342="",C342="",E342="",F342=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B342,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F342,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C342,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E342,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C342,C342),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G343" s="2" t="str">
-        <f aca="false">IF(OR(B343="",C343="",E343="",F343=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B343,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F343,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C343,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E343,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C343,C343),"000"))</f>
+        <f aca="false">IF(OR(B343="",C343="",E343="",F343=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B343,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F343,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C343,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E343,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C343,C343),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G344" s="2" t="str">
-        <f aca="false">IF(OR(B344="",C344="",E344="",F344=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B344,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F344,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C344,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E344,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C344,C344),"000"))</f>
+        <f aca="false">IF(OR(B344="",C344="",E344="",F344=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B344,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F344,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C344,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E344,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C344,C344),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G345" s="2" t="str">
-        <f aca="false">IF(OR(B345="",C345="",E345="",F345=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B345,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F345,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C345,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E345,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C345,C345),"000"))</f>
+        <f aca="false">IF(OR(B345="",C345="",E345="",F345=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B345,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F345,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C345,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E345,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C345,C345),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G346" s="2" t="str">
-        <f aca="false">IF(OR(B346="",C346="",E346="",F346=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B346,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F346,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C346,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E346,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C346,C346),"000"))</f>
+        <f aca="false">IF(OR(B346="",C346="",E346="",F346=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B346,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F346,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C346,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E346,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C346,C346),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G347" s="2" t="str">
-        <f aca="false">IF(OR(B347="",C347="",E347="",F347=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B347,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F347,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C347,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E347,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C347,C347),"000"))</f>
+        <f aca="false">IF(OR(B347="",C347="",E347="",F347=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B347,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F347,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C347,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E347,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C347,C347),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G348" s="2" t="str">
-        <f aca="false">IF(OR(B348="",C348="",E348="",F348=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B348,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F348,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C348,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E348,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C348,C348),"000"))</f>
+        <f aca="false">IF(OR(B348="",C348="",E348="",F348=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B348,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F348,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C348,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E348,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C348,C348),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G349" s="2" t="str">
-        <f aca="false">IF(OR(B349="",C349="",E349="",F349=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B349,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F349,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C349,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E349,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C349,C349),"000"))</f>
+        <f aca="false">IF(OR(B349="",C349="",E349="",F349=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B349,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F349,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C349,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E349,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C349,C349),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G350" s="2" t="str">
-        <f aca="false">IF(OR(B350="",C350="",E350="",F350=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B350,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F350,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C350,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E350,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C350,C350),"000"))</f>
+        <f aca="false">IF(OR(B350="",C350="",E350="",F350=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B350,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F350,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C350,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E350,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C350,C350),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G351" s="2" t="str">
-        <f aca="false">IF(OR(B351="",C351="",E351="",F351=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B351,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F351,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C351,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E351,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C351,C351),"000"))</f>
+        <f aca="false">IF(OR(B351="",C351="",E351="",F351=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B351,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F351,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C351,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E351,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C351,C351),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G352" s="2" t="str">
-        <f aca="false">IF(OR(B352="",C352="",E352="",F352=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B352,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F352,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C352,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E352,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C352,C352),"000"))</f>
+        <f aca="false">IF(OR(B352="",C352="",E352="",F352=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B352,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F352,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C352,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E352,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C352,C352),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G353" s="2" t="str">
-        <f aca="false">IF(OR(B353="",C353="",E353="",F353=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B353,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F353,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C353,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E353,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C353,C353),"000"))</f>
+        <f aca="false">IF(OR(B353="",C353="",E353="",F353=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B353,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F353,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C353,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E353,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C353,C353),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G354" s="2" t="str">
-        <f aca="false">IF(OR(B354="",C354="",E354="",F354=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B354,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F354,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C354,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E354,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C354,C354),"000"))</f>
+        <f aca="false">IF(OR(B354="",C354="",E354="",F354=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B354,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F354,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C354,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E354,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C354,C354),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G355" s="2" t="str">
-        <f aca="false">IF(OR(B355="",C355="",E355="",F355=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B355,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F355,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C355,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E355,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C355,C355),"000"))</f>
+        <f aca="false">IF(OR(B355="",C355="",E355="",F355=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B355,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F355,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C355,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E355,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C355,C355),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G356" s="2" t="str">
-        <f aca="false">IF(OR(B356="",C356="",E356="",F356=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B356,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F356,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C356,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E356,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C356,C356),"000"))</f>
+        <f aca="false">IF(OR(B356="",C356="",E356="",F356=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B356,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F356,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C356,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E356,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C356,C356),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G357" s="2" t="str">
-        <f aca="false">IF(OR(B357="",C357="",E357="",F357=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B357,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F357,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C357,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E357,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C357,C357),"000"))</f>
+        <f aca="false">IF(OR(B357="",C357="",E357="",F357=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B357,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F357,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C357,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E357,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C357,C357),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G358" s="2" t="str">
-        <f aca="false">IF(OR(B358="",C358="",E358="",F358=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B358,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F358,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C358,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E358,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C358,C358),"000"))</f>
+        <f aca="false">IF(OR(B358="",C358="",E358="",F358=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B358,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F358,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C358,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E358,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C358,C358),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G359" s="2" t="str">
-        <f aca="false">IF(OR(B359="",C359="",E359="",F359=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B359,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F359,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C359,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E359,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C359,C359),"000"))</f>
+        <f aca="false">IF(OR(B359="",C359="",E359="",F359=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B359,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F359,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C359,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E359,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C359,C359),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G360" s="2" t="str">
-        <f aca="false">IF(OR(B360="",C360="",E360="",F360=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B360,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F360,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C360,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E360,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C360,C360),"000"))</f>
+        <f aca="false">IF(OR(B360="",C360="",E360="",F360=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B360,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F360,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C360,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E360,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C360,C360),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G361" s="2" t="str">
-        <f aca="false">IF(OR(B361="",C361="",E361="",F361=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B361,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F361,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C361,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E361,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C361,C361),"000"))</f>
+        <f aca="false">IF(OR(B361="",C361="",E361="",F361=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B361,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F361,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C361,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E361,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C361,C361),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G362" s="2" t="str">
-        <f aca="false">IF(OR(B362="",C362="",E362="",F362=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B362,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F362,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C362,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E362,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C362,C362),"000"))</f>
+        <f aca="false">IF(OR(B362="",C362="",E362="",F362=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B362,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F362,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C362,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E362,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C362,C362),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G363" s="2" t="str">
-        <f aca="false">IF(OR(B363="",C363="",E363="",F363=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B363,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F363,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C363,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E363,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C363,C363),"000"))</f>
+        <f aca="false">IF(OR(B363="",C363="",E363="",F363=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B363,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F363,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C363,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E363,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C363,C363),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G364" s="2" t="str">
-        <f aca="false">IF(OR(B364="",C364="",E364="",F364=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B364,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F364,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C364,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E364,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C364,C364),"000"))</f>
+        <f aca="false">IF(OR(B364="",C364="",E364="",F364=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B364,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F364,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C364,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E364,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C364,C364),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G365" s="2" t="str">
-        <f aca="false">IF(OR(B365="",C365="",E365="",F365=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B365,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F365,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C365,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E365,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C365,C365),"000"))</f>
+        <f aca="false">IF(OR(B365="",C365="",E365="",F365=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B365,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F365,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C365,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E365,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C365,C365),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G366" s="2" t="str">
-        <f aca="false">IF(OR(B366="",C366="",E366="",F366=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B366,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F366,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C366,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E366,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C366,C366),"000"))</f>
+        <f aca="false">IF(OR(B366="",C366="",E366="",F366=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B366,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F366,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C366,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E366,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C366,C366),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G367" s="2" t="str">
-        <f aca="false">IF(OR(B367="",C367="",E367="",F367=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B367,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F367,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C367,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E367,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C367,C367),"000"))</f>
+        <f aca="false">IF(OR(B367="",C367="",E367="",F367=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B367,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F367,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C367,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E367,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C367,C367),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G368" s="2" t="str">
-        <f aca="false">IF(OR(B368="",C368="",E368="",F368=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B368,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F368,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C368,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E368,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C368,C368),"000"))</f>
+        <f aca="false">IF(OR(B368="",C368="",E368="",F368=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B368,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F368,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C368,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E368,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C368,C368),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G369" s="2" t="str">
-        <f aca="false">IF(OR(B369="",C369="",E369="",F369=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B369,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F369,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C369,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E369,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C369,C369),"000"))</f>
+        <f aca="false">IF(OR(B369="",C369="",E369="",F369=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B369,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F369,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C369,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E369,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C369,C369),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G370" s="2" t="str">
-        <f aca="false">IF(OR(B370="",C370="",E370="",F370=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B370,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F370,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C370,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E370,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C370,C370),"000"))</f>
+        <f aca="false">IF(OR(B370="",C370="",E370="",F370=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B370,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F370,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C370,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E370,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C370,C370),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G371" s="2" t="str">
-        <f aca="false">IF(OR(B371="",C371="",E371="",F371=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B371,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F371,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C371,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E371,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C371,C371),"000"))</f>
+        <f aca="false">IF(OR(B371="",C371="",E371="",F371=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B371,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F371,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C371,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E371,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C371,C371),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G372" s="2" t="str">
-        <f aca="false">IF(OR(B372="",C372="",E372="",F372=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B372,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F372,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C372,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E372,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C372,C372),"000"))</f>
+        <f aca="false">IF(OR(B372="",C372="",E372="",F372=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B372,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F372,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C372,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E372,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C372,C372),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G373" s="2" t="str">
-        <f aca="false">IF(OR(B373="",C373="",E373="",F373=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B373,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F373,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C373,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E373,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C373,C373),"000"))</f>
+        <f aca="false">IF(OR(B373="",C373="",E373="",F373=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B373,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F373,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C373,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E373,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C373,C373),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G374" s="2" t="str">
-        <f aca="false">IF(OR(B374="",C374="",E374="",F374=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B374,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F374,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C374,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E374,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C374,C374),"000"))</f>
+        <f aca="false">IF(OR(B374="",C374="",E374="",F374=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B374,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F374,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C374,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E374,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C374,C374),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G375" s="2" t="str">
-        <f aca="false">IF(OR(B375="",C375="",E375="",F375=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B375,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F375,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C375,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E375,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C375,C375),"000"))</f>
+        <f aca="false">IF(OR(B375="",C375="",E375="",F375=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B375,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F375,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C375,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E375,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C375,C375),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G376" s="2" t="str">
-        <f aca="false">IF(OR(B376="",C376="",E376="",F376=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B376,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F376,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C376,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E376,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C376,C376),"000"))</f>
+        <f aca="false">IF(OR(B376="",C376="",E376="",F376=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B376,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F376,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C376,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E376,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C376,C376),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G377" s="2" t="str">
-        <f aca="false">IF(OR(B377="",C377="",E377="",F377=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B377,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F377,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C377,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E377,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C377,C377),"000"))</f>
+        <f aca="false">IF(OR(B377="",C377="",E377="",F377=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B377,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F377,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C377,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E377,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C377,C377),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G378" s="2" t="str">
-        <f aca="false">IF(OR(B378="",C378="",E378="",F378=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B378,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F378,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C378,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E378,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C378,C378),"000"))</f>
+        <f aca="false">IF(OR(B378="",C378="",E378="",F378=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B378,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F378,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C378,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E378,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C378,C378),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G379" s="2" t="str">
-        <f aca="false">IF(OR(B379="",C379="",E379="",F379=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B379,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F379,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C379,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E379,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C379,C379),"000"))</f>
+        <f aca="false">IF(OR(B379="",C379="",E379="",F379=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B379,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F379,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C379,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E379,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C379,C379),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G380" s="2" t="str">
-        <f aca="false">IF(OR(B380="",C380="",E380="",F380=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B380,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F380,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C380,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E380,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C380,C380),"000"))</f>
+        <f aca="false">IF(OR(B380="",C380="",E380="",F380=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B380,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F380,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C380,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E380,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C380,C380),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G381" s="2" t="str">
-        <f aca="false">IF(OR(B381="",C381="",E381="",F381=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B381,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F381,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C381,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E381,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C381,C381),"000"))</f>
+        <f aca="false">IF(OR(B381="",C381="",E381="",F381=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B381,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F381,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C381,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E381,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C381,C381),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G382" s="2" t="str">
-        <f aca="false">IF(OR(B382="",C382="",E382="",F382=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B382,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F382,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C382,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E382,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C382,C382),"000"))</f>
+        <f aca="false">IF(OR(B382="",C382="",E382="",F382=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B382,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F382,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C382,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E382,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C382,C382),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G383" s="2" t="str">
-        <f aca="false">IF(OR(B383="",C383="",E383="",F383=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B383,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F383,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C383,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E383,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C383,C383),"000"))</f>
+        <f aca="false">IF(OR(B383="",C383="",E383="",F383=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B383,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F383,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C383,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E383,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C383,C383),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G384" s="2" t="str">
-        <f aca="false">IF(OR(B384="",C384="",E384="",F384=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B384,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F384,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C384,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E384,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C384,C384),"000"))</f>
+        <f aca="false">IF(OR(B384="",C384="",E384="",F384=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B384,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F384,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C384,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E384,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C384,C384),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G385" s="2" t="str">
-        <f aca="false">IF(OR(B385="",C385="",E385="",F385=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B385,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F385,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C385,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E385,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C385,C385),"000"))</f>
+        <f aca="false">IF(OR(B385="",C385="",E385="",F385=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B385,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F385,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C385,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E385,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C385,C385),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G386" s="2" t="str">
-        <f aca="false">IF(OR(B386="",C386="",E386="",F386=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B386,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F386,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C386,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E386,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C386,C386),"000"))</f>
+        <f aca="false">IF(OR(B386="",C386="",E386="",F386=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B386,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F386,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C386,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E386,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C386,C386),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G387" s="2" t="str">
-        <f aca="false">IF(OR(B387="",C387="",E387="",F387=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B387,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F387,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C387,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E387,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C387,C387),"000"))</f>
+        <f aca="false">IF(OR(B387="",C387="",E387="",F387=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B387,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F387,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C387,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E387,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C387,C387),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G388" s="2" t="str">
-        <f aca="false">IF(OR(B388="",C388="",E388="",F388=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B388,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F388,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C388,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E388,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C388,C388),"000"))</f>
+        <f aca="false">IF(OR(B388="",C388="",E388="",F388=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B388,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F388,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C388,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E388,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C388,C388),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G389" s="2" t="str">
-        <f aca="false">IF(OR(B389="",C389="",E389="",F389=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B389,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F389,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C389,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E389,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C389,C389),"000"))</f>
+        <f aca="false">IF(OR(B389="",C389="",E389="",F389=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B389,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F389,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C389,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E389,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C389,C389),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G390" s="2" t="str">
-        <f aca="false">IF(OR(B390="",C390="",E390="",F390=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B390,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F390,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C390,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E390,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C390,C390),"000"))</f>
+        <f aca="false">IF(OR(B390="",C390="",E390="",F390=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B390,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F390,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C390,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E390,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C390,C390),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="391" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G391" s="2" t="str">
-        <f aca="false">IF(OR(B391="",C391="",E391="",F391=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B391,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F391,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C391,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E391,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C391,C391),"000"))</f>
+        <f aca="false">IF(OR(B391="",C391="",E391="",F391=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B391,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F391,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C391,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E391,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C391,C391),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G392" s="2" t="str">
-        <f aca="false">IF(OR(B392="",C392="",E392="",F392=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B392,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F392,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C392,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E392,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C392,C392),"000"))</f>
+        <f aca="false">IF(OR(B392="",C392="",E392="",F392=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B392,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F392,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C392,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E392,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C392,C392),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G393" s="2" t="str">
-        <f aca="false">IF(OR(B393="",C393="",E393="",F393=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B393,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F393,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C393,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E393,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C393,C393),"000"))</f>
+        <f aca="false">IF(OR(B393="",C393="",E393="",F393=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B393,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F393,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C393,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E393,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C393,C393),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G394" s="2" t="str">
-        <f aca="false">IF(OR(B394="",C394="",E394="",F394=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B394,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F394,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C394,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E394,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C394,C394),"000"))</f>
+        <f aca="false">IF(OR(B394="",C394="",E394="",F394=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B394,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F394,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C394,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E394,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C394,C394),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G395" s="2" t="str">
-        <f aca="false">IF(OR(B395="",C395="",E395="",F395=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B395,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F395,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C395,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E395,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C395,C395),"000"))</f>
+        <f aca="false">IF(OR(B395="",C395="",E395="",F395=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B395,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F395,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C395,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E395,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C395,C395),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G396" s="2" t="str">
-        <f aca="false">IF(OR(B396="",C396="",E396="",F396=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B396,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F396,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C396,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E396,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C396,C396),"000"))</f>
+        <f aca="false">IF(OR(B396="",C396="",E396="",F396=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B396,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F396,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C396,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E396,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C396,C396),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G397" s="2" t="str">
-        <f aca="false">IF(OR(B397="",C397="",E397="",F397=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B397,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F397,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C397,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E397,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C397,C397),"000"))</f>
+        <f aca="false">IF(OR(B397="",C397="",E397="",F397=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B397,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F397,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C397,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E397,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C397,C397),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G398" s="2" t="str">
-        <f aca="false">IF(OR(B398="",C398="",E398="",F398=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B398,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F398,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C398,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E398,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C398,C398),"000"))</f>
+        <f aca="false">IF(OR(B398="",C398="",E398="",F398=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B398,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F398,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C398,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E398,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C398,C398),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G399" s="2" t="str">
-        <f aca="false">IF(OR(B399="",C399="",E399="",F399=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B399,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F399,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C399,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E399,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C399,C399),"000"))</f>
+        <f aca="false">IF(OR(B399="",C399="",E399="",F399=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B399,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F399,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C399,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E399,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C399,C399),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G400" s="2" t="str">
-        <f aca="false">IF(OR(B400="",C400="",E400="",F400=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B400,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F400,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C400,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E400,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C400,C400),"000"))</f>
+        <f aca="false">IF(OR(B400="",C400="",E400="",F400=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B400,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F400,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C400,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E400,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C400,C400),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G401" s="2" t="str">
-        <f aca="false">IF(OR(B401="",C401="",E401="",F401=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B401,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F401,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C401,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E401,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C401,C401),"000"))</f>
+        <f aca="false">IF(OR(B401="",C401="",E401="",F401=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B401,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F401,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C401,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E401,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C401,C401),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G402" s="2" t="str">
-        <f aca="false">IF(OR(B402="",C402="",E402="",F402=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B402,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F402,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C402,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E402,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C402,C402),"000"))</f>
+        <f aca="false">IF(OR(B402="",C402="",E402="",F402=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B402,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F402,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C402,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E402,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C402,C402),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G403" s="2" t="str">
-        <f aca="false">IF(OR(B403="",C403="",E403="",F403=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B403,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F403,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C403,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E403,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C403,C403),"000"))</f>
+        <f aca="false">IF(OR(B403="",C403="",E403="",F403=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B403,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F403,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C403,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E403,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C403,C403),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G404" s="2" t="str">
-        <f aca="false">IF(OR(B404="",C404="",E404="",F404=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B404,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F404,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C404,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E404,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C404,C404),"000"))</f>
+        <f aca="false">IF(OR(B404="",C404="",E404="",F404=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B404,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F404,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C404,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E404,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C404,C404),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G405" s="2" t="str">
-        <f aca="false">IF(OR(B405="",C405="",E405="",F405=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B405,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F405,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C405,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E405,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C405,C405),"000"))</f>
+        <f aca="false">IF(OR(B405="",C405="",E405="",F405=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B405,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F405,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C405,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E405,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C405,C405),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="406" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G406" s="2" t="str">
-        <f aca="false">IF(OR(B406="",C406="",E406="",F406=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B406,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F406,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C406,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E406,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C406,C406),"000"))</f>
+        <f aca="false">IF(OR(B406="",C406="",E406="",F406=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B406,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F406,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C406,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E406,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C406,C406),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G407" s="2" t="str">
-        <f aca="false">IF(OR(B407="",C407="",E407="",F407=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B407,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F407,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C407,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E407,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C407,C407),"000"))</f>
+        <f aca="false">IF(OR(B407="",C407="",E407="",F407=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B407,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F407,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C407,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E407,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C407,C407),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G408" s="2" t="str">
-        <f aca="false">IF(OR(B408="",C408="",E408="",F408=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B408,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F408,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C408,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E408,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C408,C408),"000"))</f>
+        <f aca="false">IF(OR(B408="",C408="",E408="",F408=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B408,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F408,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C408,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E408,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C408,C408),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G409" s="2" t="str">
-        <f aca="false">IF(OR(B409="",C409="",E409="",F409=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B409,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F409,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C409,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E409,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C409,C409),"000"))</f>
+        <f aca="false">IF(OR(B409="",C409="",E409="",F409=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B409,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F409,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C409,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E409,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C409,C409),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G410" s="2" t="str">
-        <f aca="false">IF(OR(B410="",C410="",E410="",F410=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B410,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F410,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C410,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E410,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C410,C410),"000"))</f>
+        <f aca="false">IF(OR(B410="",C410="",E410="",F410=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B410,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F410,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C410,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E410,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C410,C410),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G411" s="2" t="str">
-        <f aca="false">IF(OR(B411="",C411="",E411="",F411=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B411,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F411,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C411,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E411,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C411,C411),"000"))</f>
+        <f aca="false">IF(OR(B411="",C411="",E411="",F411=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B411,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F411,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C411,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E411,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C411,C411),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G412" s="2" t="str">
-        <f aca="false">IF(OR(B412="",C412="",E412="",F412=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B412,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F412,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C412,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E412,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C412,C412),"000"))</f>
+        <f aca="false">IF(OR(B412="",C412="",E412="",F412=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B412,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F412,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C412,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E412,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C412,C412),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G413" s="2" t="str">
-        <f aca="false">IF(OR(B413="",C413="",E413="",F413=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B413,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F413,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C413,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E413,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C413,C413),"000"))</f>
+        <f aca="false">IF(OR(B413="",C413="",E413="",F413=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B413,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F413,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C413,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E413,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C413,C413),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G414" s="2" t="str">
-        <f aca="false">IF(OR(B414="",C414="",E414="",F414=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B414,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F414,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C414,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E414,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C414,C414),"000"))</f>
+        <f aca="false">IF(OR(B414="",C414="",E414="",F414=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B414,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F414,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C414,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E414,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C414,C414),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G415" s="2" t="str">
-        <f aca="false">IF(OR(B415="",C415="",E415="",F415=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B415,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F415,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C415,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E415,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C415,C415),"000"))</f>
+        <f aca="false">IF(OR(B415="",C415="",E415="",F415=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B415,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F415,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C415,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E415,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C415,C415),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G416" s="2" t="str">
-        <f aca="false">IF(OR(B416="",C416="",E416="",F416=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B416,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F416,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C416,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E416,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C416,C416),"000"))</f>
+        <f aca="false">IF(OR(B416="",C416="",E416="",F416=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B416,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F416,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C416,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E416,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C416,C416),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G417" s="2" t="str">
-        <f aca="false">IF(OR(B417="",C417="",E417="",F417=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B417,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F417,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C417,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E417,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C417,C417),"000"))</f>
+        <f aca="false">IF(OR(B417="",C417="",E417="",F417=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B417,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F417,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C417,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E417,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C417,C417),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G418" s="2" t="str">
-        <f aca="false">IF(OR(B418="",C418="",E418="",F418=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B418,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F418,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C418,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E418,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C418,C418),"000"))</f>
+        <f aca="false">IF(OR(B418="",C418="",E418="",F418=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B418,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F418,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C418,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E418,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C418,C418),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G419" s="2" t="str">
-        <f aca="false">IF(OR(B419="",C419="",E419="",F419=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B419,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F419,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C419,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E419,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C419,C419),"000"))</f>
+        <f aca="false">IF(OR(B419="",C419="",E419="",F419=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B419,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F419,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C419,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E419,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C419,C419),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G420" s="2" t="str">
-        <f aca="false">IF(OR(B420="",C420="",E420="",F420=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B420,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F420,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C420,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E420,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C420,C420),"000"))</f>
+        <f aca="false">IF(OR(B420="",C420="",E420="",F420=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B420,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F420,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C420,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E420,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C420,C420),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G421" s="2" t="str">
-        <f aca="false">IF(OR(B421="",C421="",E421="",F421=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B421,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F421,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C421,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E421,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C421,C421),"000"))</f>
+        <f aca="false">IF(OR(B421="",C421="",E421="",F421=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B421,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F421,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C421,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E421,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C421,C421),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="422" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G422" s="2" t="str">
-        <f aca="false">IF(OR(B422="",C422="",E422="",F422=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B422,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F422,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C422,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E422,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C422,C422),"000"))</f>
+        <f aca="false">IF(OR(B422="",C422="",E422="",F422=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B422,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F422,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C422,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E422,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C422,C422),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G423" s="2" t="str">
-        <f aca="false">IF(OR(B423="",C423="",E423="",F423=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B423,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F423,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C423,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E423,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C423,C423),"000"))</f>
+        <f aca="false">IF(OR(B423="",C423="",E423="",F423=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B423,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F423,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C423,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E423,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C423,C423),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G424" s="2" t="str">
-        <f aca="false">IF(OR(B424="",C424="",E424="",F424=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B424,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F424,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C424,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E424,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C424,C424),"000"))</f>
+        <f aca="false">IF(OR(B424="",C424="",E424="",F424=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B424,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F424,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C424,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E424,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C424,C424),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G425" s="2" t="str">
-        <f aca="false">IF(OR(B425="",C425="",E425="",F425=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B425,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F425,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C425,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E425,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C425,C425),"000"))</f>
+        <f aca="false">IF(OR(B425="",C425="",E425="",F425=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B425,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F425,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C425,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E425,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C425,C425),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G426" s="2" t="str">
-        <f aca="false">IF(OR(B426="",C426="",E426="",F426=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B426,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F426,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C426,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E426,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C426,C426),"000"))</f>
+        <f aca="false">IF(OR(B426="",C426="",E426="",F426=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B426,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F426,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C426,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E426,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C426,C426),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G427" s="2" t="str">
-        <f aca="false">IF(OR(B427="",C427="",E427="",F427=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B427,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F427,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C427,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E427,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C427,C427),"000"))</f>
+        <f aca="false">IF(OR(B427="",C427="",E427="",F427=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B427,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F427,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C427,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E427,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C427,C427),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G428" s="2" t="str">
-        <f aca="false">IF(OR(B428="",C428="",E428="",F428=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B428,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F428,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C428,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E428,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C428,C428),"000"))</f>
+        <f aca="false">IF(OR(B428="",C428="",E428="",F428=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B428,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F428,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C428,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E428,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C428,C428),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G429" s="2" t="str">
-        <f aca="false">IF(OR(B429="",C429="",E429="",F429=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B429,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F429,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C429,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E429,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C429,C429),"000"))</f>
+        <f aca="false">IF(OR(B429="",C429="",E429="",F429=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B429,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F429,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C429,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E429,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C429,C429),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G430" s="2" t="str">
-        <f aca="false">IF(OR(B430="",C430="",E430="",F430=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B430,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F430,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C430,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E430,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C430,C430),"000"))</f>
+        <f aca="false">IF(OR(B430="",C430="",E430="",F430=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B430,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F430,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C430,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E430,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C430,C430),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G431" s="2" t="str">
-        <f aca="false">IF(OR(B431="",C431="",E431="",F431=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B431,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F431,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C431,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E431,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C431,C431),"000"))</f>
+        <f aca="false">IF(OR(B431="",C431="",E431="",F431=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B431,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F431,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C431,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E431,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C431,C431),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G432" s="2" t="str">
-        <f aca="false">IF(OR(B432="",C432="",E432="",F432=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B432,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F432,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C432,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E432,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C432,C432),"000"))</f>
+        <f aca="false">IF(OR(B432="",C432="",E432="",F432=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B432,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F432,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C432,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E432,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C432,C432),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G433" s="2" t="str">
-        <f aca="false">IF(OR(B433="",C433="",E433="",F433=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B433,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F433,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C433,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E433,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C433,C433),"000"))</f>
+        <f aca="false">IF(OR(B433="",C433="",E433="",F433=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B433,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F433,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C433,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E433,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C433,C433),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G434" s="2" t="str">
-        <f aca="false">IF(OR(B434="",C434="",E434="",F434=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B434,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F434,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C434,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E434,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C434,C434),"000"))</f>
+        <f aca="false">IF(OR(B434="",C434="",E434="",F434=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B434,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F434,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C434,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E434,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C434,C434),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G435" s="2" t="str">
-        <f aca="false">IF(OR(B435="",C435="",E435="",F435=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B435,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F435,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C435,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E435,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C435,C435),"000"))</f>
+        <f aca="false">IF(OR(B435="",C435="",E435="",F435=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B435,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F435,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C435,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E435,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C435,C435),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G436" s="2" t="str">
-        <f aca="false">IF(OR(B436="",C436="",E436="",F436=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B436,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F436,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C436,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E436,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C436,C436),"000"))</f>
+        <f aca="false">IF(OR(B436="",C436="",E436="",F436=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B436,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F436,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C436,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E436,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C436,C436),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G437" s="2" t="str">
-        <f aca="false">IF(OR(B437="",C437="",E437="",F437=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B437,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F437,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C437,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E437,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C437,C437),"000"))</f>
+        <f aca="false">IF(OR(B437="",C437="",E437="",F437=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B437,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F437,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C437,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E437,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C437,C437),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G438" s="2" t="str">
-        <f aca="false">IF(OR(B438="",C438="",E438="",F438=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B438,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F438,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C438,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E438,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C438,C438),"000"))</f>
+        <f aca="false">IF(OR(B438="",C438="",E438="",F438=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B438,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F438,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C438,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E438,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C438,C438),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G439" s="2" t="str">
-        <f aca="false">IF(OR(B439="",C439="",E439="",F439=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B439,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F439,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C439,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E439,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C439,C439),"000"))</f>
+        <f aca="false">IF(OR(B439="",C439="",E439="",F439=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B439,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F439,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C439,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E439,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C439,C439),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G440" s="2" t="str">
-        <f aca="false">IF(OR(B440="",C440="",E440="",F440=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B440,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F440,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C440,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E440,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C440,C440),"000"))</f>
+        <f aca="false">IF(OR(B440="",C440="",E440="",F440=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B440,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F440,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C440,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E440,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C440,C440),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G441" s="2" t="str">
-        <f aca="false">IF(OR(B441="",C441="",E441="",F441=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B441,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F441,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C441,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E441,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C441,C441),"000"))</f>
+        <f aca="false">IF(OR(B441="",C441="",E441="",F441=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B441,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F441,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C441,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E441,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C441,C441),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G442" s="2" t="str">
-        <f aca="false">IF(OR(B442="",C442="",E442="",F442=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B442,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F442,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C442,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E442,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C442,C442),"000"))</f>
+        <f aca="false">IF(OR(B442="",C442="",E442="",F442=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B442,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F442,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C442,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E442,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C442,C442),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G443" s="2" t="str">
-        <f aca="false">IF(OR(B443="",C443="",E443="",F443=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B443,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F443,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C443,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E443,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C443,C443),"000"))</f>
+        <f aca="false">IF(OR(B443="",C443="",E443="",F443=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B443,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F443,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C443,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E443,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C443,C443),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G444" s="2" t="str">
-        <f aca="false">IF(OR(B444="",C444="",E444="",F444=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B444,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F444,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C444,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E444,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C444,C444),"000"))</f>
+        <f aca="false">IF(OR(B444="",C444="",E444="",F444=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B444,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F444,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C444,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E444,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C444,C444),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G445" s="2" t="str">
-        <f aca="false">IF(OR(B445="",C445="",E445="",F445=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B445,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F445,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C445,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E445,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C445,C445),"000"))</f>
+        <f aca="false">IF(OR(B445="",C445="",E445="",F445=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B445,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F445,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C445,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E445,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C445,C445),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G446" s="2" t="str">
-        <f aca="false">IF(OR(B446="",C446="",E446="",F446=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B446,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F446,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C446,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E446,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C446,C446),"000"))</f>
+        <f aca="false">IF(OR(B446="",C446="",E446="",F446=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B446,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F446,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C446,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E446,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C446,C446),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G447" s="2" t="str">
-        <f aca="false">IF(OR(B447="",C447="",E447="",F447=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B447,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F447,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C447,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E447,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C447,C447),"000"))</f>
+        <f aca="false">IF(OR(B447="",C447="",E447="",F447=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B447,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F447,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C447,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E447,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C447,C447),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G448" s="2" t="str">
-        <f aca="false">IF(OR(B448="",C448="",E448="",F448=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B448,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F448,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C448,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E448,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C448,C448),"000"))</f>
+        <f aca="false">IF(OR(B448="",C448="",E448="",F448=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B448,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F448,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C448,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E448,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C448,C448),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G449" s="2" t="str">
-        <f aca="false">IF(OR(B449="",C449="",E449="",F449=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B449,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F449,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C449,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E449,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C449,C449),"000"))</f>
+        <f aca="false">IF(OR(B449="",C449="",E449="",F449=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B449,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F449,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C449,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E449,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C449,C449),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G450" s="2" t="str">
-        <f aca="false">IF(OR(B450="",C450="",E450="",F450=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B450,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F450,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C450,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E450,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C450,C450),"000"))</f>
+        <f aca="false">IF(OR(B450="",C450="",E450="",F450=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B450,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F450,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C450,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E450,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C450,C450),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G451" s="2" t="str">
-        <f aca="false">IF(OR(B451="",C451="",E451="",F451=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B451,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F451,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C451,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E451,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C451,C451),"000"))</f>
+        <f aca="false">IF(OR(B451="",C451="",E451="",F451=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B451,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F451,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C451,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E451,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C451,C451),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G452" s="2" t="str">
-        <f aca="false">IF(OR(B452="",C452="",E452="",F452=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B452,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F452,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C452,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E452,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C452,C452),"000"))</f>
+        <f aca="false">IF(OR(B452="",C452="",E452="",F452=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B452,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F452,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C452,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E452,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C452,C452),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G453" s="2" t="str">
-        <f aca="false">IF(OR(B453="",C453="",E453="",F453=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B453,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F453,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C453,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E453,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C453,C453),"000"))</f>
+        <f aca="false">IF(OR(B453="",C453="",E453="",F453=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B453,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F453,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C453,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E453,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C453,C453),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G454" s="2" t="str">
-        <f aca="false">IF(OR(B454="",C454="",E454="",F454=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B454,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F454,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C454,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E454,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C454,C454),"000"))</f>
+        <f aca="false">IF(OR(B454="",C454="",E454="",F454=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B454,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F454,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C454,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E454,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C454,C454),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G455" s="2" t="str">
-        <f aca="false">IF(OR(B455="",C455="",E455="",F455=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B455,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F455,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C455,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E455,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C455,C455),"000"))</f>
+        <f aca="false">IF(OR(B455="",C455="",E455="",F455=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B455,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F455,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C455,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E455,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C455,C455),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G456" s="2" t="str">
-        <f aca="false">IF(OR(B456="",C456="",E456="",F456=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B456,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F456,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C456,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E456,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C456,C456),"000"))</f>
+        <f aca="false">IF(OR(B456="",C456="",E456="",F456=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B456,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F456,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C456,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E456,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C456,C456),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G457" s="2" t="str">
-        <f aca="false">IF(OR(B457="",C457="",E457="",F457=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B457,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F457,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C457,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E457,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C457,C457),"000"))</f>
+        <f aca="false">IF(OR(B457="",C457="",E457="",F457=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B457,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F457,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C457,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E457,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C457,C457),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G458" s="2" t="str">
-        <f aca="false">IF(OR(B458="",C458="",E458="",F458=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B458,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F458,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C458,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E458,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C458,C458),"000"))</f>
+        <f aca="false">IF(OR(B458="",C458="",E458="",F458=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B458,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F458,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C458,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E458,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C458,C458),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G459" s="2" t="str">
-        <f aca="false">IF(OR(B459="",C459="",E459="",F459=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B459,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F459,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C459,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E459,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C459,C459),"000"))</f>
+        <f aca="false">IF(OR(B459="",C459="",E459="",F459=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B459,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F459,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C459,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E459,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C459,C459),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G460" s="2" t="str">
-        <f aca="false">IF(OR(B460="",C460="",E460="",F460=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B460,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F460,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C460,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E460,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C460,C460),"000"))</f>
+        <f aca="false">IF(OR(B460="",C460="",E460="",F460=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B460,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F460,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C460,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E460,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C460,C460),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G461" s="2" t="str">
-        <f aca="false">IF(OR(B461="",C461="",E461="",F461=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B461,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F461,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C461,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E461,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C461,C461),"000"))</f>
+        <f aca="false">IF(OR(B461="",C461="",E461="",F461=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B461,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F461,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C461,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E461,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C461,C461),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G462" s="2" t="str">
-        <f aca="false">IF(OR(B462="",C462="",E462="",F462=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B462,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F462,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C462,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E462,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C462,C462),"000"))</f>
+        <f aca="false">IF(OR(B462="",C462="",E462="",F462=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B462,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F462,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C462,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E462,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C462,C462),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G463" s="2" t="str">
-        <f aca="false">IF(OR(B463="",C463="",E463="",F463=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B463,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F463,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C463,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E463,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C463,C463),"000"))</f>
+        <f aca="false">IF(OR(B463="",C463="",E463="",F463=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B463,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F463,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C463,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E463,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C463,C463),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G464" s="2" t="str">
-        <f aca="false">IF(OR(B464="",C464="",E464="",F464=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B464,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F464,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C464,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E464,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C464,C464),"000"))</f>
+        <f aca="false">IF(OR(B464="",C464="",E464="",F464=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B464,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F464,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C464,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E464,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C464,C464),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G465" s="2" t="str">
-        <f aca="false">IF(OR(B465="",C465="",E465="",F465=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B465,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F465,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C465,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E465,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C465,C465),"000"))</f>
+        <f aca="false">IF(OR(B465="",C465="",E465="",F465=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B465,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F465,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C465,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E465,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C465,C465),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G466" s="2" t="str">
-        <f aca="false">IF(OR(B466="",C466="",E466="",F466=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B466,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F466,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C466,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E466,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C466,C466),"000"))</f>
+        <f aca="false">IF(OR(B466="",C466="",E466="",F466=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B466,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F466,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C466,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E466,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C466,C466),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G467" s="2" t="str">
-        <f aca="false">IF(OR(B467="",C467="",E467="",F467=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B467,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F467,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C467,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E467,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C467,C467),"000"))</f>
+        <f aca="false">IF(OR(B467="",C467="",E467="",F467=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B467,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F467,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C467,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E467,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C467,C467),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G468" s="2" t="str">
-        <f aca="false">IF(OR(B468="",C468="",E468="",F468=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B468,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F468,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C468,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E468,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C468,C468),"000"))</f>
+        <f aca="false">IF(OR(B468="",C468="",E468="",F468=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B468,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F468,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C468,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E468,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C468,C468),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G469" s="2" t="str">
-        <f aca="false">IF(OR(B469="",C469="",E469="",F469=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B469,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F469,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C469,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E469,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C469,C469),"000"))</f>
+        <f aca="false">IF(OR(B469="",C469="",E469="",F469=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B469,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F469,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C469,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E469,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C469,C469),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G470" s="2" t="str">
-        <f aca="false">IF(OR(B470="",C470="",E470="",F470=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B470,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F470,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C470,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E470,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C470,C470),"000"))</f>
+        <f aca="false">IF(OR(B470="",C470="",E470="",F470=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B470,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F470,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C470,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E470,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C470,C470),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G471" s="2" t="str">
-        <f aca="false">IF(OR(B471="",C471="",E471="",F471=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B471,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F471,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C471,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E471,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C471,C471),"000"))</f>
+        <f aca="false">IF(OR(B471="",C471="",E471="",F471=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B471,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F471,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C471,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E471,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C471,C471),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G472" s="2" t="str">
-        <f aca="false">IF(OR(B472="",C472="",E472="",F472=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B472,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F472,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C472,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E472,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C472,C472),"000"))</f>
+        <f aca="false">IF(OR(B472="",C472="",E472="",F472=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B472,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F472,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C472,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E472,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C472,C472),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G473" s="2" t="str">
-        <f aca="false">IF(OR(B473="",C473="",E473="",F473=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B473,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F473,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C473,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E473,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C473,C473),"000"))</f>
+        <f aca="false">IF(OR(B473="",C473="",E473="",F473=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B473,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F473,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C473,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E473,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C473,C473),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G474" s="2" t="str">
-        <f aca="false">IF(OR(B474="",C474="",E474="",F474=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B474,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F474,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C474,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E474,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C474,C474),"000"))</f>
+        <f aca="false">IF(OR(B474="",C474="",E474="",F474=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B474,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F474,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C474,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E474,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C474,C474),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G475" s="2" t="str">
-        <f aca="false">IF(OR(B475="",C475="",E475="",F475=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B475,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F475,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C475,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E475,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C475,C475),"000"))</f>
+        <f aca="false">IF(OR(B475="",C475="",E475="",F475=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B475,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F475,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C475,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E475,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C475,C475),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G476" s="2" t="str">
-        <f aca="false">IF(OR(B476="",C476="",E476="",F476=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B476,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F476,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C476,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E476,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C476,C476),"000"))</f>
+        <f aca="false">IF(OR(B476="",C476="",E476="",F476=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B476,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F476,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C476,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E476,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C476,C476),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G477" s="2" t="str">
-        <f aca="false">IF(OR(B477="",C477="",E477="",F477=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B477,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F477,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C477,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E477,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C477,C477),"000"))</f>
+        <f aca="false">IF(OR(B477="",C477="",E477="",F477=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B477,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F477,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C477,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E477,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C477,C477),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G478" s="2" t="str">
-        <f aca="false">IF(OR(B478="",C478="",E478="",F478=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B478,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F478,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C478,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E478,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C478,C478),"000"))</f>
+        <f aca="false">IF(OR(B478="",C478="",E478="",F478=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B478,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F478,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C478,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E478,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C478,C478),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G479" s="2" t="str">
-        <f aca="false">IF(OR(B479="",C479="",E479="",F479=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B479,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F479,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C479,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E479,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C479,C479),"000"))</f>
+        <f aca="false">IF(OR(B479="",C479="",E479="",F479=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B479,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F479,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C479,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E479,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C479,C479),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G480" s="2" t="str">
-        <f aca="false">IF(OR(B480="",C480="",E480="",F480=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B480,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F480,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C480,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E480,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C480,C480),"000"))</f>
+        <f aca="false">IF(OR(B480="",C480="",E480="",F480=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B480,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F480,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C480,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E480,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C480,C480),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G481" s="2" t="str">
-        <f aca="false">IF(OR(B481="",C481="",E481="",F481=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B481,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F481,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C481,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E481,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C481,C481),"000"))</f>
+        <f aca="false">IF(OR(B481="",C481="",E481="",F481=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B481,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F481,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C481,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E481,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C481,C481),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G482" s="2" t="str">
-        <f aca="false">IF(OR(B482="",C482="",E482="",F482=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B482,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F482,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C482,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E482,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C482,C482),"000"))</f>
+        <f aca="false">IF(OR(B482="",C482="",E482="",F482=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B482,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F482,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C482,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E482,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C482,C482),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="483" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G483" s="2" t="str">
-        <f aca="false">IF(OR(B483="",C483="",E483="",F483=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B483,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F483,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C483,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E483,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C483,C483),"000"))</f>
+        <f aca="false">IF(OR(B483="",C483="",E483="",F483=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B483,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F483,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C483,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E483,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C483,C483),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="484" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G484" s="2" t="str">
-        <f aca="false">IF(OR(B484="",C484="",E484="",F484=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B484,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F484,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C484,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E484,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C484,C484),"000"))</f>
+        <f aca="false">IF(OR(B484="",C484="",E484="",F484=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B484,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F484,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C484,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E484,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C484,C484),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="485" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G485" s="2" t="str">
-        <f aca="false">IF(OR(B485="",C485="",E485="",F485=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B485,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F485,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C485,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E485,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C485,C485),"000"))</f>
+        <f aca="false">IF(OR(B485="",C485="",E485="",F485=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B485,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F485,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C485,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E485,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C485,C485),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G486" s="2" t="str">
-        <f aca="false">IF(OR(B486="",C486="",E486="",F486=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B486,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F486,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C486,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E486,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C486,C486),"000"))</f>
+        <f aca="false">IF(OR(B486="",C486="",E486="",F486=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B486,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F486,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C486,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E486,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C486,C486),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="487" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G487" s="2" t="str">
-        <f aca="false">IF(OR(B487="",C487="",E487="",F487=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B487,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F487,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C487,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E487,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C487,C487),"000"))</f>
+        <f aca="false">IF(OR(B487="",C487="",E487="",F487=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B487,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F487,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C487,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E487,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C487,C487),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G488" s="2" t="str">
-        <f aca="false">IF(OR(B488="",C488="",E488="",F488=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B488,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F488,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C488,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E488,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C488,C488),"000"))</f>
+        <f aca="false">IF(OR(B488="",C488="",E488="",F488=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B488,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F488,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C488,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E488,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C488,C488),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G489" s="2" t="str">
-        <f aca="false">IF(OR(B489="",C489="",E489="",F489=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B489,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F489,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C489,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E489,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C489,C489),"000"))</f>
+        <f aca="false">IF(OR(B489="",C489="",E489="",F489=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B489,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F489,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C489,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E489,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C489,C489),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="490" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G490" s="2" t="str">
-        <f aca="false">IF(OR(B490="",C490="",E490="",F490=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B490,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F490,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C490,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E490,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C490,C490),"000"))</f>
+        <f aca="false">IF(OR(B490="",C490="",E490="",F490=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B490,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F490,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C490,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E490,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C490,C490),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G491" s="2" t="str">
-        <f aca="false">IF(OR(B491="",C491="",E491="",F491=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B491,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F491,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C491,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E491,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C491,C491),"000"))</f>
+        <f aca="false">IF(OR(B491="",C491="",E491="",F491=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B491,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F491,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C491,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E491,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C491,C491),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="492" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G492" s="2" t="str">
-        <f aca="false">IF(OR(B492="",C492="",E492="",F492=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B492,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F492,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C492,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E492,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C492,C492),"000"))</f>
+        <f aca="false">IF(OR(B492="",C492="",E492="",F492=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B492,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F492,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C492,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E492,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C492,C492),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G493" s="2" t="str">
-        <f aca="false">IF(OR(B493="",C493="",E493="",F493=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B493,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F493,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C493,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E493,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C493,C493),"000"))</f>
+        <f aca="false">IF(OR(B493="",C493="",E493="",F493=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B493,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F493,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C493,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E493,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C493,C493),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G494" s="2" t="str">
-        <f aca="false">IF(OR(B494="",C494="",E494="",F494=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B494,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F494,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C494,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E494,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C494,C494),"000"))</f>
+        <f aca="false">IF(OR(B494="",C494="",E494="",F494=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B494,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F494,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C494,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E494,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C494,C494),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G495" s="2" t="str">
-        <f aca="false">IF(OR(B495="",C495="",E495="",F495=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B495,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F495,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C495,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E495,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C495,C495),"000"))</f>
+        <f aca="false">IF(OR(B495="",C495="",E495="",F495=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B495,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F495,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C495,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E495,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C495,C495),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G496" s="2" t="str">
-        <f aca="false">IF(OR(B496="",C496="",E496="",F496=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B496,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F496,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C496,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E496,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C496,C496),"000"))</f>
+        <f aca="false">IF(OR(B496="",C496="",E496="",F496=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B496,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F496,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C496,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E496,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C496,C496),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G497" s="2" t="str">
-        <f aca="false">IF(OR(B497="",C497="",E497="",F497=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B497,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F497,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C497,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E497,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C497,C497),"000"))</f>
+        <f aca="false">IF(OR(B497="",C497="",E497="",F497=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B497,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F497,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C497,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E497,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C497,C497),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G498" s="2" t="str">
-        <f aca="false">IF(OR(B498="",C498="",E498="",F498=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B498,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F498,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C498,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E498,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C498,C498),"000"))</f>
+        <f aca="false">IF(OR(B498="",C498="",E498="",F498=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B498,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F498,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C498,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E498,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C498,C498),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G499" s="2" t="str">
-        <f aca="false">IF(OR(B499="",C499="",E499="",F499=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B499,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F499,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C499,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E499,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C499,C499),"000"))</f>
+        <f aca="false">IF(OR(B499="",C499="",E499="",F499=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B499,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F499,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C499,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E499,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C499,C499),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G500" s="2" t="str">
-        <f aca="false">IF(OR(B500="",C500="",E500="",F500=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B500,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F500,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C500,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E500,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C500,C500),"000"))</f>
+        <f aca="false">IF(OR(B500="",C500="",E500="",F500=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B500,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F500,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C500,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E500,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C500,C500),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G501" s="2" t="str">
-        <f aca="false">IF(OR(B501="",C501="",E501="",F501=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B501,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F501,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C501,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E501,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C501,C501),"000"))</f>
+        <f aca="false">IF(OR(B501="",C501="",E501="",F501=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B501,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F501,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C501,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E501,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C501,C501),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="502" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G502" s="2" t="str">
-        <f aca="false">IF(OR(B502="",C502="",E502="",F502=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B502,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F502,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C502,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E502,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C502,C502),"000"))</f>
+        <f aca="false">IF(OR(B502="",C502="",E502="",F502=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B502,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F502,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C502,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E502,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C502,C502),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G503" s="2" t="str">
-        <f aca="false">IF(OR(B503="",C503="",E503="",F503=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B503,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F503,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C503,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E503,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C503,C503),"000"))</f>
+        <f aca="false">IF(OR(B503="",C503="",E503="",F503=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B503,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F503,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C503,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E503,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C503,C503),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="504" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G504" s="2" t="str">
-        <f aca="false">IF(OR(B504="",C504="",E504="",F504=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B504,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F504,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C504,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E504,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C504,C504),"000"))</f>
+        <f aca="false">IF(OR(B504="",C504="",E504="",F504=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B504,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F504,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C504,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E504,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C504,C504),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="505" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G505" s="2" t="str">
-        <f aca="false">IF(OR(B505="",C505="",E505="",F505=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B505,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F505,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C505,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E505,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C505,C505),"000"))</f>
+        <f aca="false">IF(OR(B505="",C505="",E505="",F505=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B505,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F505,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C505,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E505,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C505,C505),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="506" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G506" s="2" t="str">
-        <f aca="false">IF(OR(B506="",C506="",E506="",F506=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B506,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F506,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C506,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E506,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C506,C506),"000"))</f>
+        <f aca="false">IF(OR(B506="",C506="",E506="",F506=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B506,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F506,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C506,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E506,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C506,C506),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="507" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G507" s="2" t="str">
-        <f aca="false">IF(OR(B507="",C507="",E507="",F507=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B507,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F507,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C507,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E507,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C507,C507),"000"))</f>
+        <f aca="false">IF(OR(B507="",C507="",E507="",F507=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B507,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F507,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C507,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E507,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C507,C507),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="508" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G508" s="2" t="str">
-        <f aca="false">IF(OR(B508="",C508="",E508="",F508=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B508,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F508,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C508,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E508,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C508,C508),"000"))</f>
+        <f aca="false">IF(OR(B508="",C508="",E508="",F508=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B508,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F508,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C508,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E508,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C508,C508),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="509" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G509" s="2" t="str">
-        <f aca="false">IF(OR(B509="",C509="",E509="",F509=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B509,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F509,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C509,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E509,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C509,C509),"000"))</f>
+        <f aca="false">IF(OR(B509="",C509="",E509="",F509=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B509,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F509,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C509,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E509,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C509,C509),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="510" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G510" s="2" t="str">
-        <f aca="false">IF(OR(B510="",C510="",E510="",F510=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B510,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F510,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C510,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E510,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C510,C510),"000"))</f>
+        <f aca="false">IF(OR(B510="",C510="",E510="",F510=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B510,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F510,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C510,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E510,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C510,C510),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="511" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G511" s="2" t="str">
-        <f aca="false">IF(OR(B511="",C511="",E511="",F511=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B511,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F511,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C511,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E511,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C511,C511),"000"))</f>
+        <f aca="false">IF(OR(B511="",C511="",E511="",F511=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B511,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F511,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C511,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E511,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C511,C511),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="512" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G512" s="2" t="str">
-        <f aca="false">IF(OR(B512="",C512="",E512="",F512=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B512,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F512,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C512,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E512,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C512,C512),"000"))</f>
+        <f aca="false">IF(OR(B512="",C512="",E512="",F512=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B512,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F512,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C512,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E512,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C512,C512),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="513" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G513" s="2" t="str">
-        <f aca="false">IF(OR(B513="",C513="",E513="",F513=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B513,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F513,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C513,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E513,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C513,C513),"000"))</f>
+        <f aca="false">IF(OR(B513="",C513="",E513="",F513=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B513,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F513,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C513,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E513,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C513,C513),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="514" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G514" s="2" t="str">
-        <f aca="false">IF(OR(B514="",C514="",E514="",F514=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B514,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F514,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C514,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E514,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C514,C514),"000"))</f>
+        <f aca="false">IF(OR(B514="",C514="",E514="",F514=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B514,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F514,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C514,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E514,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C514,C514),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="515" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G515" s="2" t="str">
-        <f aca="false">IF(OR(B515="",C515="",E515="",F515=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B515,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F515,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C515,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E515,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C515,C515),"000"))</f>
+        <f aca="false">IF(OR(B515="",C515="",E515="",F515=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B515,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F515,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C515,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E515,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C515,C515),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="516" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G516" s="2" t="str">
-        <f aca="false">IF(OR(B516="",C516="",E516="",F516=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B516,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F516,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C516,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E516,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C516,C516),"000"))</f>
+        <f aca="false">IF(OR(B516="",C516="",E516="",F516=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B516,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F516,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C516,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E516,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C516,C516),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="517" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G517" s="2" t="str">
-        <f aca="false">IF(OR(B517="",C517="",E517="",F517=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B517,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F517,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C517,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E517,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C517,C517),"000"))</f>
+        <f aca="false">IF(OR(B517="",C517="",E517="",F517=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B517,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F517,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C517,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E517,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C517,C517),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="518" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G518" s="2" t="str">
-        <f aca="false">IF(OR(B518="",C518="",E518="",F518=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B518,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F518,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C518,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E518,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C518,C518),"000"))</f>
+        <f aca="false">IF(OR(B518="",C518="",E518="",F518=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B518,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F518,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C518,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E518,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C518,C518),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="519" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G519" s="2" t="str">
-        <f aca="false">IF(OR(B519="",C519="",E519="",F519=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B519,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F519,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C519,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E519,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C519,C519),"000"))</f>
+        <f aca="false">IF(OR(B519="",C519="",E519="",F519=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B519,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F519,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C519,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E519,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C519,C519),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="520" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G520" s="2" t="str">
-        <f aca="false">IF(OR(B520="",C520="",E520="",F520=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B520,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F520,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C520,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E520,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C520,C520),"000"))</f>
+        <f aca="false">IF(OR(B520="",C520="",E520="",F520=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B520,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F520,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C520,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E520,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C520,C520),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="521" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G521" s="2" t="str">
-        <f aca="false">IF(OR(B521="",C521="",E521="",F521=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B521,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F521,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C521,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E521,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C521,C521),"000"))</f>
+        <f aca="false">IF(OR(B521="",C521="",E521="",F521=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B521,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F521,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C521,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E521,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C521,C521),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="522" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G522" s="2" t="str">
-        <f aca="false">IF(OR(B522="",C522="",E522="",F522=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B522,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F522,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C522,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E522,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C522,C522),"000"))</f>
+        <f aca="false">IF(OR(B522="",C522="",E522="",F522=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B522,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F522,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C522,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E522,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C522,C522),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="523" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G523" s="2" t="str">
-        <f aca="false">IF(OR(B523="",C523="",E523="",F523=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B523,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F523,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C523,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E523,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C523,C523),"000"))</f>
+        <f aca="false">IF(OR(B523="",C523="",E523="",F523=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B523,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F523,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C523,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E523,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C523,C523),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="524" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G524" s="2" t="str">
-        <f aca="false">IF(OR(B524="",C524="",E524="",F524=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B524,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F524,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C524,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E524,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C524,C524),"000"))</f>
+        <f aca="false">IF(OR(B524="",C524="",E524="",F524=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B524,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F524,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C524,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E524,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C524,C524),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="525" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G525" s="2" t="str">
-        <f aca="false">IF(OR(B525="",C525="",E525="",F525=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B525,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F525,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C525,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E525,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C525,C525),"000"))</f>
+        <f aca="false">IF(OR(B525="",C525="",E525="",F525=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B525,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F525,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C525,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E525,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C525,C525),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="526" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G526" s="2" t="str">
-        <f aca="false">IF(OR(B526="",C526="",E526="",F526=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B526,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F526,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C526,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E526,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C526,C526),"000"))</f>
+        <f aca="false">IF(OR(B526="",C526="",E526="",F526=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B526,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F526,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C526,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E526,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C526,C526),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="527" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G527" s="2" t="str">
-        <f aca="false">IF(OR(B527="",C527="",E527="",F527=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B527,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F527,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C527,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E527,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C527,C527),"000"))</f>
+        <f aca="false">IF(OR(B527="",C527="",E527="",F527=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B527,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F527,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C527,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E527,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C527,C527),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="528" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G528" s="2" t="str">
-        <f aca="false">IF(OR(B528="",C528="",E528="",F528=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B528,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F528,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C528,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E528,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C528,C528),"000"))</f>
+        <f aca="false">IF(OR(B528="",C528="",E528="",F528=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B528,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F528,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C528,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E528,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C528,C528),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="529" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G529" s="2" t="str">
-        <f aca="false">IF(OR(B529="",C529="",E529="",F529=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B529,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F529,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C529,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E529,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C529,C529),"000"))</f>
+        <f aca="false">IF(OR(B529="",C529="",E529="",F529=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B529,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F529,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C529,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E529,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C529,C529),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="530" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G530" s="2" t="str">
-        <f aca="false">IF(OR(B530="",C530="",E530="",F530=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B530,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F530,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C530,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E530,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C530,C530),"000"))</f>
+        <f aca="false">IF(OR(B530="",C530="",E530="",F530=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B530,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F530,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C530,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E530,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C530,C530),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="531" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G531" s="2" t="str">
-        <f aca="false">IF(OR(B531="",C531="",E531="",F531=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B531,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F531,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C531,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E531,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C531,C531),"000"))</f>
+        <f aca="false">IF(OR(B531="",C531="",E531="",F531=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B531,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F531,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C531,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E531,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C531,C531),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="532" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G532" s="2" t="str">
-        <f aca="false">IF(OR(B532="",C532="",E532="",F532=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B532,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F532,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C532,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E532,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C532,C532),"000"))</f>
+        <f aca="false">IF(OR(B532="",C532="",E532="",F532=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B532,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F532,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C532,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E532,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C532,C532),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="533" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G533" s="2" t="str">
-        <f aca="false">IF(OR(B533="",C533="",E533="",F533=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B533,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F533,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C533,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E533,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C533,C533),"000"))</f>
+        <f aca="false">IF(OR(B533="",C533="",E533="",F533=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B533,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F533,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C533,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E533,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C533,C533),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="534" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G534" s="2" t="str">
-        <f aca="false">IF(OR(B534="",C534="",E534="",F534=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B534,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F534,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C534,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E534,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C534,C534),"000"))</f>
+        <f aca="false">IF(OR(B534="",C534="",E534="",F534=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B534,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F534,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C534,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E534,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C534,C534),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="535" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G535" s="2" t="str">
-        <f aca="false">IF(OR(B535="",C535="",E535="",F535=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B535,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F535,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C535,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E535,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C535,C535),"000"))</f>
+        <f aca="false">IF(OR(B535="",C535="",E535="",F535=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B535,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F535,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C535,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E535,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C535,C535),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="536" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G536" s="2" t="str">
-        <f aca="false">IF(OR(B536="",C536="",E536="",F536=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B536,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F536,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C536,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E536,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C536,C536),"000"))</f>
+        <f aca="false">IF(OR(B536="",C536="",E536="",F536=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B536,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F536,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C536,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E536,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C536,C536),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="537" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G537" s="2" t="str">
-        <f aca="false">IF(OR(B537="",C537="",E537="",F537=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B537,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F537,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C537,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E537,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C537,C537),"000"))</f>
+        <f aca="false">IF(OR(B537="",C537="",E537="",F537=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B537,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F537,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C537,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E537,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C537,C537),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="538" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G538" s="2" t="str">
-        <f aca="false">IF(OR(B538="",C538="",E538="",F538=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B538,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F538,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C538,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E538,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C538,C538),"000"))</f>
+        <f aca="false">IF(OR(B538="",C538="",E538="",F538=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B538,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F538,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C538,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E538,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C538,C538),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="539" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G539" s="2" t="str">
-        <f aca="false">IF(OR(B539="",C539="",E539="",F539=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B539,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F539,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C539,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E539,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C539,C539),"000"))</f>
+        <f aca="false">IF(OR(B539="",C539="",E539="",F539=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B539,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F539,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C539,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E539,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C539,C539),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="540" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G540" s="2" t="str">
-        <f aca="false">IF(OR(B540="",C540="",E540="",F540=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B540,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F540,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C540,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E540,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C540,C540),"000"))</f>
+        <f aca="false">IF(OR(B540="",C540="",E540="",F540=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B540,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F540,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C540,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E540,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C540,C540),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="541" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G541" s="2" t="str">
-        <f aca="false">IF(OR(B541="",C541="",E541="",F541=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B541,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F541,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C541,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E541,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C541,C541),"000"))</f>
+        <f aca="false">IF(OR(B541="",C541="",E541="",F541=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B541,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F541,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C541,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E541,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C541,C541),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="542" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G542" s="2" t="str">
-        <f aca="false">IF(OR(B542="",C542="",E542="",F542=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B542,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F542,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C542,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E542,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C542,C542),"000"))</f>
+        <f aca="false">IF(OR(B542="",C542="",E542="",F542=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B542,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F542,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C542,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E542,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C542,C542),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="543" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G543" s="2" t="str">
-        <f aca="false">IF(OR(B543="",C543="",E543="",F543=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B543,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F543,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C543,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E543,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C543,C543),"000"))</f>
+        <f aca="false">IF(OR(B543="",C543="",E543="",F543=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B543,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F543,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C543,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E543,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C543,C543),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="544" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G544" s="2" t="str">
-        <f aca="false">IF(OR(B544="",C544="",E544="",F544=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B544,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F544,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C544,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E544,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C544,C544),"000"))</f>
+        <f aca="false">IF(OR(B544="",C544="",E544="",F544=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B544,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F544,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C544,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E544,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C544,C544),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="545" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G545" s="2" t="str">
-        <f aca="false">IF(OR(B545="",C545="",E545="",F545=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B545,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F545,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C545,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E545,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C545,C545),"000"))</f>
+        <f aca="false">IF(OR(B545="",C545="",E545="",F545=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B545,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F545,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C545,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E545,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C545,C545),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="546" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G546" s="2" t="str">
-        <f aca="false">IF(OR(B546="",C546="",E546="",F546=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B546,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F546,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C546,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E546,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C546,C546),"000"))</f>
+        <f aca="false">IF(OR(B546="",C546="",E546="",F546=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B546,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F546,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C546,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E546,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C546,C546),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="547" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G547" s="2" t="str">
-        <f aca="false">IF(OR(B547="",C547="",E547="",F547=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B547,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F547,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C547,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E547,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C547,C547),"000"))</f>
+        <f aca="false">IF(OR(B547="",C547="",E547="",F547=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B547,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F547,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C547,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E547,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C547,C547),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="548" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G548" s="2" t="str">
-        <f aca="false">IF(OR(B548="",C548="",E548="",F548=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B548,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F548,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C548,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E548,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C548,C548),"000"))</f>
+        <f aca="false">IF(OR(B548="",C548="",E548="",F548=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B548,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F548,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C548,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E548,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C548,C548),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="549" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G549" s="2" t="str">
-        <f aca="false">IF(OR(B549="",C549="",E549="",F549=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B549,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F549,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C549,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E549,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C549,C549),"000"))</f>
+        <f aca="false">IF(OR(B549="",C549="",E549="",F549=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B549,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F549,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C549,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E549,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C549,C549),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="550" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G550" s="2" t="str">
-        <f aca="false">IF(OR(B550="",C550="",E550="",F550=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B550,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F550,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C550,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E550,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C550,C550),"000"))</f>
+        <f aca="false">IF(OR(B550="",C550="",E550="",F550=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B550,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F550,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C550,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E550,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C550,C550),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="551" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G551" s="2" t="str">
-        <f aca="false">IF(OR(B551="",C551="",E551="",F551=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B551,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F551,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C551,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E551,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C551,C551),"000"))</f>
+        <f aca="false">IF(OR(B551="",C551="",E551="",F551=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B551,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F551,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C551,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E551,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C551,C551),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="552" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G552" s="2" t="str">
-        <f aca="false">IF(OR(B552="",C552="",E552="",F552=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B552,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F552,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C552,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E552,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C552,C552),"000"))</f>
+        <f aca="false">IF(OR(B552="",C552="",E552="",F552=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B552,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F552,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C552,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E552,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C552,C552),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="553" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G553" s="2" t="str">
-        <f aca="false">IF(OR(B553="",C553="",E553="",F553=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B553,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F553,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C553,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E553,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C553,C553),"000"))</f>
+        <f aca="false">IF(OR(B553="",C553="",E553="",F553=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B553,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F553,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C553,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E553,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C553,C553),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="554" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G554" s="2" t="str">
-        <f aca="false">IF(OR(B554="",C554="",E554="",F554=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B554,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F554,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C554,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E554,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C554,C554),"000"))</f>
+        <f aca="false">IF(OR(B554="",C554="",E554="",F554=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B554,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F554,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C554,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E554,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C554,C554),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="555" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G555" s="2" t="str">
-        <f aca="false">IF(OR(B555="",C555="",E555="",F555=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B555,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F555,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C555,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E555,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C555,C555),"000"))</f>
+        <f aca="false">IF(OR(B555="",C555="",E555="",F555=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B555,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F555,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C555,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E555,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C555,C555),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="556" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G556" s="2" t="str">
-        <f aca="false">IF(OR(B556="",C556="",E556="",F556=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B556,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F556,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C556,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E556,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C556,C556),"000"))</f>
+        <f aca="false">IF(OR(B556="",C556="",E556="",F556=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B556,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F556,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C556,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E556,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C556,C556),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="557" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G557" s="2" t="str">
-        <f aca="false">IF(OR(B557="",C557="",E557="",F557=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B557,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F557,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C557,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E557,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C557,C557),"000"))</f>
+        <f aca="false">IF(OR(B557="",C557="",E557="",F557=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B557,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F557,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C557,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E557,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C557,C557),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="558" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G558" s="2" t="str">
-        <f aca="false">IF(OR(B558="",C558="",E558="",F558=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B558,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F558,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C558,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E558,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C558,C558),"000"))</f>
+        <f aca="false">IF(OR(B558="",C558="",E558="",F558=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B558,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F558,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C558,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E558,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C558,C558),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="559" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G559" s="2" t="str">
-        <f aca="false">IF(OR(B559="",C559="",E559="",F559=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B559,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F559,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C559,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E559,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C559,C559),"000"))</f>
+        <f aca="false">IF(OR(B559="",C559="",E559="",F559=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B559,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F559,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C559,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E559,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C559,C559),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="560" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G560" s="2" t="str">
-        <f aca="false">IF(OR(B560="",C560="",E560="",F560=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B560,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F560,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C560,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E560,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C560,C560),"000"))</f>
+        <f aca="false">IF(OR(B560="",C560="",E560="",F560=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B560,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F560,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C560,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E560,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C560,C560),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="561" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G561" s="2" t="str">
-        <f aca="false">IF(OR(B561="",C561="",E561="",F561=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B561,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F561,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C561,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E561,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C561,C561),"000"))</f>
+        <f aca="false">IF(OR(B561="",C561="",E561="",F561=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B561,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F561,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C561,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E561,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C561,C561),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="562" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G562" s="2" t="str">
-        <f aca="false">IF(OR(B562="",C562="",E562="",F562=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B562,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F562,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C562,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E562,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C562,C562),"000"))</f>
+        <f aca="false">IF(OR(B562="",C562="",E562="",F562=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B562,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F562,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C562,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E562,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C562,C562),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="563" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G563" s="2" t="str">
-        <f aca="false">IF(OR(B563="",C563="",E563="",F563=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B563,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F563,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C563,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E563,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C563,C563),"000"))</f>
+        <f aca="false">IF(OR(B563="",C563="",E563="",F563=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B563,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F563,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C563,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E563,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C563,C563),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="564" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G564" s="2" t="str">
-        <f aca="false">IF(OR(B564="",C564="",E564="",F564=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B564,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F564,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C564,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E564,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C564,C564),"000"))</f>
+        <f aca="false">IF(OR(B564="",C564="",E564="",F564=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B564,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F564,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C564,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E564,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C564,C564),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="565" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G565" s="2" t="str">
-        <f aca="false">IF(OR(B565="",C565="",E565="",F565=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B565,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F565,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C565,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E565,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C565,C565),"000"))</f>
+        <f aca="false">IF(OR(B565="",C565="",E565="",F565=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B565,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F565,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C565,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E565,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C565,C565),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="566" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G566" s="2" t="str">
-        <f aca="false">IF(OR(B566="",C566="",E566="",F566=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B566,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F566,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C566,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E566,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C566,C566),"000"))</f>
+        <f aca="false">IF(OR(B566="",C566="",E566="",F566=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B566,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F566,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C566,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E566,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C566,C566),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="567" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G567" s="2" t="str">
-        <f aca="false">IF(OR(B567="",C567="",E567="",F567=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B567,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F567,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C567,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E567,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C567,C567),"000"))</f>
+        <f aca="false">IF(OR(B567="",C567="",E567="",F567=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B567,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F567,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C567,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E567,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C567,C567),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="568" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G568" s="2" t="str">
-        <f aca="false">IF(OR(B568="",C568="",E568="",F568=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B568,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F568,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C568,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E568,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C568,C568),"000"))</f>
+        <f aca="false">IF(OR(B568="",C568="",E568="",F568=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B568,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F568,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C568,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E568,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C568,C568),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="569" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G569" s="2" t="str">
-        <f aca="false">IF(OR(B569="",C569="",E569="",F569=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B569,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F569,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C569,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E569,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C569,C569),"000"))</f>
+        <f aca="false">IF(OR(B569="",C569="",E569="",F569=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B569,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F569,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C569,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E569,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C569,C569),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="570" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G570" s="2" t="str">
-        <f aca="false">IF(OR(B570="",C570="",E570="",F570=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B570,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F570,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C570,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E570,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C570,C570),"000"))</f>
+        <f aca="false">IF(OR(B570="",C570="",E570="",F570=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B570,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F570,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C570,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E570,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C570,C570),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="571" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G571" s="2" t="str">
-        <f aca="false">IF(OR(B571="",C571="",E571="",F571=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B571,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F571,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C571,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E571,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C571,C571),"000"))</f>
+        <f aca="false">IF(OR(B571="",C571="",E571="",F571=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B571,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F571,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C571,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E571,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C571,C571),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="572" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G572" s="2" t="str">
-        <f aca="false">IF(OR(B572="",C572="",E572="",F572=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B572,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F572,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C572,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E572,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C572,C572),"000"))</f>
+        <f aca="false">IF(OR(B572="",C572="",E572="",F572=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B572,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F572,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C572,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E572,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C572,C572),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="573" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G573" s="2" t="str">
-        <f aca="false">IF(OR(B573="",C573="",E573="",F573=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B573,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F573,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C573,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E573,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C573,C573),"000"))</f>
+        <f aca="false">IF(OR(B573="",C573="",E573="",F573=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B573,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F573,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C573,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E573,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C573,C573),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="574" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G574" s="2" t="str">
-        <f aca="false">IF(OR(B574="",C574="",E574="",F574=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B574,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F574,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C574,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E574,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C574,C574),"000"))</f>
+        <f aca="false">IF(OR(B574="",C574="",E574="",F574=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B574,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F574,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C574,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E574,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C574,C574),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="575" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G575" s="2" t="str">
-        <f aca="false">IF(OR(B575="",C575="",E575="",F575=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B575,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F575,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C575,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E575,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C575,C575),"000"))</f>
+        <f aca="false">IF(OR(B575="",C575="",E575="",F575=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B575,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F575,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C575,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E575,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C575,C575),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="576" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G576" s="2" t="str">
-        <f aca="false">IF(OR(B576="",C576="",E576="",F576=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B576,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F576,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C576,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E576,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C576,C576),"000"))</f>
+        <f aca="false">IF(OR(B576="",C576="",E576="",F576=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B576,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F576,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C576,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E576,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C576,C576),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="577" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G577" s="2" t="str">
-        <f aca="false">IF(OR(B577="",C577="",E577="",F577=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B577,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F577,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C577,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E577,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C577,C577),"000"))</f>
+        <f aca="false">IF(OR(B577="",C577="",E577="",F577=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B577,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F577,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C577,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E577,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C577,C577),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="578" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G578" s="2" t="str">
-        <f aca="false">IF(OR(B578="",C578="",E578="",F578=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B578,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F578,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C578,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E578,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C578,C578),"000"))</f>
+        <f aca="false">IF(OR(B578="",C578="",E578="",F578=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B578,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F578,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C578,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E578,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C578,C578),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="579" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G579" s="2" t="str">
-        <f aca="false">IF(OR(B579="",C579="",E579="",F579=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B579,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F579,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C579,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E579,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C579,C579),"000"))</f>
+        <f aca="false">IF(OR(B579="",C579="",E579="",F579=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B579,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F579,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C579,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E579,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C579,C579),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="580" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G580" s="2" t="str">
-        <f aca="false">IF(OR(B580="",C580="",E580="",F580=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B580,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F580,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C580,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E580,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C580,C580),"000"))</f>
+        <f aca="false">IF(OR(B580="",C580="",E580="",F580=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B580,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F580,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C580,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E580,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C580,C580),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="581" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G581" s="2" t="str">
-        <f aca="false">IF(OR(B581="",C581="",E581="",F581=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B581,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F581,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C581,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E581,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C581,C581),"000"))</f>
+        <f aca="false">IF(OR(B581="",C581="",E581="",F581=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B581,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F581,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C581,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E581,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C581,C581),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="582" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G582" s="2" t="str">
-        <f aca="false">IF(OR(B582="",C582="",E582="",F582=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B582,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F582,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C582,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E582,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C582,C582),"000"))</f>
+        <f aca="false">IF(OR(B582="",C582="",E582="",F582=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B582,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F582,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C582,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E582,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C582,C582),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="583" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G583" s="2" t="str">
-        <f aca="false">IF(OR(B583="",C583="",E583="",F583=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B583,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F583,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C583,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E583,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C583,C583),"000"))</f>
+        <f aca="false">IF(OR(B583="",C583="",E583="",F583=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B583,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F583,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C583,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E583,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C583,C583),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="584" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G584" s="2" t="str">
-        <f aca="false">IF(OR(B584="",C584="",E584="",F584=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B584,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F584,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C584,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E584,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C584,C584),"000"))</f>
+        <f aca="false">IF(OR(B584="",C584="",E584="",F584=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B584,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F584,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C584,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E584,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C584,C584),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="585" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G585" s="2" t="str">
-        <f aca="false">IF(OR(B585="",C585="",E585="",F585=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B585,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F585,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C585,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E585,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C585,C585),"000"))</f>
+        <f aca="false">IF(OR(B585="",C585="",E585="",F585=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B585,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F585,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C585,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E585,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C585,C585),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="586" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G586" s="2" t="str">
-        <f aca="false">IF(OR(B586="",C586="",E586="",F586=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B586,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F586,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C586,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E586,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C586,C586),"000"))</f>
+        <f aca="false">IF(OR(B586="",C586="",E586="",F586=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B586,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F586,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C586,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E586,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C586,C586),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="587" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G587" s="2" t="str">
-        <f aca="false">IF(OR(B587="",C587="",E587="",F587=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B587,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F587,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C587,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E587,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C587,C587),"000"))</f>
+        <f aca="false">IF(OR(B587="",C587="",E587="",F587=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B587,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F587,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C587,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E587,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C587,C587),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="588" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G588" s="2" t="str">
-        <f aca="false">IF(OR(B588="",C588="",E588="",F588=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B588,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F588,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C588,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E588,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C588,C588),"000"))</f>
+        <f aca="false">IF(OR(B588="",C588="",E588="",F588=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B588,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F588,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C588,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E588,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C588,C588),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="589" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G589" s="2" t="str">
-        <f aca="false">IF(OR(B589="",C589="",E589="",F589=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B589,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F589,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C589,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E589,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C589,C589),"000"))</f>
+        <f aca="false">IF(OR(B589="",C589="",E589="",F589=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B589,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F589,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C589,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E589,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C589,C589),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="590" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G590" s="2" t="str">
-        <f aca="false">IF(OR(B590="",C590="",E590="",F590=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B590,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F590,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C590,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E590,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C590,C590),"000"))</f>
+        <f aca="false">IF(OR(B590="",C590="",E590="",F590=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B590,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F590,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C590,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E590,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C590,C590),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="591" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G591" s="2" t="str">
-        <f aca="false">IF(OR(B591="",C591="",E591="",F591=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B591,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F591,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C591,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E591,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C591,C591),"000"))</f>
+        <f aca="false">IF(OR(B591="",C591="",E591="",F591=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B591,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F591,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C591,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E591,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C591,C591),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="592" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G592" s="2" t="str">
-        <f aca="false">IF(OR(B592="",C592="",E592="",F592=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B592,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F592,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C592,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E592,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C592,C592),"000"))</f>
+        <f aca="false">IF(OR(B592="",C592="",E592="",F592=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B592,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F592,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C592,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E592,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C592,C592),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="593" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G593" s="2" t="str">
-        <f aca="false">IF(OR(B593="",C593="",E593="",F593=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B593,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F593,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C593,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E593,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C593,C593),"000"))</f>
+        <f aca="false">IF(OR(B593="",C593="",E593="",F593=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B593,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F593,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C593,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E593,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C593,C593),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="594" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G594" s="2" t="str">
-        <f aca="false">IF(OR(B594="",C594="",E594="",F594=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B594,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F594,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C594,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E594,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C594,C594),"000"))</f>
+        <f aca="false">IF(OR(B594="",C594="",E594="",F594=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B594,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F594,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C594,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E594,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C594,C594),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="595" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G595" s="2" t="str">
-        <f aca="false">IF(OR(B595="",C595="",E595="",F595=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B595,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F595,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C595,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E595,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C595,C595),"000"))</f>
+        <f aca="false">IF(OR(B595="",C595="",E595="",F595=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B595,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F595,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C595,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E595,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C595,C595),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="596" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G596" s="2" t="str">
-        <f aca="false">IF(OR(B596="",C596="",E596="",F596=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B596,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F596,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C596,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E596,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C596,C596),"000"))</f>
+        <f aca="false">IF(OR(B596="",C596="",E596="",F596=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B596,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F596,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C596,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E596,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C596,C596),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="597" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G597" s="2" t="str">
-        <f aca="false">IF(OR(B597="",C597="",E597="",F597=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B597,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F597,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C597,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E597,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C597,C597),"000"))</f>
+        <f aca="false">IF(OR(B597="",C597="",E597="",F597=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B597,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F597,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C597,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E597,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C597,C597),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="598" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G598" s="2" t="str">
-        <f aca="false">IF(OR(B598="",C598="",E598="",F598=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B598,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F598,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C598,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E598,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C598,C598),"000"))</f>
+        <f aca="false">IF(OR(B598="",C598="",E598="",F598=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B598,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F598,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C598,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E598,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C598,C598),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="599" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G599" s="2" t="str">
-        <f aca="false">IF(OR(B599="",C599="",E599="",F599=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B599,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F599,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C599,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E599,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C599,C599),"000"))</f>
+        <f aca="false">IF(OR(B599="",C599="",E599="",F599=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B599,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F599,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C599,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E599,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C599,C599),"000"))</f>
         <v/>
       </c>
     </row>
     <row r="600" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G600" s="2" t="str">
-        <f aca="false">IF(OR(B600="",C600="",E600="",F600=""),"",INDEX('Code Key'!$B$2:$B$2,MATCH(B600,'Code Key'!$A$2:$A$2,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$5,MATCH(F600,'Code Key'!$D$2:$D$5,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$18,MATCH(C600,'Code Key'!$G$2:$G$18,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$9,MATCH(E600,'Code Key'!$J$2:$J$9,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C600,C600),"000"))</f>
+        <f aca="false">IF(OR(B600="",C600="",E600="",F600=""),"",INDEX('Code Key'!$B$2:$B$10,MATCH(B600,'Code Key'!$A$2:$A$10,0))&amp;"-"&amp;INDEX('Code Key'!$E$2:$E$25,MATCH(F600,'Code Key'!$D$2:$D$25,0))&amp;"-"&amp;INDEX('Code Key'!$H$2:$H$33,MATCH(C600,'Code Key'!$G$2:$G$33,0))&amp;"-"&amp;INDEX('Code Key'!$K$2:$K$19,MATCH(E600,'Code Key'!$J$2:$J$19,0))&amp;"-"&amp;TEXT(COUNTIF($C$2:C600,C600),"000"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="4">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B600" type="list">
-      <formula1>'Code Key'!$A$2:$A$2</formula1>
+      <formula1>'Code Key'!$A$2:$A$10</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C2:C600" type="list">
-      <formula1>'Code Key'!$G$2:$G$18</formula1>
+      <formula1>'Code Key'!$G$2:$G$33</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E600" type="list">
-      <formula1>'Code Key'!$J$2:$J$9</formula1>
+      <formula1>'Code Key'!$J$2:$J$19</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F600" type="list">
-      <formula1>'Code Key'!$D$2:$D$5</formula1>
+      <formula1>'Code Key'!$D$2:$D$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -10007,7 +10007,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -10263,18 +10263,18 @@
         <v>338</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
         <v>341</v>
       </c>
     </row>

</xml_diff>